<commit_message>
Rebuild crosswalk from labeled Roads Export, Onyx report, and Master dashboard
Map Roads Requested Resources → Onyx Total Staff Requested → Master Required.
Use only headers from the user-labeled screenshots; refresh the Word guide.

Co-authored-by: echenry6f <echenry6f@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Roads_Onyx_Master_Column_Crosswalk.xlsx
+++ b/Roads_Onyx_Master_Column_Crosswalk.xlsx
@@ -61,17 +61,15 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="9"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001A2332"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="001A2332"/>
       <sz val="11"/>
     </font>
     <font>
@@ -150,11 +148,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -180,10 +176,10 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -206,7 +202,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -573,11 +568,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI9"/>
+  <dimension ref="A1:AW9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -611,19 +606,33 @@
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="20" customWidth="1" min="34" max="34"/>
     <col width="20" customWidth="1" min="35" max="35"/>
+    <col width="20" customWidth="1" min="36" max="36"/>
+    <col width="20" customWidth="1" min="37" max="37"/>
+    <col width="20" customWidth="1" min="38" max="38"/>
+    <col width="20" customWidth="1" min="39" max="39"/>
+    <col width="20" customWidth="1" min="40" max="40"/>
+    <col width="20" customWidth="1" min="41" max="41"/>
+    <col width="20" customWidth="1" min="42" max="42"/>
+    <col width="20" customWidth="1" min="43" max="43"/>
+    <col width="20" customWidth="1" min="44" max="44"/>
+    <col width="20" customWidth="1" min="45" max="45"/>
+    <col width="20" customWidth="1" min="46" max="46"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="48" max="48"/>
+    <col width="20" customWidth="1" min="49" max="49"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Roads Export ↔ Onyx ↔ Master — Corresponding Columns (UPDATED)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="56" customHeight="1">
+          <t>Roads Export ↔ Onyx Report ↔ Master Daily Jobs Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="52" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>UPDATED: Roads = Roads export file (includes Requested). Onyx = daily dispatch extract. Master = dispatch dashboard. Bold = column heading. Italic = formula/rule. Blank = no corresponding column. Green-highlighted column = Requested staffing stack (was missing previously).</t>
+          <t>Rebuilt from your labeled screenshots. Roads = Roads Export file · Onyx = Onyx report · Master = Master Daily Jobs Dashboard. Bold = column heading · Italic = formula/rule · Blank = no corresponding column. First (green) column = Requested Resources stack.</t>
         </is>
       </c>
     </row>
@@ -737,8 +746,50 @@
       <c r="AI3" s="5" t="n">
         <v>34</v>
       </c>
-    </row>
-    <row r="4" ht="38" customHeight="1">
+      <c r="AJ3" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="AK3" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="AL3" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="AM3" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="AN3" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="AO3" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="AP3" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="AQ3" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="AR3" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="AS3" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="AT3" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="AU3" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="AV3" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="AW3" s="5" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Roads column</t>
@@ -746,317 +797,421 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Requested</t>
+          <t>Requested Resources</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Original Resources</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Subcustomer</t>
+          <t>Verified Resources</t>
         </is>
       </c>
       <c r="E4" s="9" t="n"/>
       <c r="F4" s="9" t="n"/>
       <c r="G4" s="8" t="inlineStr">
         <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>Service Location</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="n"/>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>Job ID</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>Job Reference</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="n"/>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t>Job Tags</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="n"/>
+      <c r="O4" s="8" t="inlineStr">
+        <is>
+          <t>Job Location Name</t>
+        </is>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Job Location Address</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="n"/>
+      <c r="R4" s="8" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+      <c r="S4" s="8" t="inlineStr">
+        <is>
+          <t>Contact Address</t>
+        </is>
+      </c>
+      <c r="T4" s="8" t="inlineStr">
+        <is>
+          <t>Resources</t>
+        </is>
+      </c>
+      <c r="U4" s="8" t="inlineStr">
+        <is>
+          <t>Assignment Date</t>
+        </is>
+      </c>
+      <c r="V4" s="8" t="inlineStr">
+        <is>
+          <t>Start Time</t>
+        </is>
+      </c>
+      <c r="W4" s="8" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="X4" s="8" t="inlineStr">
+        <is>
+          <t>Job Status</t>
+        </is>
+      </c>
+      <c r="Y4" s="9" t="n"/>
+      <c r="Z4" s="8" t="inlineStr">
+        <is>
+          <t>Original Equipment</t>
+        </is>
+      </c>
+      <c r="AA4" s="9" t="n"/>
+      <c r="AB4" s="9" t="n"/>
+      <c r="AC4" s="8" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+      <c r="AD4" s="8" t="inlineStr">
+        <is>
+          <t>HP/MP</t>
+        </is>
+      </c>
+      <c r="AE4" s="8" t="inlineStr">
+        <is>
+          <t>Customer Level</t>
+        </is>
+      </c>
+      <c r="AF4" s="8" t="inlineStr">
+        <is>
+          <t>Standard Time Items</t>
+        </is>
+      </c>
+      <c r="AG4" s="8" t="inlineStr">
+        <is>
+          <t>Total Time Items</t>
+        </is>
+      </c>
+      <c r="AH4" s="8" t="inlineStr">
+        <is>
+          <t>Feedback</t>
+        </is>
+      </c>
+      <c r="AI4" s="8" t="inlineStr">
+        <is>
+          <t>HP Rate</t>
+        </is>
+      </c>
+      <c r="AJ4" s="8" t="inlineStr">
+        <is>
+          <t>Level of HP Expertise</t>
+        </is>
+      </c>
+      <c r="AK4" s="8" t="inlineStr">
+        <is>
+          <t>Certification Level</t>
+        </is>
+      </c>
+      <c r="AL4" s="8" t="inlineStr">
+        <is>
+          <t>Certification Expiration</t>
+        </is>
+      </c>
+      <c r="AM4" s="8" t="inlineStr">
+        <is>
+          <t>Bill Rate</t>
+        </is>
+      </c>
+      <c r="AN4" s="8" t="inlineStr">
+        <is>
+          <t>Pay Rate</t>
+        </is>
+      </c>
+      <c r="AO4" s="8" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+      <c r="AP4" s="8" t="inlineStr">
+        <is>
+          <t>Billable Override</t>
+        </is>
+      </c>
+      <c r="AQ4" s="8" t="inlineStr">
+        <is>
+          <t>External Billable Override</t>
+        </is>
+      </c>
+      <c r="AR4" s="8" t="inlineStr">
+        <is>
+          <t>Coordination Note</t>
+        </is>
+      </c>
+      <c r="AS4" s="8" t="inlineStr">
+        <is>
+          <t>Coordination Status</t>
+        </is>
+      </c>
+      <c r="AT4" s="8" t="inlineStr">
+        <is>
+          <t>Project Status</t>
+        </is>
+      </c>
+      <c r="AU4" s="8" t="inlineStr">
+        <is>
+          <t>Configuration Status</t>
+        </is>
+      </c>
+      <c r="AV4" s="8" t="inlineStr">
+        <is>
+          <t>Last Modified Timestamp</t>
+        </is>
+      </c>
+      <c r="AW4" s="8" t="inlineStr">
+        <is>
+          <t>Role Timestamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>(Roads formula)</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Headcount requested on the Roads export row</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Original resource count on the Roads export (related staffing field)</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Verified resource count on the Roads export</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="n"/>
+      <c r="F5" s="12" t="n"/>
+      <c r="G5" s="12" t="n"/>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>Site / service sub-location on Roads export</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="n"/>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>Numeric/internal id on Roads export (confirm vs Ticket # in your file)</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>Reference string on Roads export</t>
+        </is>
+      </c>
+      <c r="L5" s="12" t="n"/>
+      <c r="M5" s="11" t="inlineStr">
+        <is>
+          <t>e.g. Flagging, TMA, Supervisor</t>
+        </is>
+      </c>
+      <c r="N5" s="12" t="n"/>
+      <c r="O5" s="12" t="n"/>
+      <c r="P5" s="12" t="n"/>
+      <c r="Q5" s="12" t="n"/>
+      <c r="R5" s="12" t="n"/>
+      <c r="S5" s="11" t="inlineStr">
+        <is>
+          <t>Email / address for contact</t>
+        </is>
+      </c>
+      <c r="T5" s="11" t="inlineStr">
+        <is>
+          <t>Assigned person name(s) on Roads export</t>
+        </is>
+      </c>
+      <c r="U5" s="12" t="n"/>
+      <c r="V5" s="12" t="n"/>
+      <c r="W5" s="12" t="n"/>
+      <c r="X5" s="12" t="n"/>
+      <c r="Y5" s="12" t="n"/>
+      <c r="Z5" s="11" t="inlineStr">
+        <is>
+          <t>Equipment listed on Roads export</t>
+        </is>
+      </c>
+      <c r="AA5" s="12" t="n"/>
+      <c r="AB5" s="12" t="n"/>
+      <c r="AC5" s="12" t="n"/>
+      <c r="AD5" s="12" t="n"/>
+      <c r="AE5" s="12" t="n"/>
+      <c r="AF5" s="12" t="n"/>
+      <c r="AG5" s="12" t="n"/>
+      <c r="AH5" s="12" t="n"/>
+      <c r="AI5" s="12" t="n"/>
+      <c r="AJ5" s="12" t="n"/>
+      <c r="AK5" s="12" t="n"/>
+      <c r="AL5" s="12" t="n"/>
+      <c r="AM5" s="12" t="n"/>
+      <c r="AN5" s="12" t="n"/>
+      <c r="AO5" s="12" t="n"/>
+      <c r="AP5" s="12" t="n"/>
+      <c r="AQ5" s="12" t="n"/>
+      <c r="AR5" s="12" t="n"/>
+      <c r="AS5" s="12" t="n"/>
+      <c r="AT5" s="12" t="n"/>
+      <c r="AU5" s="12" t="n"/>
+      <c r="AV5" s="12" t="n"/>
+      <c r="AW5" s="12" t="n"/>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>cooresponding Onyx Column</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Total Staff Requested</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Total Staff Requested</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Total Staff Sent</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Total Staff Sent</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>Total Saved</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>Subcontractor</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>Ticket #</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>Ticket #</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="n"/>
+      <c r="L6" s="9" t="n"/>
+      <c r="M6" s="14" t="inlineStr">
+        <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>Job Location Name</t>
-        </is>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>Job Location Address</t>
-        </is>
-      </c>
-      <c r="J4" s="9" t="n"/>
-      <c r="K4" s="8" t="inlineStr">
-        <is>
-          <t>Contact</t>
-        </is>
-      </c>
-      <c r="L4" s="8" t="inlineStr">
-        <is>
-          <t>Contact Details</t>
-        </is>
-      </c>
-      <c r="M4" s="8" t="inlineStr">
-        <is>
-          <t>Resource</t>
-        </is>
-      </c>
-      <c r="N4" s="8" t="inlineStr">
-        <is>
-          <t>Assignment Date</t>
-        </is>
-      </c>
-      <c r="O4" s="8" t="inlineStr">
-        <is>
-          <t>Start Time</t>
-        </is>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Duration</t>
-        </is>
-      </c>
-      <c r="Q4" s="8" t="inlineStr">
-        <is>
-          <t>End Time</t>
-        </is>
-      </c>
-      <c r="R4" s="8" t="inlineStr">
-        <is>
-          <t>Required Resources</t>
-        </is>
-      </c>
-      <c r="S4" s="8" t="inlineStr">
-        <is>
-          <t>On the Clock</t>
-        </is>
-      </c>
-      <c r="T4" s="9" t="n"/>
-      <c r="U4" s="9" t="n"/>
-      <c r="V4" s="8" t="inlineStr">
-        <is>
-          <t>Physical Equipment</t>
-        </is>
-      </c>
-      <c r="W4" s="9" t="n"/>
-      <c r="X4" s="9" t="n"/>
-      <c r="Y4" s="8" t="inlineStr">
-        <is>
-          <t>HP/MP</t>
-        </is>
-      </c>
-      <c r="Z4" s="8" t="inlineStr">
-        <is>
-          <t>Customer Level</t>
-        </is>
-      </c>
-      <c r="AA4" s="8" t="inlineStr">
-        <is>
-          <t>Standard Time Items</t>
-        </is>
-      </c>
-      <c r="AB4" s="8" t="inlineStr">
-        <is>
-          <t>Total Time Items</t>
-        </is>
-      </c>
-      <c r="AC4" s="8" t="inlineStr">
-        <is>
-          <t>Feedback</t>
-        </is>
-      </c>
-      <c r="AD4" s="8" t="inlineStr">
-        <is>
-          <t>HP Rate</t>
-        </is>
-      </c>
-      <c r="AE4" s="8" t="inlineStr">
-        <is>
-          <t>Level of HP Expertise</t>
-        </is>
-      </c>
-      <c r="AF4" s="8" t="inlineStr">
-        <is>
-          <t>Certification Level</t>
-        </is>
-      </c>
-      <c r="AG4" s="8" t="inlineStr">
-        <is>
-          <t>Certification Expiration</t>
-        </is>
-      </c>
-      <c r="AH4" s="8" t="inlineStr">
-        <is>
-          <t>Bill Rate</t>
-        </is>
-      </c>
-      <c r="AI4" s="8" t="inlineStr">
-        <is>
-          <t>Pay Rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="38" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>(Roads formula)</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>Staff / personnel requested for the job (Roads export)</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n"/>
-      <c r="D5" s="11" t="n"/>
-      <c r="E5" s="11" t="n"/>
-      <c r="F5" s="11" t="n"/>
-      <c r="G5" s="11" t="n"/>
-      <c r="H5" s="11" t="n"/>
-      <c r="I5" s="11" t="n"/>
-      <c r="J5" s="11" t="n"/>
-      <c r="K5" s="11" t="n"/>
-      <c r="L5" s="11" t="n"/>
-      <c r="M5" s="12" t="inlineStr">
-        <is>
-          <t>Assigned person / resource name</t>
-        </is>
-      </c>
-      <c r="N5" s="11" t="n"/>
-      <c r="O5" s="11" t="n"/>
-      <c r="P5" s="11" t="n"/>
-      <c r="Q5" s="12" t="inlineStr">
-        <is>
-          <t>Start Time + Duration</t>
-        </is>
-      </c>
-      <c r="R5" s="12" t="inlineStr">
-        <is>
-          <t>Resources required (may equal or relate to Requested)</t>
-        </is>
-      </c>
-      <c r="S5" s="12" t="inlineStr">
-        <is>
-          <t>Resources currently working / clocked in</t>
-        </is>
-      </c>
-      <c r="T5" s="11" t="n"/>
-      <c r="U5" s="11" t="n"/>
-      <c r="V5" s="11" t="n"/>
-      <c r="W5" s="11" t="n"/>
-      <c r="X5" s="11" t="n"/>
-      <c r="Y5" s="11" t="n"/>
-      <c r="Z5" s="11" t="n"/>
-      <c r="AA5" s="11" t="n"/>
-      <c r="AB5" s="11" t="n"/>
-      <c r="AC5" s="11" t="n"/>
-      <c r="AD5" s="11" t="n"/>
-      <c r="AE5" s="11" t="n"/>
-      <c r="AF5" s="11" t="n"/>
-      <c r="AG5" s="11" t="n"/>
-      <c r="AH5" s="11" t="n"/>
-      <c r="AI5" s="11" t="n"/>
-    </row>
-    <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>cooresponding Onyx Column</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Total Staff Requested</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>Client</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>Subcontractor</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>Ticket #</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="n"/>
-      <c r="G6" s="14" t="inlineStr">
+      <c r="N6" s="14" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
+      <c r="O6" s="14" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
+      <c r="P6" s="14" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr">
+      <c r="Q6" s="14" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="K6" s="9" t="n"/>
-      <c r="L6" s="14" t="inlineStr">
+      <c r="R6" s="9" t="n"/>
+      <c r="S6" s="14" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="M6" s="9" t="n"/>
-      <c r="N6" s="9" t="n"/>
-      <c r="O6" s="14" t="inlineStr">
+      <c r="T6" s="9" t="n"/>
+      <c r="U6" s="9" t="n"/>
+      <c r="V6" s="14" t="inlineStr">
         <is>
           <t>Work Hours</t>
         </is>
       </c>
-      <c r="P6" s="14" t="inlineStr">
+      <c r="W6" s="14" t="inlineStr">
         <is>
           <t>Work Hours</t>
         </is>
       </c>
-      <c r="Q6" s="14" t="inlineStr">
-        <is>
-          <t>Work Hours</t>
-        </is>
-      </c>
-      <c r="R6" s="14" t="inlineStr">
-        <is>
-          <t>Total Staff Requested</t>
-        </is>
-      </c>
-      <c r="S6" s="14" t="inlineStr">
-        <is>
-          <t>Total Staff Sent</t>
-        </is>
-      </c>
-      <c r="T6" s="14" t="inlineStr">
-        <is>
-          <t>Total Staff Sent</t>
-        </is>
-      </c>
-      <c r="U6" s="14" t="inlineStr">
-        <is>
-          <t>Total Saved</t>
-        </is>
-      </c>
-      <c r="V6" s="14" t="inlineStr">
+      <c r="X6" s="9" t="n"/>
+      <c r="Y6" s="14" t="inlineStr">
+        <is>
+          <t>Ticket Type</t>
+        </is>
+      </c>
+      <c r="Z6" s="14" t="inlineStr">
         <is>
           <t>AFAD Sent</t>
         </is>
       </c>
-      <c r="W6" s="14" t="inlineStr">
-        <is>
-          <t>Ticket Type</t>
-        </is>
-      </c>
-      <c r="X6" s="14" t="inlineStr">
+      <c r="AA6" s="14" t="inlineStr">
         <is>
           <t>AFAD Sent</t>
         </is>
       </c>
-      <c r="Y6" s="9" t="n"/>
-      <c r="Z6" s="9" t="n"/>
-      <c r="AA6" s="9" t="n"/>
-      <c r="AB6" s="9" t="n"/>
+      <c r="AB6" s="14" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
       <c r="AC6" s="14" t="inlineStr">
         <is>
           <t>Notes</t>
@@ -1068,105 +1223,137 @@
       <c r="AG6" s="9" t="n"/>
       <c r="AH6" s="9" t="n"/>
       <c r="AI6" s="9" t="n"/>
-    </row>
-    <row r="7" ht="38" customHeight="1">
+      <c r="AJ6" s="9" t="n"/>
+      <c r="AK6" s="9" t="n"/>
+      <c r="AL6" s="9" t="n"/>
+      <c r="AM6" s="9" t="n"/>
+      <c r="AN6" s="9" t="n"/>
+      <c r="AO6" s="9" t="n"/>
+      <c r="AP6" s="9" t="n"/>
+      <c r="AQ6" s="9" t="n"/>
+      <c r="AR6" s="9" t="n"/>
+      <c r="AS6" s="9" t="n"/>
+      <c r="AT6" s="9" t="n"/>
+      <c r="AU6" s="9" t="n"/>
+      <c r="AV6" s="9" t="n"/>
+      <c r="AW6" s="9" t="n"/>
+    </row>
+    <row r="7" ht="40" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
           <t>(Onyx formula)</t>
         </is>
       </c>
-      <c r="B7" s="11" t="n"/>
-      <c r="C7" s="11" t="n"/>
-      <c r="D7" s="11" t="n"/>
+      <c r="B7" s="12" t="n"/>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Related — often aligns with requested headcount</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>Related — people actually working / verified</t>
+        </is>
+      </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>Internal job key (one row per ticket)</t>
-        </is>
-      </c>
-      <c r="F7" s="11" t="n"/>
-      <c r="G7" s="11" t="n"/>
-      <c r="H7" s="11" t="n"/>
+          <t>People actually sent on the ticket</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>max(0, Total Staff Requested − Total Staff Sent)</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="n"/>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>Related partner / sub label (not always 1:1)</t>
+        </is>
+      </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
-          <t>(address portion)</t>
-        </is>
-      </c>
-      <c r="J7" s="11" t="n"/>
-      <c r="K7" s="11" t="n"/>
-      <c r="L7" s="15" t="inlineStr">
-        <is>
-          <t>(sometimes holds phone/email notes)</t>
-        </is>
-      </c>
-      <c r="M7" s="11" t="n"/>
-      <c r="N7" s="11" t="n"/>
-      <c r="O7" s="15" t="inlineStr">
-        <is>
-          <t>Start of the scheduled window</t>
-        </is>
-      </c>
-      <c r="P7" s="15" t="inlineStr">
-        <is>
-          <t>Used with Start to imply End / window</t>
-        </is>
-      </c>
-      <c r="Q7" s="15" t="inlineStr">
-        <is>
-          <t>End of the scheduled window</t>
-        </is>
-      </c>
-      <c r="R7" s="15" t="inlineStr">
-        <is>
-          <t>(related headcount field)</t>
-        </is>
-      </c>
+          <t>Internal job key</t>
+        </is>
+      </c>
+      <c r="J7" s="15" t="inlineStr">
+        <is>
+          <t>Confirm whether Job ID equals Ticket # / Job Number in your data</t>
+        </is>
+      </c>
+      <c r="K7" s="12" t="n"/>
+      <c r="L7" s="12" t="n"/>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>Related classification</t>
+        </is>
+      </c>
+      <c r="N7" s="12" t="n"/>
+      <c r="O7" s="12" t="n"/>
+      <c r="P7" s="12" t="n"/>
+      <c r="Q7" s="12" t="n"/>
+      <c r="R7" s="12" t="n"/>
       <c r="S7" s="15" t="inlineStr">
         <is>
-          <t>(related — who is actually working)</t>
-        </is>
-      </c>
-      <c r="T7" s="15" t="inlineStr">
-        <is>
-          <t>People actually sent on the ticket</t>
-        </is>
-      </c>
-      <c r="U7" s="15" t="inlineStr">
-        <is>
-          <t>max(0, Requested − Sent)</t>
-        </is>
-      </c>
+          <t>Sometimes carries contact-like notes</t>
+        </is>
+      </c>
+      <c r="T7" s="12" t="n"/>
+      <c r="U7" s="12" t="n"/>
       <c r="V7" s="15" t="inlineStr">
         <is>
-          <t>(when equipment is AFAD / SmartFlagging gear)</t>
+          <t>Start of window</t>
         </is>
       </c>
       <c r="W7" s="15" t="inlineStr">
         <is>
-          <t>Value "GSF" marks Guardian SmartFlagging jobs</t>
-        </is>
-      </c>
-      <c r="X7" s="15" t="inlineStr">
+          <t>Length of window</t>
+        </is>
+      </c>
+      <c r="X7" s="12" t="n"/>
+      <c r="Y7" s="15" t="inlineStr">
+        <is>
+          <t>Value "GSF" = Guardian SmartFlagging</t>
+        </is>
+      </c>
+      <c r="Z7" s="15" t="inlineStr">
+        <is>
+          <t>When equipment is AFAD / SmartFlagging devices</t>
+        </is>
+      </c>
+      <c r="AA7" s="15" t="inlineStr">
         <is>
           <t>Count of AFADs sent</t>
         </is>
       </c>
-      <c r="Y7" s="11" t="n"/>
-      <c r="Z7" s="11" t="n"/>
-      <c r="AA7" s="11" t="n"/>
-      <c r="AB7" s="11" t="n"/>
+      <c r="AB7" s="12" t="n"/>
       <c r="AC7" s="15" t="inlineStr">
         <is>
-          <t>(related free-text)</t>
-        </is>
-      </c>
-      <c r="AD7" s="11" t="n"/>
-      <c r="AE7" s="11" t="n"/>
-      <c r="AF7" s="11" t="n"/>
-      <c r="AG7" s="11" t="n"/>
-      <c r="AH7" s="11" t="n"/>
-      <c r="AI7" s="11" t="n"/>
-    </row>
-    <row r="8" ht="38" customHeight="1">
+          <t>Related free text</t>
+        </is>
+      </c>
+      <c r="AD7" s="12" t="n"/>
+      <c r="AE7" s="12" t="n"/>
+      <c r="AF7" s="12" t="n"/>
+      <c r="AG7" s="12" t="n"/>
+      <c r="AH7" s="12" t="n"/>
+      <c r="AI7" s="12" t="n"/>
+      <c r="AJ7" s="12" t="n"/>
+      <c r="AK7" s="12" t="n"/>
+      <c r="AL7" s="12" t="n"/>
+      <c r="AM7" s="12" t="n"/>
+      <c r="AN7" s="12" t="n"/>
+      <c r="AO7" s="12" t="n"/>
+      <c r="AP7" s="12" t="n"/>
+      <c r="AQ7" s="12" t="n"/>
+      <c r="AR7" s="12" t="n"/>
+      <c r="AS7" s="12" t="n"/>
+      <c r="AT7" s="12" t="n"/>
+      <c r="AU7" s="12" t="n"/>
+      <c r="AV7" s="12" t="n"/>
+      <c r="AW7" s="12" t="n"/>
+    </row>
+    <row r="8" ht="40" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Cooresponding Master Column</t>
@@ -1179,91 +1366,103 @@
       </c>
       <c r="C8" s="17" t="inlineStr">
         <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>Assignments</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>Assignments</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>Unfilled</t>
+        </is>
+      </c>
+      <c r="G8" s="17" t="inlineStr">
+        <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="H8" s="9" t="n"/>
+      <c r="I8" s="17" t="inlineStr">
         <is>
           <t>Job Number</t>
         </is>
       </c>
-      <c r="F8" s="17" t="inlineStr">
+      <c r="J8" s="17" t="inlineStr">
+        <is>
+          <t>Job Number</t>
+        </is>
+      </c>
+      <c r="K8" s="17" t="inlineStr">
         <is>
           <t>WO Number</t>
         </is>
       </c>
-      <c r="G8" s="17" t="inlineStr">
+      <c r="L8" s="17" t="inlineStr">
+        <is>
+          <t>WO Number</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="H8" s="17" t="inlineStr">
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>Job Type</t>
+        </is>
+      </c>
+      <c r="O8" s="17" t="inlineStr">
         <is>
           <t>Job Location</t>
         </is>
       </c>
-      <c r="I8" s="17" t="inlineStr">
+      <c r="P8" s="17" t="inlineStr">
         <is>
           <t>Job Location</t>
         </is>
       </c>
-      <c r="J8" s="17" t="inlineStr">
+      <c r="Q8" s="17" t="inlineStr">
         <is>
           <t>Dispatching</t>
         </is>
       </c>
-      <c r="K8" s="17" t="inlineStr">
+      <c r="R8" s="17" t="inlineStr">
         <is>
           <t>Customer Foreman</t>
         </is>
       </c>
-      <c r="L8" s="9" t="n"/>
-      <c r="M8" s="17" t="inlineStr">
+      <c r="S8" s="9" t="n"/>
+      <c r="T8" s="17" t="inlineStr">
         <is>
           <t>Crew Lead</t>
         </is>
       </c>
-      <c r="N8" s="17" t="inlineStr">
+      <c r="U8" s="17" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="O8" s="17" t="inlineStr">
+      <c r="V8" s="17" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="P8" s="9" t="n"/>
-      <c r="Q8" s="9" t="n"/>
-      <c r="R8" s="17" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="S8" s="17" t="inlineStr">
-        <is>
-          <t>Assignments</t>
-        </is>
-      </c>
-      <c r="T8" s="17" t="inlineStr">
-        <is>
-          <t>Assignments</t>
-        </is>
-      </c>
-      <c r="U8" s="17" t="inlineStr">
-        <is>
-          <t>Unfilled</t>
-        </is>
-      </c>
-      <c r="V8" s="9" t="n"/>
-      <c r="W8" s="17" t="inlineStr">
+      <c r="W8" s="9" t="n"/>
+      <c r="X8" s="9" t="n"/>
+      <c r="Y8" s="17" t="inlineStr">
         <is>
           <t>GSF</t>
         </is>
       </c>
-      <c r="X8" s="9" t="n"/>
-      <c r="Y8" s="9" t="n"/>
       <c r="Z8" s="9" t="n"/>
       <c r="AA8" s="9" t="n"/>
       <c r="AB8" s="9" t="n"/>
@@ -1274,87 +1473,123 @@
       <c r="AG8" s="9" t="n"/>
       <c r="AH8" s="9" t="n"/>
       <c r="AI8" s="9" t="n"/>
-    </row>
-    <row r="9" ht="38" customHeight="1">
+      <c r="AJ8" s="9" t="n"/>
+      <c r="AK8" s="9" t="n"/>
+      <c r="AL8" s="9" t="n"/>
+      <c r="AM8" s="9" t="n"/>
+      <c r="AN8" s="9" t="n"/>
+      <c r="AO8" s="9" t="n"/>
+      <c r="AP8" s="9" t="n"/>
+      <c r="AQ8" s="9" t="n"/>
+      <c r="AR8" s="9" t="n"/>
+      <c r="AS8" s="9" t="n"/>
+      <c r="AT8" s="9" t="n"/>
+      <c r="AU8" s="9" t="n"/>
+      <c r="AV8" s="9" t="n"/>
+      <c r="AW8" s="9" t="n"/>
+    </row>
+    <row r="9" ht="40" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
         <is>
           <t>(Master formula)</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="11" t="n"/>
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>Related</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Related — assigned slots on Master</t>
+        </is>
+      </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>Same key as Onyx Ticket #</t>
+          <t>Assigned personnel slots (often equals Required on Master)</t>
         </is>
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
+          <t>Open slots (Required − Assignments). NOT the same formula as Onyx Total Saved</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="n"/>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>Sub-label under Customer sometimes shows partner</t>
+        </is>
+      </c>
+      <c r="I9" s="18" t="inlineStr">
+        <is>
+          <t>Same internal key as Onyx Ticket #</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="18" t="inlineStr">
+        <is>
+          <t>Customer WO / EWO — different from Job Number; confirm if Job Reference maps here</t>
+        </is>
+      </c>
+      <c r="L9" s="18" t="inlineStr">
+        <is>
           <t>Customer work-order / EWO — NOT the same as Job Number / Ticket #</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n"/>
-      <c r="H9" s="11" t="n"/>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="11" t="n"/>
-      <c r="K9" s="18" t="inlineStr">
-        <is>
-          <t>Related contact role (not always 1:1)</t>
-        </is>
-      </c>
-      <c r="L9" s="11" t="n"/>
-      <c r="M9" s="18" t="inlineStr">
-        <is>
-          <t>Related assignment person (not always 1:1)</t>
-        </is>
-      </c>
-      <c r="N9" s="11" t="n"/>
-      <c r="O9" s="11" t="n"/>
-      <c r="P9" s="18" t="inlineStr">
-        <is>
-          <t>End ≈ Start + Duration (when both present)</t>
-        </is>
-      </c>
-      <c r="Q9" s="11" t="n"/>
-      <c r="R9" s="11" t="n"/>
-      <c r="S9" s="18" t="inlineStr">
-        <is>
-          <t>(related — assigned slots; may differ from On the Clock / Sent)</t>
-        </is>
-      </c>
+      <c r="M9" s="12" t="n"/>
+      <c r="N9" s="12" t="n"/>
+      <c r="O9" s="12" t="n"/>
+      <c r="P9" s="12" t="n"/>
+      <c r="Q9" s="12" t="n"/>
+      <c r="R9" s="18" t="inlineStr">
+        <is>
+          <t>Related contact (not always identical role)</t>
+        </is>
+      </c>
+      <c r="S9" s="12" t="n"/>
       <c r="T9" s="18" t="inlineStr">
         <is>
-          <t>Planned assigned slots (often = Required on Master)</t>
-        </is>
-      </c>
-      <c r="U9" s="18" t="inlineStr">
-        <is>
-          <t>Required − Assignments when open slots remain — NOT the same formula as Total Saved</t>
-        </is>
-      </c>
-      <c r="V9" s="18" t="inlineStr">
-        <is>
-          <t>No AFAD count column on Master dashboard view</t>
-        </is>
-      </c>
-      <c r="W9" s="18" t="inlineStr">
+          <t>Related assigned lead (not always 1:1)</t>
+        </is>
+      </c>
+      <c r="U9" s="12" t="n"/>
+      <c r="V9" s="12" t="n"/>
+      <c r="W9" s="12" t="n"/>
+      <c r="X9" s="12" t="n"/>
+      <c r="Y9" s="18" t="inlineStr">
         <is>
           <t>Yes / No</t>
         </is>
       </c>
-      <c r="X9" s="11" t="n"/>
-      <c r="Y9" s="11" t="n"/>
-      <c r="Z9" s="11" t="n"/>
-      <c r="AA9" s="11" t="n"/>
-      <c r="AB9" s="11" t="n"/>
-      <c r="AC9" s="11" t="n"/>
-      <c r="AD9" s="11" t="n"/>
-      <c r="AE9" s="11" t="n"/>
-      <c r="AF9" s="11" t="n"/>
-      <c r="AG9" s="11" t="n"/>
-      <c r="AH9" s="11" t="n"/>
-      <c r="AI9" s="11" t="n"/>
+      <c r="Z9" s="18" t="inlineStr">
+        <is>
+          <t>No AFAD count on Master dashboard</t>
+        </is>
+      </c>
+      <c r="AA9" s="12" t="n"/>
+      <c r="AB9" s="12" t="n"/>
+      <c r="AC9" s="12" t="n"/>
+      <c r="AD9" s="12" t="n"/>
+      <c r="AE9" s="12" t="n"/>
+      <c r="AF9" s="12" t="n"/>
+      <c r="AG9" s="12" t="n"/>
+      <c r="AH9" s="12" t="n"/>
+      <c r="AI9" s="12" t="n"/>
+      <c r="AJ9" s="12" t="n"/>
+      <c r="AK9" s="12" t="n"/>
+      <c r="AL9" s="12" t="n"/>
+      <c r="AM9" s="12" t="n"/>
+      <c r="AN9" s="12" t="n"/>
+      <c r="AO9" s="12" t="n"/>
+      <c r="AP9" s="12" t="n"/>
+      <c r="AQ9" s="12" t="n"/>
+      <c r="AR9" s="12" t="n"/>
+      <c r="AS9" s="12" t="n"/>
+      <c r="AT9" s="12" t="n"/>
+      <c r="AU9" s="12" t="n"/>
+      <c r="AV9" s="12" t="n"/>
+      <c r="AW9" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1371,16 +1606,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="108" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>How to read this workbook (UPDATED)</t>
+          <t>Legend — rebuilt crosswalk</t>
         </is>
       </c>
     </row>
@@ -1390,28 +1625,28 @@
     <row r="3">
       <c r="A3" s="20" t="inlineStr">
         <is>
-          <t>Document mapping (corrected):</t>
+          <t>Sources you labeled:</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Roads = Roads export file (wide job/resource export). Includes Requested.</t>
+          <t xml:space="preserve">  1) Roads Export file</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Onyx = daily dispatch extract (Client, Ticket #, Staff Requested/Sent, Saved, AFAD, …).</t>
+          <t xml:space="preserve">  2) Onyx report (Client … Notes; Total Staff Requested/Sent/Saved; AFAD Sent)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Master = dispatch dashboard (Customer, Job Number, Required, Assignments, Unfilled, GSF, …).</t>
+          <t xml:space="preserve">  3) Master Daily Jobs Dashboard (Customer … GSF; Required / Assignments / Unfilled)</t>
         </is>
       </c>
     </row>
@@ -1421,66 +1656,62 @@
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
         <is>
-          <t>What changed in this update:</t>
+          <t>Primary staffing correspondence:</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Roads is no longer treated as the GSF Utilization rollup report.</t>
+          <t xml:space="preserve">  Roads Requested Resources → Onyx Total Staff Requested → Master Required</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Added / highlighted the Requested stack:</t>
-        </is>
-      </c>
+      <c r="A10" s="20" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Roads Requested  →  Onyx Total Staff Requested  →  Master Required</t>
+          <t>Confirmed Onyx headers:</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Related Roads staffing fields also mapped: Required Resources, On the Clock.</t>
+          <t xml:space="preserve">  Client, Subcontractor, Job Type, Ticket #, Ticket Type, Location, Branch,</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr"/>
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Work Hours, Total Staff Requested, Total Staff Sent, Total Saved, AFAD Sent, Notes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="inlineStr">
-        <is>
-          <t>Row labels (Column A):</t>
-        </is>
-      </c>
+      <c r="A14" s="20" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Roads column / (Roads formula)</t>
+          <t>Confirmed Master headers:</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • cooresponding Onyx Column / (Onyx formula)</t>
+          <t xml:space="preserve">  Customer, Crew Lead, Customer Foreman, Dispatching, Job Number, Job Location,</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Cooresponding Master Column / (Master formula)</t>
+          <t xml:space="preserve">  WO Number, Date, Start, Required, Assignments, Unfilled, Job Type, GSF</t>
         </is>
       </c>
     </row>
@@ -1490,55 +1721,59 @@
     <row r="19">
       <c r="A19" s="20" t="inlineStr">
         <is>
-          <t>Blank cell = no corresponding column in that view.</t>
+          <t>Confirmed Roads right-side headers (clear crop):</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="20" t="inlineStr"/>
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  HP/MP, Customer Level, Standard Time Items, Total Time Items, Feedback,</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="inlineStr">
         <is>
-          <t>Key ID note:</t>
+          <t xml:space="preserve">  HP Rate, Level of HP Expertise, Certification Level, Certification Expiration,</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Master Job Number = Onyx Ticket #</t>
+          <t xml:space="preserve">  Bill Rate, Pay Rate</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Master WO Number is a different customer work-order field</t>
-        </is>
-      </c>
+      <c r="A23" s="20" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="20" t="inlineStr"/>
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t>Roads left/mid headers (from Roads Export screenshot; Requested Resources confirmed):</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="20" t="inlineStr">
         <is>
-          <t>Staffing caveat (Beaver Falls 10/05/2026):</t>
+          <t xml:space="preserve">  Customer, Service Location, Requested Resources, Original Resources, Verified Resources,</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Master Assignments often ≠ Onyx Total Staff Sent (shadows/extras on Onyx).</t>
+          <t xml:space="preserve">  Contact, Contact Address, Original Equipment, Job ID, Resources, Assignment Date,</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Master Unfilled ≠ Onyx Total Saved (different formulas).</t>
+          <t xml:space="preserve">  Start Time, Duration, Job Status, Job Location Name/Address, Job Tags, Comments, etc.</t>
         </is>
       </c>
     </row>
@@ -1548,28 +1783,31 @@
     <row r="29">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>Note on Roads header capture:</t>
+          <t>ID rules:</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • The Roads export screenshot is low-resolution; headers were reconstructed from that export</t>
+          <t xml:space="preserve">  Master Job Number = Onyx Ticket #</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">    plus your confirmation that Requested is a Roads column. If any Roads header spelling</t>
+          <t xml:space="preserve">  Master WO Number is a different customer work-order field</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    differs slightly in your file, tell me and I’ll correct the label.</t>
+      <c r="A32" s="20" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>If any Roads left/mid label differs by a word in your live export, send that exact header and it will be corrected.</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1593,33 +1831,33 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>Same crosswalk — vertical stacks (Requested highlighted at top)</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Vertical stacks — same map</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="inlineStr">
-        <is>
-          <t>Roads (export)</t>
-        </is>
-      </c>
-      <c r="B2" s="22" t="inlineStr">
-        <is>
-          <t>Onyx</t>
-        </is>
-      </c>
-      <c r="C2" s="22" t="inlineStr">
-        <is>
-          <t>Master</t>
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>Roads Export</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>Onyx Report</t>
+        </is>
+      </c>
+      <c r="C2" s="21" t="inlineStr">
+        <is>
+          <t>Master Dashboard</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Requested</t>
+          <t>Requested Resources</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -1636,7 +1874,7 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Staff / personnel requested for the job (Roads export)</t>
+          <t>Headcount requested on the Roads export row</t>
         </is>
       </c>
       <c r="B4" s="10" t="n"/>
@@ -1645,145 +1883,185 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Original Resources</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>Total Staff Requested</t>
         </is>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Required</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="n"/>
-      <c r="B7" s="15" t="n"/>
-      <c r="C7" s="18" t="n"/>
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Original resource count on the Roads export (related staffing field)</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Related — often aligns with requested headcount</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>Related</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Subcustomer</t>
+          <t>Verified Resources</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>Subcontractor</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="n"/>
+          <t>Total Staff Sent</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>Assignments</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n"/>
-      <c r="B10" s="15" t="n"/>
-      <c r="C10" s="11" t="n"/>
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Verified resource count on the Roads export</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Related — people actually working / verified</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Related — assigned slots on Master</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n"/>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>Ticket #</t>
+          <t>Total Staff Sent</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>Job Number</t>
+          <t>Assignments</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
+      <c r="A13" s="12" t="n"/>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>Internal job key (one row per ticket)</t>
+          <t>People actually sent on the ticket</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
         <is>
-          <t>Same key as Onyx Ticket #</t>
+          <t>Assigned personnel slots (often equals Required on Master)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n"/>
-      <c r="B15" s="9" t="n"/>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>Total Saved</t>
+        </is>
+      </c>
       <c r="C15" s="17" t="inlineStr">
         <is>
-          <t>WO Number</t>
+          <t>Unfilled</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n"/>
-      <c r="B16" s="11" t="n"/>
+      <c r="A16" s="12" t="n"/>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>max(0, Total Staff Requested − Total Staff Sent)</t>
+        </is>
+      </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>Customer work-order / EWO — NOT the same as Job Number / Ticket #</t>
+          <t>Open slots (Required − Assignments). NOT the same formula as Onyx Total Saved</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Job Type</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Job Type</t>
+          <t>Client</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>Job Type</t>
+          <t>Customer</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="n"/>
+      <c r="A19" s="11" t="n"/>
       <c r="B19" s="15" t="n"/>
       <c r="C19" s="18" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Job Location Name</t>
+          <t>Service Location</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="C21" s="17" t="inlineStr">
-        <is>
-          <t>Job Location</t>
-        </is>
-      </c>
+          <t>Subcontractor</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="n"/>
-      <c r="B22" s="15" t="n"/>
-      <c r="C22" s="18" t="n"/>
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Site / service sub-location on Roads export</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>Related partner / sub label (not always 1:1)</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>Sub-label under Customer sometimes shows partner</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>Job Location Address</t>
-        </is>
-      </c>
+      <c r="A24" s="9" t="n"/>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>Ticket #</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>Job Location</t>
+          <t>Job Number</t>
         </is>
       </c>
     </row>
@@ -1791,441 +2069,445 @@
       <c r="A25" s="12" t="n"/>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>(address portion)</t>
-        </is>
-      </c>
-      <c r="C25" s="18" t="n"/>
+          <t>Internal job key</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>Same internal key as Onyx Ticket #</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="n"/>
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>Job ID</t>
+        </is>
+      </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>Ticket #</t>
         </is>
       </c>
       <c r="C27" s="17" t="inlineStr">
         <is>
-          <t>Dispatching</t>
+          <t>Job Number</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="n"/>
-      <c r="B28" s="15" t="n"/>
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Numeric/internal id on Roads export (confirm vs Ticket # in your file)</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>Confirm whether Job ID equals Ticket # / Job Number in your data</t>
+        </is>
+      </c>
       <c r="C28" s="18" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>Contact</t>
+          <t>Job Reference</t>
         </is>
       </c>
       <c r="B30" s="9" t="n"/>
       <c r="C30" s="17" t="inlineStr">
         <is>
-          <t>Customer Foreman</t>
+          <t>WO Number</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="n"/>
-      <c r="B31" s="11" t="n"/>
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Reference string on Roads export</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="n"/>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>Related contact role (not always 1:1)</t>
+          <t>Customer WO / EWO — different from Job Number; confirm if Job Reference maps here</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t>Contact Details</t>
-        </is>
-      </c>
-      <c r="B33" s="14" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="n"/>
+      <c r="A33" s="9" t="n"/>
+      <c r="B33" s="9" t="n"/>
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>WO Number</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="12" t="n"/>
-      <c r="B34" s="15" t="inlineStr">
-        <is>
-          <t>(sometimes holds phone/email notes)</t>
-        </is>
-      </c>
-      <c r="C34" s="11" t="n"/>
+      <c r="B34" s="12" t="n"/>
+      <c r="C34" s="18" t="inlineStr">
+        <is>
+          <t>Customer work-order / EWO — NOT the same as Job Number / Ticket #</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>Resource</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="n"/>
+          <t>Job Tags</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>Job Type</t>
+        </is>
+      </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>Crew Lead</t>
+          <t>Job Type</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="12" t="inlineStr">
-        <is>
-          <t>Assigned person / resource name</t>
-        </is>
-      </c>
-      <c r="B37" s="11" t="n"/>
-      <c r="C37" s="18" t="inlineStr">
-        <is>
-          <t>Related assignment person (not always 1:1)</t>
-        </is>
-      </c>
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>e.g. Flagging, TMA, Supervisor</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="inlineStr">
+        <is>
+          <t>Related classification</t>
+        </is>
+      </c>
+      <c r="C37" s="18" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>Assignment Date</t>
-        </is>
-      </c>
-      <c r="B39" s="9" t="n"/>
+      <c r="A39" s="9" t="n"/>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>Job Type</t>
+        </is>
+      </c>
       <c r="C39" s="17" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Job Type</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="12" t="n"/>
-      <c r="B40" s="11" t="n"/>
+      <c r="B40" s="15" t="n"/>
       <c r="C40" s="18" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>Start Time</t>
+          <t>Job Location Name</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>Work Hours</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>Start</t>
+          <t>Job Location</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="12" t="n"/>
-      <c r="B43" s="15" t="inlineStr">
-        <is>
-          <t>Start of the scheduled window</t>
-        </is>
-      </c>
+      <c r="A43" s="11" t="n"/>
+      <c r="B43" s="15" t="n"/>
       <c r="C43" s="18" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>Duration</t>
+          <t>Job Location Address</t>
         </is>
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>Work Hours</t>
-        </is>
-      </c>
-      <c r="C45" s="9" t="n"/>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C45" s="17" t="inlineStr">
+        <is>
+          <t>Job Location</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="12" t="n"/>
-      <c r="B46" s="15" t="inlineStr">
-        <is>
-          <t>Used with Start to imply End / window</t>
-        </is>
-      </c>
-      <c r="C46" s="18" t="inlineStr">
-        <is>
-          <t>End ≈ Start + Duration (when both present)</t>
-        </is>
-      </c>
+      <c r="A46" s="11" t="n"/>
+      <c r="B46" s="15" t="n"/>
+      <c r="C46" s="18" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="inlineStr">
-        <is>
-          <t>End Time</t>
-        </is>
-      </c>
+      <c r="A48" s="9" t="n"/>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Work Hours</t>
-        </is>
-      </c>
-      <c r="C48" s="9" t="n"/>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="C48" s="17" t="inlineStr">
+        <is>
+          <t>Dispatching</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="12" t="inlineStr">
-        <is>
-          <t>Start Time + Duration</t>
-        </is>
-      </c>
-      <c r="B49" s="15" t="inlineStr">
-        <is>
-          <t>End of the scheduled window</t>
-        </is>
-      </c>
-      <c r="C49" s="11" t="n"/>
+      <c r="A49" s="12" t="n"/>
+      <c r="B49" s="15" t="n"/>
+      <c r="C49" s="18" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>Required Resources</t>
-        </is>
-      </c>
-      <c r="B51" s="14" t="inlineStr">
-        <is>
-          <t>Total Staff Requested</t>
-        </is>
-      </c>
+          <t>Contact</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="n"/>
       <c r="C51" s="17" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Customer Foreman</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="12" t="inlineStr">
-        <is>
-          <t>Resources required (may equal or relate to Requested)</t>
-        </is>
-      </c>
-      <c r="B52" s="15" t="inlineStr">
-        <is>
-          <t>(related headcount field)</t>
-        </is>
-      </c>
-      <c r="C52" s="18" t="n"/>
+      <c r="A52" s="11" t="n"/>
+      <c r="B52" s="12" t="n"/>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>Related contact (not always identical role)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>On the Clock</t>
+          <t>Contact Address</t>
         </is>
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>Total Staff Sent</t>
-        </is>
-      </c>
-      <c r="C54" s="17" t="inlineStr">
-        <is>
-          <t>Assignments</t>
-        </is>
-      </c>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="12" t="inlineStr">
-        <is>
-          <t>Resources currently working / clocked in</t>
+      <c r="A55" s="11" t="inlineStr">
+        <is>
+          <t>Email / address for contact</t>
         </is>
       </c>
       <c r="B55" s="15" t="inlineStr">
         <is>
-          <t>(related — who is actually working)</t>
-        </is>
-      </c>
-      <c r="C55" s="18" t="inlineStr">
-        <is>
-          <t>(related — assigned slots; may differ from On the Clock / Sent)</t>
-        </is>
-      </c>
+          <t>Sometimes carries contact-like notes</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="9" t="n"/>
-      <c r="B57" s="14" t="inlineStr">
-        <is>
-          <t>Total Staff Sent</t>
-        </is>
-      </c>
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>Resources</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="n"/>
       <c r="C57" s="17" t="inlineStr">
         <is>
-          <t>Assignments</t>
+          <t>Crew Lead</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="11" t="n"/>
-      <c r="B58" s="15" t="inlineStr">
-        <is>
-          <t>People actually sent on the ticket</t>
-        </is>
-      </c>
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>Assigned person name(s) on Roads export</t>
+        </is>
+      </c>
+      <c r="B58" s="12" t="n"/>
       <c r="C58" s="18" t="inlineStr">
         <is>
-          <t>Planned assigned slots (often = Required on Master)</t>
+          <t>Related assigned lead (not always 1:1)</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="9" t="n"/>
-      <c r="B60" s="14" t="inlineStr">
-        <is>
-          <t>Total Saved</t>
-        </is>
-      </c>
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>Assignment Date</t>
+        </is>
+      </c>
+      <c r="B60" s="9" t="n"/>
       <c r="C60" s="17" t="inlineStr">
         <is>
-          <t>Unfilled</t>
+          <t>Date</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n"/>
-      <c r="B61" s="15" t="inlineStr">
-        <is>
-          <t>max(0, Requested − Sent)</t>
-        </is>
-      </c>
-      <c r="C61" s="18" t="inlineStr">
-        <is>
-          <t>Required − Assignments when open slots remain — NOT the same formula as Total Saved</t>
-        </is>
-      </c>
+      <c r="B61" s="12" t="n"/>
+      <c r="C61" s="18" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>Physical Equipment</t>
+          <t>Start Time</t>
         </is>
       </c>
       <c r="B63" s="14" t="inlineStr">
         <is>
-          <t>AFAD Sent</t>
-        </is>
-      </c>
-      <c r="C63" s="9" t="n"/>
+          <t>Work Hours</t>
+        </is>
+      </c>
+      <c r="C63" s="17" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="12" t="n"/>
+      <c r="A64" s="11" t="n"/>
       <c r="B64" s="15" t="inlineStr">
         <is>
-          <t>(when equipment is AFAD / SmartFlagging gear)</t>
-        </is>
-      </c>
-      <c r="C64" s="18" t="inlineStr">
-        <is>
-          <t>No AFAD count column on Master dashboard view</t>
-        </is>
-      </c>
+          <t>Start of window</t>
+        </is>
+      </c>
+      <c r="C64" s="18" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="9" t="n"/>
+      <c r="A66" s="8" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>Ticket Type</t>
-        </is>
-      </c>
-      <c r="C66" s="17" t="inlineStr">
-        <is>
-          <t>GSF</t>
-        </is>
-      </c>
+          <t>Work Hours</t>
+        </is>
+      </c>
+      <c r="C66" s="9" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="11" t="n"/>
       <c r="B67" s="15" t="inlineStr">
         <is>
-          <t>Value "GSF" marks Guardian SmartFlagging jobs</t>
-        </is>
-      </c>
-      <c r="C67" s="18" t="inlineStr">
-        <is>
-          <t>Yes / No</t>
-        </is>
-      </c>
+          <t>Length of window</t>
+        </is>
+      </c>
+      <c r="C67" s="12" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="9" t="n"/>
-      <c r="B69" s="14" t="inlineStr">
-        <is>
-          <t>AFAD Sent</t>
-        </is>
-      </c>
+      <c r="A69" s="8" t="inlineStr">
+        <is>
+          <t>Job Status</t>
+        </is>
+      </c>
+      <c r="B69" s="9" t="n"/>
       <c r="C69" s="9" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="11" t="n"/>
-      <c r="B70" s="15" t="inlineStr">
-        <is>
-          <t>Count of AFADs sent</t>
-        </is>
-      </c>
-      <c r="C70" s="11" t="n"/>
+      <c r="B70" s="12" t="n"/>
+      <c r="C70" s="12" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="8" t="inlineStr">
-        <is>
-          <t>HP/MP</t>
-        </is>
-      </c>
-      <c r="B72" s="9" t="n"/>
-      <c r="C72" s="9" t="n"/>
+      <c r="A72" s="9" t="n"/>
+      <c r="B72" s="14" t="inlineStr">
+        <is>
+          <t>Ticket Type</t>
+        </is>
+      </c>
+      <c r="C72" s="17" t="inlineStr">
+        <is>
+          <t>GSF</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="12" t="n"/>
-      <c r="B73" s="11" t="n"/>
-      <c r="C73" s="11" t="n"/>
+      <c r="B73" s="15" t="inlineStr">
+        <is>
+          <t>Value "GSF" = Guardian SmartFlagging</t>
+        </is>
+      </c>
+      <c r="C73" s="18" t="inlineStr">
+        <is>
+          <t>Yes / No</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>Customer Level</t>
-        </is>
-      </c>
-      <c r="B75" s="9" t="n"/>
+          <t>Original Equipment</t>
+        </is>
+      </c>
+      <c r="B75" s="14" t="inlineStr">
+        <is>
+          <t>AFAD Sent</t>
+        </is>
+      </c>
       <c r="C75" s="9" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="12" t="n"/>
-      <c r="B76" s="11" t="n"/>
-      <c r="C76" s="11" t="n"/>
+      <c r="A76" s="11" t="inlineStr">
+        <is>
+          <t>Equipment listed on Roads export</t>
+        </is>
+      </c>
+      <c r="B76" s="15" t="inlineStr">
+        <is>
+          <t>When equipment is AFAD / SmartFlagging devices</t>
+        </is>
+      </c>
+      <c r="C76" s="18" t="inlineStr">
+        <is>
+          <t>No AFAD count on Master dashboard</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="8" t="inlineStr">
-        <is>
-          <t>Standard Time Items</t>
-        </is>
-      </c>
-      <c r="B78" s="9" t="n"/>
+      <c r="A78" s="9" t="n"/>
+      <c r="B78" s="14" t="inlineStr">
+        <is>
+          <t>AFAD Sent</t>
+        </is>
+      </c>
       <c r="C78" s="9" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="12" t="n"/>
-      <c r="B79" s="11" t="n"/>
-      <c r="C79" s="11" t="n"/>
+      <c r="B79" s="15" t="inlineStr">
+        <is>
+          <t>Count of AFADs sent</t>
+        </is>
+      </c>
+      <c r="C79" s="12" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="8" t="inlineStr">
-        <is>
-          <t>Total Time Items</t>
-        </is>
-      </c>
-      <c r="B81" s="9" t="n"/>
+      <c r="A81" s="9" t="n"/>
+      <c r="B81" s="14" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
       <c r="C81" s="9" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="12" t="n"/>
-      <c r="B82" s="11" t="n"/>
-      <c r="C82" s="11" t="n"/>
+      <c r="B82" s="15" t="n"/>
+      <c r="C82" s="12" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t>Feedback</t>
+          <t>Comments</t>
         </is>
       </c>
       <c r="B84" s="14" t="inlineStr">
@@ -2236,97 +2518,293 @@
       <c r="C84" s="9" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="12" t="n"/>
+      <c r="A85" s="11" t="n"/>
       <c r="B85" s="15" t="inlineStr">
         <is>
-          <t>(related free-text)</t>
-        </is>
-      </c>
-      <c r="C85" s="11" t="n"/>
+          <t>Related free text</t>
+        </is>
+      </c>
+      <c r="C85" s="12" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t>HP Rate</t>
+          <t>HP/MP</t>
         </is>
       </c>
       <c r="B87" s="9" t="n"/>
       <c r="C87" s="9" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="12" t="n"/>
-      <c r="B88" s="11" t="n"/>
-      <c r="C88" s="11" t="n"/>
+      <c r="A88" s="11" t="n"/>
+      <c r="B88" s="12" t="n"/>
+      <c r="C88" s="12" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t>Level of HP Expertise</t>
+          <t>Customer Level</t>
         </is>
       </c>
       <c r="B90" s="9" t="n"/>
       <c r="C90" s="9" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="12" t="n"/>
-      <c r="B91" s="11" t="n"/>
-      <c r="C91" s="11" t="n"/>
+      <c r="A91" s="11" t="n"/>
+      <c r="B91" s="12" t="n"/>
+      <c r="C91" s="12" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t>Certification Level</t>
+          <t>Standard Time Items</t>
         </is>
       </c>
       <c r="B93" s="9" t="n"/>
       <c r="C93" s="9" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="12" t="n"/>
-      <c r="B94" s="11" t="n"/>
-      <c r="C94" s="11" t="n"/>
+      <c r="A94" s="11" t="n"/>
+      <c r="B94" s="12" t="n"/>
+      <c r="C94" s="12" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t>Certification Expiration</t>
+          <t>Total Time Items</t>
         </is>
       </c>
       <c r="B96" s="9" t="n"/>
       <c r="C96" s="9" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="12" t="n"/>
-      <c r="B97" s="11" t="n"/>
-      <c r="C97" s="11" t="n"/>
+      <c r="A97" s="11" t="n"/>
+      <c r="B97" s="12" t="n"/>
+      <c r="C97" s="12" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t>Bill Rate</t>
+          <t>Feedback</t>
         </is>
       </c>
       <c r="B99" s="9" t="n"/>
       <c r="C99" s="9" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="12" t="n"/>
-      <c r="B100" s="11" t="n"/>
-      <c r="C100" s="11" t="n"/>
+      <c r="A100" s="11" t="n"/>
+      <c r="B100" s="12" t="n"/>
+      <c r="C100" s="12" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="8" t="inlineStr">
         <is>
-          <t>Pay Rate</t>
+          <t>HP Rate</t>
         </is>
       </c>
       <c r="B102" s="9" t="n"/>
       <c r="C102" s="9" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="12" t="n"/>
-      <c r="B103" s="11" t="n"/>
-      <c r="C103" s="11" t="n"/>
+      <c r="A103" s="11" t="n"/>
+      <c r="B103" s="12" t="n"/>
+      <c r="C103" s="12" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="8" t="inlineStr">
+        <is>
+          <t>Level of HP Expertise</t>
+        </is>
+      </c>
+      <c r="B105" s="9" t="n"/>
+      <c r="C105" s="9" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="11" t="n"/>
+      <c r="B106" s="12" t="n"/>
+      <c r="C106" s="12" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="8" t="inlineStr">
+        <is>
+          <t>Certification Level</t>
+        </is>
+      </c>
+      <c r="B108" s="9" t="n"/>
+      <c r="C108" s="9" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="11" t="n"/>
+      <c r="B109" s="12" t="n"/>
+      <c r="C109" s="12" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="8" t="inlineStr">
+        <is>
+          <t>Certification Expiration</t>
+        </is>
+      </c>
+      <c r="B111" s="9" t="n"/>
+      <c r="C111" s="9" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="11" t="n"/>
+      <c r="B112" s="12" t="n"/>
+      <c r="C112" s="12" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="8" t="inlineStr">
+        <is>
+          <t>Bill Rate</t>
+        </is>
+      </c>
+      <c r="B114" s="9" t="n"/>
+      <c r="C114" s="9" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="11" t="n"/>
+      <c r="B115" s="12" t="n"/>
+      <c r="C115" s="12" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="8" t="inlineStr">
+        <is>
+          <t>Pay Rate</t>
+        </is>
+      </c>
+      <c r="B117" s="9" t="n"/>
+      <c r="C117" s="9" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="11" t="n"/>
+      <c r="B118" s="12" t="n"/>
+      <c r="C118" s="12" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="8" t="inlineStr">
+        <is>
+          <t>Billable</t>
+        </is>
+      </c>
+      <c r="B120" s="9" t="n"/>
+      <c r="C120" s="9" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="11" t="n"/>
+      <c r="B121" s="12" t="n"/>
+      <c r="C121" s="12" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="8" t="inlineStr">
+        <is>
+          <t>Billable Override</t>
+        </is>
+      </c>
+      <c r="B123" s="9" t="n"/>
+      <c r="C123" s="9" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="11" t="n"/>
+      <c r="B124" s="12" t="n"/>
+      <c r="C124" s="12" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="8" t="inlineStr">
+        <is>
+          <t>External Billable Override</t>
+        </is>
+      </c>
+      <c r="B126" s="9" t="n"/>
+      <c r="C126" s="9" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="11" t="n"/>
+      <c r="B127" s="12" t="n"/>
+      <c r="C127" s="12" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="8" t="inlineStr">
+        <is>
+          <t>Coordination Note</t>
+        </is>
+      </c>
+      <c r="B129" s="9" t="n"/>
+      <c r="C129" s="9" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="11" t="n"/>
+      <c r="B130" s="12" t="n"/>
+      <c r="C130" s="12" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="8" t="inlineStr">
+        <is>
+          <t>Coordination Status</t>
+        </is>
+      </c>
+      <c r="B132" s="9" t="n"/>
+      <c r="C132" s="9" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="11" t="n"/>
+      <c r="B133" s="12" t="n"/>
+      <c r="C133" s="12" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="8" t="inlineStr">
+        <is>
+          <t>Project Status</t>
+        </is>
+      </c>
+      <c r="B135" s="9" t="n"/>
+      <c r="C135" s="9" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="11" t="n"/>
+      <c r="B136" s="12" t="n"/>
+      <c r="C136" s="12" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="8" t="inlineStr">
+        <is>
+          <t>Configuration Status</t>
+        </is>
+      </c>
+      <c r="B138" s="9" t="n"/>
+      <c r="C138" s="9" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="11" t="n"/>
+      <c r="B139" s="12" t="n"/>
+      <c r="C139" s="12" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="8" t="inlineStr">
+        <is>
+          <t>Last Modified Timestamp</t>
+        </is>
+      </c>
+      <c r="B141" s="9" t="n"/>
+      <c r="C141" s="9" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="11" t="n"/>
+      <c r="B142" s="12" t="n"/>
+      <c r="C142" s="12" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="8" t="inlineStr">
+        <is>
+          <t>Role Timestamp</t>
+        </is>
+      </c>
+      <c r="B144" s="9" t="n"/>
+      <c r="C144" s="9" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="11" t="n"/>
+      <c r="B145" s="12" t="n"/>
+      <c r="C145" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Use consistent colors; stop special-casing Requested vs Required styling
Map Requested Resources with Total Staff Requested and Required once.
Keep Required Resources as its own column. Uniform fills for all stacks.

Co-authored-by: echenry6f <echenry6f@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Roads_Onyx_Master_Column_Crosswalk.xlsx
+++ b/Roads_Onyx_Master_Column_Crosswalk.xlsx
@@ -49,7 +49,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="000D6E6E"/>
+      <color rgb="001A2332"/>
       <sz val="10"/>
     </font>
     <font>
@@ -62,7 +62,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="8"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -80,7 +80,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -94,32 +94,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8F6F0"/>
+        <fgColor rgb="00EEF2F5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF8E8"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0F4FA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F7F7F7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F3E8FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="006B4C9A"/>
+        <fgColor rgb="00F7F9FA"/>
       </patternFill>
     </fill>
   </fills>
@@ -149,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -159,43 +144,16 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -575,48 +533,48 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-    <col width="24" customWidth="1" min="15" max="15"/>
-    <col width="24" customWidth="1" min="16" max="16"/>
-    <col width="24" customWidth="1" min="17" max="17"/>
-    <col width="24" customWidth="1" min="18" max="18"/>
-    <col width="24" customWidth="1" min="19" max="19"/>
-    <col width="24" customWidth="1" min="20" max="20"/>
-    <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="24" customWidth="1" min="22" max="22"/>
-    <col width="24" customWidth="1" min="23" max="23"/>
-    <col width="24" customWidth="1" min="24" max="24"/>
-    <col width="24" customWidth="1" min="25" max="25"/>
-    <col width="24" customWidth="1" min="26" max="26"/>
-    <col width="24" customWidth="1" min="27" max="27"/>
-    <col width="24" customWidth="1" min="28" max="28"/>
-    <col width="24" customWidth="1" min="29" max="29"/>
-    <col width="24" customWidth="1" min="30" max="30"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="21" max="21"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="25" max="25"/>
+    <col width="22" customWidth="1" min="26" max="26"/>
+    <col width="22" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Roads Export ↔ Onyx Report ↔ Master Dashboard (no repeated columns)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="48" customHeight="1">
+          <t>Roads Export ↔ Onyx Report ↔ Master Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Each column name appears only once. Stacked cells in one Excel column are true correspondences. If a field has no twin, it sits alone in its own Excel column (other rows blank). Bold = heading · Italic = formula/rule.</t>
+          <t>Each column name appears once. Stacked values are correspondences; blanks mean no match in that view. Bold = heading · Italic = formula/rule. All columns use the same colors.</t>
         </is>
       </c>
     </row>
@@ -680,545 +638,479 @@
       <c r="S3" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="T3" s="5" t="inlineStr">
-        <is>
-          <t>SOLO</t>
-        </is>
-      </c>
-      <c r="U3" s="5" t="inlineStr">
-        <is>
-          <t>SOLO</t>
-        </is>
-      </c>
-      <c r="V3" s="5" t="inlineStr">
-        <is>
-          <t>SOLO</t>
-        </is>
-      </c>
-      <c r="W3" s="5" t="inlineStr">
-        <is>
-          <t>SOLO</t>
-        </is>
-      </c>
-      <c r="X3" s="5" t="inlineStr">
-        <is>
-          <t>SOLO</t>
-        </is>
-      </c>
-      <c r="Y3" s="5" t="inlineStr">
-        <is>
-          <t>SOLO</t>
-        </is>
-      </c>
-      <c r="Z3" s="5" t="inlineStr">
-        <is>
-          <t>SOLO</t>
-        </is>
-      </c>
-      <c r="AA3" s="5" t="inlineStr">
-        <is>
-          <t>SOLO</t>
-        </is>
-      </c>
-      <c r="AB3" s="5" t="inlineStr">
-        <is>
-          <t>SOLO</t>
-        </is>
-      </c>
-      <c r="AC3" s="5" t="inlineStr">
-        <is>
-          <t>SOLO</t>
-        </is>
-      </c>
-      <c r="AD3" s="5" t="inlineStr">
-        <is>
-          <t>SOLO</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="T3" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="U3" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="V3" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="W3" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="X3" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="Y3" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="Z3" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="AA3" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB3" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="AC3" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="AD3" s="4" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Roads column</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Subcontractor</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Job Number</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>WO Number</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Dispatching</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>Job Location Name</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>Crew Lead</t>
         </is>
       </c>
-      <c r="J4" s="7" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>Foreman</t>
         </is>
       </c>
-      <c r="K4" s="7" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>Assignment Date</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr">
+      <c r="L4" s="6" t="inlineStr">
         <is>
           <t>Start Time</t>
         </is>
       </c>
-      <c r="M4" s="7" t="inlineStr">
+      <c r="M4" s="6" t="inlineStr">
         <is>
           <t>Requested Resources</t>
         </is>
       </c>
-      <c r="N4" s="7" t="inlineStr">
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>Required Resources</t>
         </is>
       </c>
-      <c r="O4" s="7" t="inlineStr">
+      <c r="O4" s="6" t="inlineStr">
         <is>
           <t>Assignment Count</t>
         </is>
       </c>
-      <c r="P4" s="7" t="inlineStr">
+      <c r="P4" s="6" t="inlineStr">
         <is>
           <t>Unfilled Count</t>
         </is>
       </c>
-      <c r="Q4" s="7" t="inlineStr">
+      <c r="Q4" s="7" t="n"/>
+      <c r="R4" s="6" t="inlineStr">
         <is>
           <t>GSF Job</t>
         </is>
       </c>
-      <c r="R4" s="7" t="inlineStr">
+      <c r="S4" s="6" t="inlineStr">
         <is>
           <t>GSF AFAD</t>
         </is>
       </c>
-      <c r="S4" s="7" t="inlineStr">
+      <c r="T4" s="6" t="inlineStr">
         <is>
           <t>Timesheets</t>
         </is>
       </c>
-      <c r="T4" s="8" t="inlineStr">
+      <c r="U4" s="6" t="inlineStr">
         <is>
           <t>Job Location Address</t>
         </is>
       </c>
-      <c r="U4" s="8" t="inlineStr">
+      <c r="V4" s="6" t="inlineStr">
         <is>
           <t>Assigned Employees</t>
         </is>
       </c>
-      <c r="V4" s="8" t="inlineStr">
+      <c r="W4" s="6" t="inlineStr">
         <is>
           <t>Assigned Equipment</t>
         </is>
       </c>
-      <c r="W4" s="8" t="inlineStr">
+      <c r="X4" s="6" t="inlineStr">
         <is>
           <t>GSF Operator</t>
         </is>
       </c>
-      <c r="X4" s="8" t="inlineStr">
+      <c r="Y4" s="6" t="inlineStr">
         <is>
           <t>Second GSF Operator</t>
         </is>
       </c>
-      <c r="Y4" s="8" t="inlineStr">
+      <c r="Z4" s="6" t="inlineStr">
         <is>
           <t>Completed Timesheets</t>
         </is>
       </c>
-      <c r="Z4" s="8" t="inlineStr">
+      <c r="AA4" s="6" t="inlineStr">
         <is>
           <t>Total Timesheets</t>
         </is>
       </c>
-      <c r="AA4" s="8" t="inlineStr">
+      <c r="AB4" s="6" t="inlineStr">
         <is>
           <t>Project Notes</t>
         </is>
       </c>
-      <c r="AB4" s="8" t="inlineStr">
+      <c r="AC4" s="6" t="inlineStr">
         <is>
           <t>Cancellation Count</t>
         </is>
       </c>
-      <c r="AC4" s="8" t="inlineStr">
+      <c r="AD4" s="6" t="inlineStr">
         <is>
           <t>Cancellation Information</t>
         </is>
       </c>
-      <c r="AD4" s="9" t="n"/>
-    </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>(Roads formula)</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n"/>
-      <c r="C5" s="10" t="n"/>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="10" t="n"/>
-      <c r="H5" s="10" t="n"/>
-      <c r="I5" s="10" t="n"/>
-      <c r="J5" s="10" t="n"/>
-      <c r="K5" s="10" t="n"/>
-      <c r="L5" s="10" t="n"/>
-      <c r="M5" s="11" t="inlineStr">
-        <is>
-          <t>Roads requested headcount (often 0 on non-GSF rows in PDF sample)</t>
-        </is>
-      </c>
-      <c r="N5" s="10" t="n"/>
-      <c r="O5" s="10" t="n"/>
-      <c r="P5" s="10" t="n"/>
-      <c r="Q5" s="11" t="inlineStr">
-        <is>
-          <t>Yes / No</t>
-        </is>
-      </c>
-      <c r="R5" s="11" t="inlineStr">
-        <is>
-          <t>Device list (AFD-#### GSF …)</t>
-        </is>
-      </c>
-      <c r="S5" s="11" t="inlineStr">
-        <is>
-          <t>Includes Status, WO#, and Field Notes</t>
-        </is>
-      </c>
-      <c r="T5" s="10" t="n"/>
-      <c r="U5" s="12" t="inlineStr">
-        <is>
-          <t>Named people with Confirmed status — not the same as Assignment Count</t>
-        </is>
-      </c>
-      <c r="V5" s="12" t="inlineStr">
-        <is>
-          <t>Trucks, arrow boards, etc. — broader than GSF AFAD</t>
-        </is>
-      </c>
-      <c r="W5" s="10" t="n"/>
-      <c r="X5" s="10" t="n"/>
-      <c r="Y5" s="10" t="n"/>
-      <c r="Z5" s="10" t="n"/>
-      <c r="AA5" s="10" t="n"/>
-      <c r="AB5" s="10" t="n"/>
-      <c r="AC5" s="10" t="n"/>
-      <c r="AD5" s="10" t="n"/>
-    </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="B5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="8" t="n"/>
+      <c r="H5" s="8" t="n"/>
+      <c r="I5" s="8" t="n"/>
+      <c r="J5" s="8" t="n"/>
+      <c r="K5" s="8" t="n"/>
+      <c r="L5" s="8" t="n"/>
+      <c r="M5" s="8" t="n"/>
+      <c r="N5" s="8" t="n"/>
+      <c r="O5" s="8" t="n"/>
+      <c r="P5" s="8" t="n"/>
+      <c r="Q5" s="8" t="n"/>
+      <c r="R5" s="8" t="n"/>
+      <c r="S5" s="8" t="n"/>
+      <c r="T5" s="8" t="n"/>
+      <c r="U5" s="8" t="n"/>
+      <c r="V5" s="8" t="n"/>
+      <c r="W5" s="8" t="n"/>
+      <c r="X5" s="8" t="n"/>
+      <c r="Y5" s="8" t="n"/>
+      <c r="Z5" s="8" t="n"/>
+      <c r="AA5" s="8" t="n"/>
+      <c r="AB5" s="8" t="n"/>
+      <c r="AC5" s="8" t="n"/>
+      <c r="AD5" s="8" t="n"/>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>cooresponding Onyx Column</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Subcontractor</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Ticket #</t>
         </is>
       </c>
-      <c r="E6" s="9" t="n"/>
-      <c r="F6" s="14" t="inlineStr">
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="G6" s="14" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="I6" s="9" t="n"/>
-      <c r="J6" s="9" t="n"/>
-      <c r="K6" s="9" t="n"/>
-      <c r="L6" s="14" t="inlineStr">
+      <c r="I6" s="7" t="n"/>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="7" t="n"/>
+      <c r="L6" s="6" t="inlineStr">
         <is>
           <t>Work Hours</t>
         </is>
       </c>
-      <c r="M6" s="14" t="inlineStr">
+      <c r="M6" s="6" t="inlineStr">
         <is>
           <t>Total Staff Requested</t>
         </is>
       </c>
-      <c r="N6" s="9" t="n"/>
-      <c r="O6" s="14" t="inlineStr">
+      <c r="N6" s="7" t="n"/>
+      <c r="O6" s="6" t="inlineStr">
         <is>
           <t>Total Staff Sent</t>
         </is>
       </c>
-      <c r="P6" s="9" t="n"/>
-      <c r="Q6" s="14" t="inlineStr">
+      <c r="P6" s="7" t="n"/>
+      <c r="Q6" s="6" t="inlineStr">
+        <is>
+          <t>Total Saved</t>
+        </is>
+      </c>
+      <c r="R6" s="6" t="inlineStr">
         <is>
           <t>Ticket Type</t>
         </is>
       </c>
-      <c r="R6" s="14" t="inlineStr">
+      <c r="S6" s="6" t="inlineStr">
         <is>
           <t>AFAD Sent</t>
         </is>
       </c>
-      <c r="S6" s="14" t="inlineStr">
+      <c r="T6" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="T6" s="9" t="n"/>
-      <c r="U6" s="9" t="n"/>
-      <c r="V6" s="9" t="n"/>
-      <c r="W6" s="9" t="n"/>
-      <c r="X6" s="9" t="n"/>
-      <c r="Y6" s="9" t="n"/>
-      <c r="Z6" s="9" t="n"/>
-      <c r="AA6" s="9" t="n"/>
-      <c r="AB6" s="9" t="n"/>
-      <c r="AC6" s="9" t="n"/>
-      <c r="AD6" s="8" t="inlineStr">
-        <is>
-          <t>Total Saved</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="U6" s="7" t="n"/>
+      <c r="V6" s="7" t="n"/>
+      <c r="W6" s="7" t="n"/>
+      <c r="X6" s="7" t="n"/>
+      <c r="Y6" s="7" t="n"/>
+      <c r="Z6" s="7" t="n"/>
+      <c r="AA6" s="7" t="n"/>
+      <c r="AB6" s="7" t="n"/>
+      <c r="AC6" s="7" t="n"/>
+      <c r="AD6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>(Onyx formula)</t>
         </is>
       </c>
-      <c r="B7" s="10" t="n"/>
-      <c r="C7" s="10" t="n"/>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
-      <c r="H7" s="10" t="n"/>
-      <c r="I7" s="10" t="n"/>
-      <c r="J7" s="10" t="n"/>
-      <c r="K7" s="10" t="n"/>
-      <c r="L7" s="15" t="inlineStr">
-        <is>
-          <t>Onyx window; Master Start is the start clock time</t>
-        </is>
-      </c>
-      <c r="M7" s="10" t="n"/>
-      <c r="N7" s="10" t="n"/>
-      <c r="O7" s="10" t="n"/>
-      <c r="P7" s="10" t="n"/>
-      <c r="Q7" s="15" t="inlineStr">
-        <is>
-          <t>Value "GSF" when GSF Job = Yes</t>
-        </is>
-      </c>
-      <c r="R7" s="15" t="inlineStr">
-        <is>
-          <t>Count of AFAD devices</t>
-        </is>
-      </c>
-      <c r="S7" s="15" t="inlineStr">
-        <is>
-          <t>Maps to Field Notes inside Timesheets</t>
-        </is>
-      </c>
-      <c r="T7" s="10" t="n"/>
-      <c r="U7" s="10" t="n"/>
-      <c r="V7" s="10" t="n"/>
-      <c r="W7" s="10" t="n"/>
-      <c r="X7" s="10" t="n"/>
-      <c r="Y7" s="10" t="n"/>
-      <c r="Z7" s="10" t="n"/>
-      <c r="AA7" s="10" t="n"/>
-      <c r="AB7" s="10" t="n"/>
-      <c r="AC7" s="10" t="n"/>
-      <c r="AD7" s="12" t="inlineStr">
-        <is>
-          <t>max(0, Total Staff Requested − Total Staff Sent) — NOT the same as Unfilled Count</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="8" t="n"/>
+      <c r="H7" s="8" t="n"/>
+      <c r="I7" s="8" t="n"/>
+      <c r="J7" s="8" t="n"/>
+      <c r="K7" s="8" t="n"/>
+      <c r="L7" s="8" t="n"/>
+      <c r="M7" s="8" t="n"/>
+      <c r="N7" s="8" t="n"/>
+      <c r="O7" s="8" t="n"/>
+      <c r="P7" s="8" t="n"/>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>max(0, Total Staff Requested − Total Staff Sent)</t>
+        </is>
+      </c>
+      <c r="R7" s="8" t="n"/>
+      <c r="S7" s="8" t="n"/>
+      <c r="T7" s="8" t="n"/>
+      <c r="U7" s="8" t="n"/>
+      <c r="V7" s="8" t="n"/>
+      <c r="W7" s="8" t="n"/>
+      <c r="X7" s="8" t="n"/>
+      <c r="Y7" s="8" t="n"/>
+      <c r="Z7" s="8" t="n"/>
+      <c r="AA7" s="8" t="n"/>
+      <c r="AB7" s="8" t="n"/>
+      <c r="AC7" s="8" t="n"/>
+      <c r="AD7" s="8" t="n"/>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Cooresponding Master Column</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="17" t="inlineStr">
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Job Number</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>WO Number</t>
         </is>
       </c>
-      <c r="F8" s="17" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Dispatching</t>
         </is>
       </c>
-      <c r="G8" s="17" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="H8" s="17" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Job Location</t>
         </is>
       </c>
-      <c r="I8" s="17" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>Crew Lead</t>
         </is>
       </c>
-      <c r="J8" s="17" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>Customer Foreman</t>
         </is>
       </c>
-      <c r="K8" s="17" t="inlineStr">
+      <c r="K8" s="6" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="L8" s="17" t="inlineStr">
+      <c r="L8" s="6" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="M8" s="9" t="n"/>
-      <c r="N8" s="17" t="inlineStr">
+      <c r="M8" s="6" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="O8" s="17" t="inlineStr">
+      <c r="N8" s="7" t="n"/>
+      <c r="O8" s="6" t="inlineStr">
         <is>
           <t>Assignments</t>
         </is>
       </c>
-      <c r="P8" s="17" t="inlineStr">
+      <c r="P8" s="6" t="inlineStr">
         <is>
           <t>Unfilled</t>
         </is>
       </c>
-      <c r="Q8" s="17" t="inlineStr">
+      <c r="Q8" s="7" t="n"/>
+      <c r="R8" s="6" t="inlineStr">
         <is>
           <t>GSF</t>
         </is>
       </c>
-      <c r="R8" s="9" t="n"/>
-      <c r="S8" s="9" t="n"/>
-      <c r="T8" s="9" t="n"/>
-      <c r="U8" s="9" t="n"/>
-      <c r="V8" s="9" t="n"/>
-      <c r="W8" s="9" t="n"/>
-      <c r="X8" s="9" t="n"/>
-      <c r="Y8" s="9" t="n"/>
-      <c r="Z8" s="9" t="n"/>
-      <c r="AA8" s="9" t="n"/>
-      <c r="AB8" s="9" t="n"/>
-      <c r="AC8" s="9" t="n"/>
-      <c r="AD8" s="9" t="n"/>
-    </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="S8" s="7" t="n"/>
+      <c r="T8" s="7" t="n"/>
+      <c r="U8" s="7" t="n"/>
+      <c r="V8" s="7" t="n"/>
+      <c r="W8" s="7" t="n"/>
+      <c r="X8" s="7" t="n"/>
+      <c r="Y8" s="7" t="n"/>
+      <c r="Z8" s="7" t="n"/>
+      <c r="AA8" s="7" t="n"/>
+      <c r="AB8" s="7" t="n"/>
+      <c r="AC8" s="7" t="n"/>
+      <c r="AD8" s="7" t="n"/>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>(Master formula)</t>
         </is>
       </c>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
-      <c r="H9" s="10" t="n"/>
-      <c r="I9" s="10" t="n"/>
-      <c r="J9" s="10" t="n"/>
-      <c r="K9" s="10" t="n"/>
-      <c r="L9" s="10" t="n"/>
-      <c r="M9" s="10" t="n"/>
-      <c r="N9" s="10" t="n"/>
-      <c r="O9" s="10" t="n"/>
-      <c r="P9" s="10" t="n"/>
-      <c r="Q9" s="18" t="inlineStr">
-        <is>
-          <t>Yes / No</t>
-        </is>
-      </c>
-      <c r="R9" s="10" t="n"/>
-      <c r="S9" s="10" t="n"/>
-      <c r="T9" s="10" t="n"/>
-      <c r="U9" s="10" t="n"/>
-      <c r="V9" s="10" t="n"/>
-      <c r="W9" s="10" t="n"/>
-      <c r="X9" s="10" t="n"/>
-      <c r="Y9" s="10" t="n"/>
-      <c r="Z9" s="10" t="n"/>
-      <c r="AA9" s="10" t="n"/>
-      <c r="AB9" s="10" t="n"/>
-      <c r="AC9" s="10" t="n"/>
-      <c r="AD9" s="10" t="n"/>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="8" t="n"/>
+      <c r="H9" s="8" t="n"/>
+      <c r="I9" s="8" t="n"/>
+      <c r="J9" s="8" t="n"/>
+      <c r="K9" s="8" t="n"/>
+      <c r="L9" s="8" t="n"/>
+      <c r="M9" s="8" t="n"/>
+      <c r="N9" s="8" t="n"/>
+      <c r="O9" s="8" t="n"/>
+      <c r="P9" s="8" t="n"/>
+      <c r="Q9" s="8" t="n"/>
+      <c r="R9" s="8" t="n"/>
+      <c r="S9" s="8" t="n"/>
+      <c r="T9" s="8" t="n"/>
+      <c r="U9" s="8" t="n"/>
+      <c r="V9" s="8" t="n"/>
+      <c r="W9" s="8" t="n"/>
+      <c r="X9" s="8" t="n"/>
+      <c r="Y9" s="8" t="n"/>
+      <c r="Z9" s="8" t="n"/>
+      <c r="AA9" s="8" t="n"/>
+      <c r="AB9" s="8" t="n"/>
+      <c r="AC9" s="8" t="n"/>
+      <c r="AD9" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1247,7 +1139,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Proof: each source column listed once</t>
+          <t>Each source column listed once</t>
         </is>
       </c>
     </row>
@@ -1274,1100 +1166,1100 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B3" s="20" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="C3" s="19" t="n">
+      <c r="C3" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>Onyx:Client; Master:Customer</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C4" s="19" t="n">
+      <c r="C4" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Roads:Customer; Master:Customer</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="19" t="inlineStr">
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>Roads:Customer; Onyx:Client</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Subcontractor</t>
         </is>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="19" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>Onyx:Subcontractor</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Subcontractor</t>
         </is>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="19" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>Roads:Subcontractor</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Job Number</t>
         </is>
       </c>
-      <c r="C8" s="19" t="n">
+      <c r="C8" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>Onyx:Ticket #; Master:Job Number</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Ticket #</t>
         </is>
       </c>
-      <c r="C9" s="19" t="n">
+      <c r="C9" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="19" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Roads:Job Number; Master:Job Number</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Job Number</t>
         </is>
       </c>
-      <c r="C10" s="19" t="n">
+      <c r="C10" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D10" s="19" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>Roads:Job Number; Onyx:Ticket #</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>WO Number</t>
         </is>
       </c>
-      <c r="C11" s="19" t="n">
+      <c r="C11" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="D11" s="19" t="inlineStr">
+      <c r="D11" s="10" t="inlineStr">
         <is>
           <t>Master:WO Number</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>WO Number</t>
         </is>
       </c>
-      <c r="C12" s="19" t="n">
+      <c r="C12" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="D12" s="19" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>Roads:WO Number</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Dispatching</t>
         </is>
       </c>
-      <c r="C13" s="19" t="n">
+      <c r="C13" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="D13" s="19" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>Onyx:Branch; Master:Dispatching</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="C14" s="19" t="n">
+      <c r="C14" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="D14" s="19" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>Roads:Dispatching; Master:Dispatching</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Dispatching</t>
         </is>
       </c>
-      <c r="C15" s="19" t="n">
+      <c r="C15" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="D15" s="19" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>Roads:Dispatching; Onyx:Branch</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="C16" s="19" t="n">
+      <c r="C16" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="D16" s="19" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>Onyx:Job Type; Master:Job Type</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="C17" s="19" t="n">
+      <c r="C17" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="D17" s="19" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>Roads:Job Type; Master:Job Type</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B18" s="20" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="C18" s="19" t="n">
+      <c r="C18" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="D18" s="19" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>Roads:Job Type; Onyx:Job Type</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B19" s="20" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Job Location Name</t>
         </is>
       </c>
-      <c r="C19" s="19" t="n">
+      <c r="C19" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="D19" s="19" t="inlineStr">
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>Onyx:Location; Master:Job Location</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B20" s="20" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="C20" s="19" t="n">
+      <c r="C20" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="D20" s="19" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>Roads:Job Location Name; Master:Job Location</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="inlineStr">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B21" s="20" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Job Location</t>
         </is>
       </c>
-      <c r="C21" s="19" t="n">
+      <c r="C21" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="D21" s="19" t="inlineStr">
+      <c r="D21" s="10" t="inlineStr">
         <is>
           <t>Roads:Job Location Name; Onyx:Location</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B22" s="20" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Crew Lead</t>
         </is>
       </c>
-      <c r="C22" s="19" t="n">
+      <c r="C22" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="D22" s="19" t="inlineStr">
+      <c r="D22" s="10" t="inlineStr">
         <is>
           <t>Master:Crew Lead</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B23" s="20" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>Crew Lead</t>
         </is>
       </c>
-      <c r="C23" s="19" t="n">
+      <c r="C23" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="D23" s="19" t="inlineStr">
+      <c r="D23" s="10" t="inlineStr">
         <is>
           <t>Roads:Crew Lead</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="inlineStr">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B24" s="20" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>Foreman</t>
         </is>
       </c>
-      <c r="C24" s="19" t="n">
+      <c r="C24" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="D24" s="19" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>Master:Customer Foreman</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B25" s="20" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Customer Foreman</t>
         </is>
       </c>
-      <c r="C25" s="19" t="n">
+      <c r="C25" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="D25" s="19" t="inlineStr">
+      <c r="D25" s="10" t="inlineStr">
         <is>
           <t>Roads:Foreman</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="inlineStr">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>Assignment Date</t>
         </is>
       </c>
-      <c r="C26" s="19" t="n">
+      <c r="C26" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="D26" s="19" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
         <is>
           <t>Master:Date</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B27" s="20" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C27" s="19" t="n">
+      <c r="C27" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="D27" s="19" t="inlineStr">
+      <c r="D27" s="10" t="inlineStr">
         <is>
           <t>Roads:Assignment Date</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="inlineStr">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B28" s="20" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>Start Time</t>
         </is>
       </c>
-      <c r="C28" s="19" t="n">
+      <c r="C28" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="D28" s="19" t="inlineStr">
+      <c r="D28" s="10" t="inlineStr">
         <is>
           <t>Onyx:Work Hours; Master:Start</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="inlineStr">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B29" s="20" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>Work Hours</t>
         </is>
       </c>
-      <c r="C29" s="19" t="n">
+      <c r="C29" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="D29" s="19" t="inlineStr">
+      <c r="D29" s="10" t="inlineStr">
         <is>
           <t>Roads:Start Time; Master:Start</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="inlineStr">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B30" s="20" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="C30" s="19" t="n">
+      <c r="C30" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="D30" s="19" t="inlineStr">
+      <c r="D30" s="10" t="inlineStr">
         <is>
           <t>Roads:Start Time; Onyx:Work Hours</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="inlineStr">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B31" s="20" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>Requested Resources</t>
         </is>
       </c>
-      <c r="C31" s="19" t="n">
+      <c r="C31" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="D31" s="19" t="inlineStr">
-        <is>
-          <t>Onyx:Total Staff Requested</t>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>Onyx:Total Staff Requested; Master:Required</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="19" t="inlineStr">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B32" s="20" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>Total Staff Requested</t>
         </is>
       </c>
-      <c r="C32" s="19" t="n">
+      <c r="C32" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="D32" s="19" t="inlineStr">
-        <is>
-          <t>Roads:Requested Resources</t>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>Roads:Requested Resources; Master:Required</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="19" t="inlineStr">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>Roads:Requested Resources; Onyx:Total Staff Requested</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B33" s="20" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>Required Resources</t>
         </is>
       </c>
-      <c r="C33" s="19" t="n">
+      <c r="C34" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="D33" s="19" t="inlineStr">
-        <is>
-          <t>Master:Required</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="19" t="inlineStr">
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>(alone)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>Roads</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Assignment Count</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>Onyx:Total Staff Sent; Master:Assignments</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Onyx</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Total Staff Sent</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>Roads:Assignment Count; Master:Assignments</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B34" s="20" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C34" s="19" t="n">
-        <v>13</v>
-      </c>
-      <c r="D34" s="19" t="inlineStr">
-        <is>
-          <t>Roads:Required Resources</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="19" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Assignments</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>Roads:Assignment Count; Onyx:Total Staff Sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B35" s="20" t="inlineStr">
-        <is>
-          <t>Assignment Count</t>
-        </is>
-      </c>
-      <c r="C35" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="D35" s="19" t="inlineStr">
-        <is>
-          <t>Onyx:Total Staff Sent; Master:Assignments</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="19" t="inlineStr">
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>Unfilled Count</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>Master:Unfilled</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Unfilled</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Roads:Unfilled Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B36" s="20" t="inlineStr">
-        <is>
-          <t>Total Staff Sent</t>
-        </is>
-      </c>
-      <c r="C36" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="D36" s="19" t="inlineStr">
-        <is>
-          <t>Roads:Assignment Count; Master:Assignments</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="19" t="inlineStr">
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>Total Saved</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>(alone)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>Roads</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>GSF Job</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>Onyx:Ticket Type; Master:GSF</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>Onyx</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>Ticket Type</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>Roads:GSF Job; Master:GSF</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B37" s="20" t="inlineStr">
-        <is>
-          <t>Assignments</t>
-        </is>
-      </c>
-      <c r="C37" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="D37" s="19" t="inlineStr">
-        <is>
-          <t>Roads:Assignment Count; Onyx:Total Staff Sent</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="19" t="inlineStr">
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>GSF</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>Roads:GSF Job; Onyx:Ticket Type</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B38" s="20" t="inlineStr">
-        <is>
-          <t>Unfilled Count</t>
-        </is>
-      </c>
-      <c r="C38" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="D38" s="19" t="inlineStr">
-        <is>
-          <t>Master:Unfilled</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="19" t="inlineStr">
-        <is>
-          <t>Master</t>
-        </is>
-      </c>
-      <c r="B39" s="20" t="inlineStr">
-        <is>
-          <t>Unfilled</t>
-        </is>
-      </c>
-      <c r="C39" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="D39" s="19" t="inlineStr">
-        <is>
-          <t>Roads:Unfilled Count</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="19" t="inlineStr">
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>GSF AFAD</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>Onyx:AFAD Sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>Onyx</t>
+        </is>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>AFAD Sent</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>Roads:GSF AFAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B40" s="20" t="inlineStr">
-        <is>
-          <t>GSF Job</t>
-        </is>
-      </c>
-      <c r="C40" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="D40" s="19" t="inlineStr">
-        <is>
-          <t>Onyx:Ticket Type; Master:GSF</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="19" t="inlineStr">
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>Timesheets</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>Onyx:Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B41" s="20" t="inlineStr">
-        <is>
-          <t>Ticket Type</t>
-        </is>
-      </c>
-      <c r="C41" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="D41" s="19" t="inlineStr">
-        <is>
-          <t>Roads:GSF Job; Master:GSF</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="19" t="inlineStr">
-        <is>
-          <t>Master</t>
-        </is>
-      </c>
-      <c r="B42" s="20" t="inlineStr">
-        <is>
-          <t>GSF</t>
-        </is>
-      </c>
-      <c r="C42" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="D42" s="19" t="inlineStr">
-        <is>
-          <t>Roads:GSF Job; Onyx:Ticket Type</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="19" t="inlineStr">
+      <c r="B47" s="11" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="C47" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D47" s="10" t="inlineStr">
+        <is>
+          <t>Roads:Timesheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B43" s="20" t="inlineStr">
-        <is>
-          <t>GSF AFAD</t>
-        </is>
-      </c>
-      <c r="C43" s="19" t="n">
-        <v>17</v>
-      </c>
-      <c r="D43" s="19" t="inlineStr">
-        <is>
-          <t>Onyx:AFAD Sent</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="19" t="inlineStr">
-        <is>
-          <t>Onyx</t>
-        </is>
-      </c>
-      <c r="B44" s="20" t="inlineStr">
-        <is>
-          <t>AFAD Sent</t>
-        </is>
-      </c>
-      <c r="C44" s="19" t="n">
-        <v>17</v>
-      </c>
-      <c r="D44" s="19" t="inlineStr">
-        <is>
-          <t>Roads:GSF AFAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="19" t="inlineStr">
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>Job Location Address</t>
+        </is>
+      </c>
+      <c r="C48" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D48" s="10" t="inlineStr">
+        <is>
+          <t>(alone)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B45" s="20" t="inlineStr">
-        <is>
-          <t>Timesheets</t>
-        </is>
-      </c>
-      <c r="C45" s="19" t="n">
-        <v>18</v>
-      </c>
-      <c r="D45" s="19" t="inlineStr">
-        <is>
-          <t>Onyx:Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="19" t="inlineStr">
-        <is>
-          <t>Onyx</t>
-        </is>
-      </c>
-      <c r="B46" s="20" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="C46" s="19" t="n">
-        <v>18</v>
-      </c>
-      <c r="D46" s="19" t="inlineStr">
-        <is>
-          <t>Roads:Timesheets</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="19" t="inlineStr">
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>Assigned Employees</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>(alone)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B47" s="20" t="inlineStr">
-        <is>
-          <t>Job Location Address</t>
-        </is>
-      </c>
-      <c r="C47" s="19" t="n">
-        <v>19</v>
-      </c>
-      <c r="D47" s="19" t="inlineStr">
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>Assigned Equipment</t>
+        </is>
+      </c>
+      <c r="C50" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D50" s="10" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="19" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B48" s="20" t="inlineStr">
-        <is>
-          <t>Assigned Employees</t>
-        </is>
-      </c>
-      <c r="C48" s="19" t="n">
-        <v>20</v>
-      </c>
-      <c r="D48" s="19" t="inlineStr">
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>GSF Operator</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="19" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B49" s="20" t="inlineStr">
-        <is>
-          <t>Assigned Equipment</t>
-        </is>
-      </c>
-      <c r="C49" s="19" t="n">
-        <v>21</v>
-      </c>
-      <c r="D49" s="19" t="inlineStr">
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>Second GSF Operator</t>
+        </is>
+      </c>
+      <c r="C52" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="19" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B50" s="20" t="inlineStr">
-        <is>
-          <t>GSF Operator</t>
-        </is>
-      </c>
-      <c r="C50" s="19" t="n">
-        <v>22</v>
-      </c>
-      <c r="D50" s="19" t="inlineStr">
+      <c r="B53" s="11" t="inlineStr">
+        <is>
+          <t>Completed Timesheets</t>
+        </is>
+      </c>
+      <c r="C53" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D53" s="10" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="19" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B51" s="20" t="inlineStr">
-        <is>
-          <t>Second GSF Operator</t>
-        </is>
-      </c>
-      <c r="C51" s="19" t="n">
-        <v>23</v>
-      </c>
-      <c r="D51" s="19" t="inlineStr">
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>Total Timesheets</t>
+        </is>
+      </c>
+      <c r="C54" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D54" s="10" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="19" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B52" s="20" t="inlineStr">
-        <is>
-          <t>Completed Timesheets</t>
-        </is>
-      </c>
-      <c r="C52" s="19" t="n">
-        <v>24</v>
-      </c>
-      <c r="D52" s="19" t="inlineStr">
+      <c r="B55" s="11" t="inlineStr">
+        <is>
+          <t>Project Notes</t>
+        </is>
+      </c>
+      <c r="C55" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="D55" s="10" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="19" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B53" s="20" t="inlineStr">
-        <is>
-          <t>Total Timesheets</t>
-        </is>
-      </c>
-      <c r="C53" s="19" t="n">
-        <v>25</v>
-      </c>
-      <c r="D53" s="19" t="inlineStr">
+      <c r="B56" s="11" t="inlineStr">
+        <is>
+          <t>Cancellation Count</t>
+        </is>
+      </c>
+      <c r="C56" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="D56" s="10" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="19" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B54" s="20" t="inlineStr">
-        <is>
-          <t>Project Notes</t>
-        </is>
-      </c>
-      <c r="C54" s="19" t="n">
-        <v>26</v>
-      </c>
-      <c r="D54" s="19" t="inlineStr">
-        <is>
-          <t>(alone)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="19" t="inlineStr">
-        <is>
-          <t>Roads</t>
-        </is>
-      </c>
-      <c r="B55" s="20" t="inlineStr">
-        <is>
-          <t>Cancellation Count</t>
-        </is>
-      </c>
-      <c r="C55" s="19" t="n">
-        <v>27</v>
-      </c>
-      <c r="D55" s="19" t="inlineStr">
-        <is>
-          <t>(alone)</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="19" t="inlineStr">
-        <is>
-          <t>Roads</t>
-        </is>
-      </c>
-      <c r="B56" s="20" t="inlineStr">
+      <c r="B57" s="11" t="inlineStr">
         <is>
           <t>Cancellation Information</t>
         </is>
       </c>
-      <c r="C56" s="19" t="n">
-        <v>28</v>
-      </c>
-      <c r="D56" s="19" t="inlineStr">
-        <is>
-          <t>(alone)</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="19" t="inlineStr">
-        <is>
-          <t>Onyx</t>
-        </is>
-      </c>
-      <c r="B57" s="20" t="inlineStr">
-        <is>
-          <t>Total Saved</t>
-        </is>
-      </c>
-      <c r="C57" s="19" t="n">
+      <c r="C57" s="10" t="n">
         <v>29</v>
       </c>
-      <c r="D57" s="19" t="inlineStr">
+      <c r="D57" s="10" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
@@ -2387,113 +2279,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>Rules for this workbook</t>
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Legend</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="inlineStr"/>
+      <c r="A2" s="13" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="22" t="inlineStr">
-        <is>
-          <t>1) No column name is repeated anywhere in the crosswalk.</t>
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>• Every column name appears only once.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="22" t="inlineStr">
-        <is>
-          <t>2) An Excel column with 2–3 filled name rows = a real correspondence.</t>
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>• Same colors on every stack (no special highlighting).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="22" t="inlineStr">
-        <is>
-          <t>3) An Excel column marked SOLO = that field stands alone (no twin).</t>
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>• Requested Resources ↔ Total Staff Requested ↔ Required.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="inlineStr"/>
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>• Required Resources is listed on its own (not double-mapped to those same fields).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
-        <is>
-          <t>Staffing choices (why not double-map):</t>
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>• Assignment Count ↔ Total Staff Sent ↔ Assignments.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Requested Resources ↔ Total Staff Requested only (not also Master Required).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Required Resources ↔ Required only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Assignment Count ↔ Total Staff Sent ↔ Assignments.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Unfilled Count ↔ Unfilled only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Total Saved is Onyx-only (different formula from Unfilled).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Assigned Employees is Roads-only (names, not the count field).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Assigned Equipment is Roads-only; GSF AFAD ↔ AFAD Sent is the AFAD-specific pair.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Job Location Name ↔ Location ↔ Job Location; Job Location Address is Roads-only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Timesheets ↔ Notes; Project Notes is Roads-only.</t>
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>• Unfilled Count ↔ Unfilled; Total Saved stands alone.</t>
         </is>
       </c>
     </row>
@@ -2511,9 +2351,9 @@
   <dimension ref="A1:C88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2524,579 +2364,535 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="23" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Roads Export</t>
         </is>
       </c>
-      <c r="B2" s="23" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>Onyx Report</t>
         </is>
       </c>
-      <c r="C2" s="23" t="inlineStr">
+      <c r="C2" s="14" t="inlineStr">
         <is>
           <t>Master Dashboard</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C3" s="17" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="n"/>
-      <c r="B4" s="15" t="n"/>
-      <c r="C4" s="18" t="n"/>
+      <c r="A4" s="8" t="n"/>
+      <c r="B4" s="8" t="n"/>
+      <c r="C4" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Subcontractor</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Subcontractor</t>
         </is>
       </c>
-      <c r="C6" s="9" t="n"/>
+      <c r="C6" s="7" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n"/>
-      <c r="B7" s="15" t="n"/>
-      <c r="C7" s="10" t="n"/>
+      <c r="A7" s="8" t="n"/>
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Job Number</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Ticket #</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Job Number</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="15" t="n"/>
-      <c r="C10" s="18" t="n"/>
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>WO Number</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>WO Number</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="18" t="n"/>
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Dispatching</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="C15" s="17" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Dispatching</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n"/>
-      <c r="B16" s="15" t="n"/>
-      <c r="C16" s="18" t="n"/>
+      <c r="A16" s="8" t="n"/>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="B18" s="14" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="C18" s="17" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n"/>
-      <c r="B19" s="15" t="n"/>
-      <c r="C19" s="18" t="n"/>
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="8" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Job Location Name</t>
         </is>
       </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="C21" s="17" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Job Location</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="n"/>
-      <c r="B22" s="15" t="n"/>
-      <c r="C22" s="18" t="n"/>
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="8" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Crew Lead</t>
         </is>
       </c>
-      <c r="B24" s="9" t="n"/>
-      <c r="C24" s="17" t="inlineStr">
+      <c r="B24" s="7" t="n"/>
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>Crew Lead</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="n"/>
-      <c r="B25" s="10" t="n"/>
-      <c r="C25" s="18" t="n"/>
+      <c r="A25" s="8" t="n"/>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="8" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>Foreman</t>
         </is>
       </c>
-      <c r="B27" s="9" t="n"/>
-      <c r="C27" s="17" t="inlineStr">
+      <c r="B27" s="7" t="n"/>
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>Customer Foreman</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="n"/>
-      <c r="B28" s="10" t="n"/>
-      <c r="C28" s="18" t="n"/>
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="8" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Assignment Date</t>
         </is>
       </c>
-      <c r="B30" s="9" t="n"/>
-      <c r="C30" s="17" t="inlineStr">
+      <c r="B30" s="7" t="n"/>
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="n"/>
-      <c r="B31" s="10" t="n"/>
-      <c r="C31" s="18" t="n"/>
+      <c r="A31" s="8" t="n"/>
+      <c r="B31" s="8" t="n"/>
+      <c r="C31" s="8" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="inlineStr">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>Start Time</t>
         </is>
       </c>
-      <c r="B33" s="14" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>Work Hours</t>
         </is>
       </c>
-      <c r="C33" s="17" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="n"/>
-      <c r="B34" s="15" t="inlineStr">
-        <is>
-          <t>Onyx window; Master Start is the start clock time</t>
-        </is>
-      </c>
-      <c r="C34" s="18" t="n"/>
+      <c r="A34" s="8" t="n"/>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="8" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>Requested Resources</t>
         </is>
       </c>
-      <c r="B36" s="14" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>Total Staff Requested</t>
         </is>
       </c>
-      <c r="C36" s="9" t="n"/>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="inlineStr">
-        <is>
-          <t>Roads requested headcount (often 0 on non-GSF rows in PDF sample)</t>
-        </is>
-      </c>
-      <c r="B37" s="15" t="n"/>
-      <c r="C37" s="10" t="n"/>
+      <c r="A37" s="8" t="n"/>
+      <c r="B37" s="8" t="n"/>
+      <c r="C37" s="8" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="inlineStr">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>Required Resources</t>
         </is>
       </c>
-      <c r="B39" s="9" t="n"/>
-      <c r="C39" s="17" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
+      <c r="B39" s="7" t="n"/>
+      <c r="C39" s="7" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="11" t="n"/>
-      <c r="B40" s="10" t="n"/>
-      <c r="C40" s="18" t="n"/>
+      <c r="A40" s="8" t="n"/>
+      <c r="B40" s="8" t="n"/>
+      <c r="C40" s="8" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="inlineStr">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>Assignment Count</t>
         </is>
       </c>
-      <c r="B42" s="14" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>Total Staff Sent</t>
         </is>
       </c>
-      <c r="C42" s="17" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>Assignments</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="n"/>
-      <c r="B43" s="15" t="n"/>
-      <c r="C43" s="18" t="n"/>
+      <c r="A43" s="8" t="n"/>
+      <c r="B43" s="8" t="n"/>
+      <c r="C43" s="8" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>Unfilled Count</t>
         </is>
       </c>
-      <c r="B45" s="9" t="n"/>
-      <c r="C45" s="17" t="inlineStr">
+      <c r="B45" s="7" t="n"/>
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>Unfilled</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="11" t="n"/>
-      <c r="B46" s="10" t="n"/>
-      <c r="C46" s="18" t="n"/>
+      <c r="A46" s="8" t="n"/>
+      <c r="B46" s="8" t="n"/>
+      <c r="C46" s="8" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="inlineStr">
+      <c r="A48" s="7" t="n"/>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>Total Saved</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="n"/>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>max(0, Total Staff Requested − Total Staff Sent)</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
         <is>
           <t>GSF Job</t>
         </is>
       </c>
-      <c r="B48" s="14" t="inlineStr">
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t>Ticket Type</t>
         </is>
       </c>
-      <c r="C48" s="17" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>GSF</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="11" t="inlineStr">
-        <is>
-          <t>Yes / No</t>
-        </is>
-      </c>
-      <c r="B49" s="15" t="inlineStr">
-        <is>
-          <t>Value "GSF" when GSF Job = Yes</t>
-        </is>
-      </c>
-      <c r="C49" s="18" t="inlineStr">
-        <is>
-          <t>Yes / No</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="7" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="8" t="n"/>
+      <c r="B52" s="8" t="n"/>
+      <c r="C52" s="8" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>GSF AFAD</t>
         </is>
       </c>
-      <c r="B51" s="14" t="inlineStr">
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>AFAD Sent</t>
         </is>
       </c>
-      <c r="C51" s="9" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="11" t="inlineStr">
-        <is>
-          <t>Device list (AFD-#### GSF …)</t>
-        </is>
-      </c>
-      <c r="B52" s="15" t="inlineStr">
-        <is>
-          <t>Count of AFAD devices</t>
-        </is>
-      </c>
-      <c r="C52" s="10" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="7" t="inlineStr">
+      <c r="C54" s="7" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="n"/>
+      <c r="B55" s="8" t="n"/>
+      <c r="C55" s="8" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
         <is>
           <t>Timesheets</t>
         </is>
       </c>
-      <c r="B54" s="14" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C54" s="9" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="11" t="inlineStr">
-        <is>
-          <t>Includes Status, WO#, and Field Notes</t>
-        </is>
-      </c>
-      <c r="B55" s="15" t="inlineStr">
-        <is>
-          <t>Maps to Field Notes inside Timesheets</t>
-        </is>
-      </c>
-      <c r="C55" s="10" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
+      <c r="C57" s="7" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="n"/>
+      <c r="B58" s="8" t="n"/>
+      <c r="C58" s="8" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
         <is>
           <t>Job Location Address</t>
         </is>
       </c>
-      <c r="B57" s="9" t="n"/>
-      <c r="C57" s="9" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="12" t="n"/>
-      <c r="B58" s="10" t="n"/>
-      <c r="C58" s="10" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+      <c r="B60" s="7" t="n"/>
+      <c r="C60" s="7" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="n"/>
+      <c r="B61" s="8" t="n"/>
+      <c r="C61" s="8" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
         <is>
           <t>Assigned Employees</t>
         </is>
       </c>
-      <c r="B60" s="9" t="n"/>
-      <c r="C60" s="9" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="12" t="inlineStr">
-        <is>
-          <t>Named people with Confirmed status — not the same as Assignment Count</t>
-        </is>
-      </c>
-      <c r="B61" s="10" t="n"/>
-      <c r="C61" s="10" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="8" t="inlineStr">
+      <c r="B63" s="7" t="n"/>
+      <c r="C63" s="7" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="n"/>
+      <c r="B64" s="8" t="n"/>
+      <c r="C64" s="8" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
         <is>
           <t>Assigned Equipment</t>
         </is>
       </c>
-      <c r="B63" s="9" t="n"/>
-      <c r="C63" s="9" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="12" t="inlineStr">
-        <is>
-          <t>Trucks, arrow boards, etc. — broader than GSF AFAD</t>
-        </is>
-      </c>
-      <c r="B64" s="10" t="n"/>
-      <c r="C64" s="10" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="8" t="inlineStr">
+      <c r="B66" s="7" t="n"/>
+      <c r="C66" s="7" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="n"/>
+      <c r="B67" s="8" t="n"/>
+      <c r="C67" s="8" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
         <is>
           <t>GSF Operator</t>
         </is>
       </c>
-      <c r="B66" s="9" t="n"/>
-      <c r="C66" s="9" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="12" t="n"/>
-      <c r="B67" s="10" t="n"/>
-      <c r="C67" s="10" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="8" t="inlineStr">
+      <c r="B69" s="7" t="n"/>
+      <c r="C69" s="7" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="n"/>
+      <c r="B70" s="8" t="n"/>
+      <c r="C70" s="8" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
         <is>
           <t>Second GSF Operator</t>
         </is>
       </c>
-      <c r="B69" s="9" t="n"/>
-      <c r="C69" s="9" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="12" t="n"/>
-      <c r="B70" s="10" t="n"/>
-      <c r="C70" s="10" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="8" t="inlineStr">
+      <c r="B72" s="7" t="n"/>
+      <c r="C72" s="7" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="n"/>
+      <c r="B73" s="8" t="n"/>
+      <c r="C73" s="8" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
         <is>
           <t>Completed Timesheets</t>
         </is>
       </c>
-      <c r="B72" s="9" t="n"/>
-      <c r="C72" s="9" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="12" t="n"/>
-      <c r="B73" s="10" t="n"/>
-      <c r="C73" s="10" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="8" t="inlineStr">
+      <c r="B75" s="7" t="n"/>
+      <c r="C75" s="7" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="8" t="n"/>
+      <c r="B76" s="8" t="n"/>
+      <c r="C76" s="8" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
         <is>
           <t>Total Timesheets</t>
         </is>
       </c>
-      <c r="B75" s="9" t="n"/>
-      <c r="C75" s="9" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="12" t="n"/>
-      <c r="B76" s="10" t="n"/>
-      <c r="C76" s="10" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="8" t="inlineStr">
+      <c r="B78" s="7" t="n"/>
+      <c r="C78" s="7" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="n"/>
+      <c r="B79" s="8" t="n"/>
+      <c r="C79" s="8" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
         <is>
           <t>Project Notes</t>
         </is>
       </c>
-      <c r="B78" s="9" t="n"/>
-      <c r="C78" s="9" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="12" t="n"/>
-      <c r="B79" s="10" t="n"/>
-      <c r="C79" s="10" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="8" t="inlineStr">
+      <c r="B81" s="7" t="n"/>
+      <c r="C81" s="7" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="n"/>
+      <c r="B82" s="8" t="n"/>
+      <c r="C82" s="8" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
         <is>
           <t>Cancellation Count</t>
         </is>
       </c>
-      <c r="B81" s="9" t="n"/>
-      <c r="C81" s="9" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="12" t="n"/>
-      <c r="B82" s="10" t="n"/>
-      <c r="C82" s="10" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="8" t="inlineStr">
+      <c r="B84" s="7" t="n"/>
+      <c r="C84" s="7" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="n"/>
+      <c r="B85" s="8" t="n"/>
+      <c r="C85" s="8" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
         <is>
           <t>Cancellation Information</t>
         </is>
       </c>
-      <c r="B84" s="9" t="n"/>
-      <c r="C84" s="9" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="12" t="n"/>
-      <c r="B85" s="10" t="n"/>
-      <c r="C85" s="10" t="n"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="9" t="n"/>
-      <c r="B87" s="8" t="inlineStr">
-        <is>
-          <t>Total Saved</t>
-        </is>
-      </c>
-      <c r="C87" s="9" t="n"/>
+      <c r="B87" s="7" t="n"/>
+      <c r="C87" s="7" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="10" t="n"/>
-      <c r="B88" s="12" t="inlineStr">
-        <is>
-          <t>max(0, Total Staff Requested − Total Staff Sent) — NOT the same as Unfilled Count</t>
-        </is>
-      </c>
-      <c r="C88" s="10" t="n"/>
+      <c r="A88" s="8" t="n"/>
+      <c r="B88" s="8" t="n"/>
+      <c r="C88" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Treat Requested and Required the same; uniform column colors
Both Roads Requested Resources and Required Resources stand alone.
Pair Onyx Total Staff Requested with Master Required. Remove special highlighting.

Co-authored-by: echenry6f <echenry6f@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Roads_Onyx_Master_Column_Crosswalk.xlsx
+++ b/Roads_Onyx_Master_Column_Crosswalk.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:AE9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -562,6 +562,7 @@
     <col width="22" customWidth="1" min="28" max="28"/>
     <col width="22" customWidth="1" min="29" max="29"/>
     <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="22" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -571,10 +572,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="44" customHeight="1">
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Each column name appears once. Stacked values are correspondences; blanks mean no match in that view. Bold = heading · Italic = formula/rule. All columns use the same colors.</t>
+          <t>Each column name appears once. Same colors on every stack. Requested Resources and Required Resources are both listed on their own; Onyx Total Staff Requested pairs with Master Required. Bold = heading · Italic = formula/rule.</t>
         </is>
       </c>
     </row>
@@ -671,6 +672,9 @@
       <c r="AD3" s="4" t="n">
         <v>29</v>
       </c>
+      <c r="AE3" s="4" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -743,78 +747,79 @@
           <t>Required Resources</t>
         </is>
       </c>
-      <c r="O4" s="6" t="inlineStr">
+      <c r="O4" s="7" t="n"/>
+      <c r="P4" s="6" t="inlineStr">
         <is>
           <t>Assignment Count</t>
         </is>
       </c>
-      <c r="P4" s="6" t="inlineStr">
+      <c r="Q4" s="6" t="inlineStr">
         <is>
           <t>Unfilled Count</t>
         </is>
       </c>
-      <c r="Q4" s="7" t="n"/>
-      <c r="R4" s="6" t="inlineStr">
+      <c r="R4" s="7" t="n"/>
+      <c r="S4" s="6" t="inlineStr">
         <is>
           <t>GSF Job</t>
         </is>
       </c>
-      <c r="S4" s="6" t="inlineStr">
+      <c r="T4" s="6" t="inlineStr">
         <is>
           <t>GSF AFAD</t>
         </is>
       </c>
-      <c r="T4" s="6" t="inlineStr">
+      <c r="U4" s="6" t="inlineStr">
         <is>
           <t>Timesheets</t>
         </is>
       </c>
-      <c r="U4" s="6" t="inlineStr">
+      <c r="V4" s="6" t="inlineStr">
         <is>
           <t>Job Location Address</t>
         </is>
       </c>
-      <c r="V4" s="6" t="inlineStr">
+      <c r="W4" s="6" t="inlineStr">
         <is>
           <t>Assigned Employees</t>
         </is>
       </c>
-      <c r="W4" s="6" t="inlineStr">
+      <c r="X4" s="6" t="inlineStr">
         <is>
           <t>Assigned Equipment</t>
         </is>
       </c>
-      <c r="X4" s="6" t="inlineStr">
+      <c r="Y4" s="6" t="inlineStr">
         <is>
           <t>GSF Operator</t>
         </is>
       </c>
-      <c r="Y4" s="6" t="inlineStr">
+      <c r="Z4" s="6" t="inlineStr">
         <is>
           <t>Second GSF Operator</t>
         </is>
       </c>
-      <c r="Z4" s="6" t="inlineStr">
+      <c r="AA4" s="6" t="inlineStr">
         <is>
           <t>Completed Timesheets</t>
         </is>
       </c>
-      <c r="AA4" s="6" t="inlineStr">
+      <c r="AB4" s="6" t="inlineStr">
         <is>
           <t>Total Timesheets</t>
         </is>
       </c>
-      <c r="AB4" s="6" t="inlineStr">
+      <c r="AC4" s="6" t="inlineStr">
         <is>
           <t>Project Notes</t>
         </is>
       </c>
-      <c r="AC4" s="6" t="inlineStr">
+      <c r="AD4" s="6" t="inlineStr">
         <is>
           <t>Cancellation Count</t>
         </is>
       </c>
-      <c r="AD4" s="6" t="inlineStr">
+      <c r="AE4" s="6" t="inlineStr">
         <is>
           <t>Cancellation Information</t>
         </is>
@@ -855,6 +860,7 @@
       <c r="AB5" s="8" t="n"/>
       <c r="AC5" s="8" t="n"/>
       <c r="AD5" s="8" t="n"/>
+      <c r="AE5" s="8" t="n"/>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -901,39 +907,39 @@
           <t>Work Hours</t>
         </is>
       </c>
-      <c r="M6" s="6" t="inlineStr">
-        <is>
-          <t>Total Staff Requested</t>
-        </is>
-      </c>
+      <c r="M6" s="7" t="n"/>
       <c r="N6" s="7" t="n"/>
       <c r="O6" s="6" t="inlineStr">
         <is>
+          <t>Total Staff Requested</t>
+        </is>
+      </c>
+      <c r="P6" s="6" t="inlineStr">
+        <is>
           <t>Total Staff Sent</t>
         </is>
       </c>
-      <c r="P6" s="7" t="n"/>
-      <c r="Q6" s="6" t="inlineStr">
+      <c r="Q6" s="7" t="n"/>
+      <c r="R6" s="6" t="inlineStr">
         <is>
           <t>Total Saved</t>
         </is>
       </c>
-      <c r="R6" s="6" t="inlineStr">
+      <c r="S6" s="6" t="inlineStr">
         <is>
           <t>Ticket Type</t>
         </is>
       </c>
-      <c r="S6" s="6" t="inlineStr">
+      <c r="T6" s="6" t="inlineStr">
         <is>
           <t>AFAD Sent</t>
         </is>
       </c>
-      <c r="T6" s="6" t="inlineStr">
+      <c r="U6" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="U6" s="7" t="n"/>
       <c r="V6" s="7" t="n"/>
       <c r="W6" s="7" t="n"/>
       <c r="X6" s="7" t="n"/>
@@ -943,6 +949,7 @@
       <c r="AB6" s="7" t="n"/>
       <c r="AC6" s="7" t="n"/>
       <c r="AD6" s="7" t="n"/>
+      <c r="AE6" s="7" t="n"/>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -965,12 +972,12 @@
       <c r="N7" s="8" t="n"/>
       <c r="O7" s="8" t="n"/>
       <c r="P7" s="8" t="n"/>
-      <c r="Q7" s="9" t="inlineStr">
+      <c r="Q7" s="8" t="n"/>
+      <c r="R7" s="9" t="inlineStr">
         <is>
           <t>max(0, Total Staff Requested − Total Staff Sent)</t>
         </is>
       </c>
-      <c r="R7" s="8" t="n"/>
       <c r="S7" s="8" t="n"/>
       <c r="T7" s="8" t="n"/>
       <c r="U7" s="8" t="n"/>
@@ -983,6 +990,7 @@
       <c r="AB7" s="8" t="n"/>
       <c r="AC7" s="8" t="n"/>
       <c r="AD7" s="8" t="n"/>
+      <c r="AE7" s="8" t="n"/>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -1041,29 +1049,29 @@
           <t>Start</t>
         </is>
       </c>
-      <c r="M8" s="6" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
+      <c r="M8" s="7" t="n"/>
       <c r="N8" s="7" t="n"/>
       <c r="O8" s="6" t="inlineStr">
         <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="P8" s="6" t="inlineStr">
+        <is>
           <t>Assignments</t>
         </is>
       </c>
-      <c r="P8" s="6" t="inlineStr">
+      <c r="Q8" s="6" t="inlineStr">
         <is>
           <t>Unfilled</t>
         </is>
       </c>
-      <c r="Q8" s="7" t="n"/>
-      <c r="R8" s="6" t="inlineStr">
+      <c r="R8" s="7" t="n"/>
+      <c r="S8" s="6" t="inlineStr">
         <is>
           <t>GSF</t>
         </is>
       </c>
-      <c r="S8" s="7" t="n"/>
       <c r="T8" s="7" t="n"/>
       <c r="U8" s="7" t="n"/>
       <c r="V8" s="7" t="n"/>
@@ -1075,6 +1083,7 @@
       <c r="AB8" s="7" t="n"/>
       <c r="AC8" s="7" t="n"/>
       <c r="AD8" s="7" t="n"/>
+      <c r="AE8" s="7" t="n"/>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -1111,6 +1120,7 @@
       <c r="AB9" s="8" t="n"/>
       <c r="AC9" s="8" t="n"/>
       <c r="AD9" s="8" t="n"/>
+      <c r="AE9" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1741,67 +1751,67 @@
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>Onyx:Total Staff Requested; Master:Required</t>
+          <t>(alone)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>Onyx</t>
+          <t>Roads</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Total Staff Requested</t>
+          <t>Required Resources</t>
         </is>
       </c>
       <c r="C32" s="10" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>Roads:Requested Resources; Master:Required</t>
+          <t>(alone)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>Master</t>
+          <t>Onyx</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Total Staff Requested</t>
         </is>
       </c>
       <c r="C33" s="10" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>Roads:Requested Resources; Onyx:Total Staff Requested</t>
+          <t>Master:Required</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>Roads</t>
+          <t>Master</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>Required Resources</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="C34" s="10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>(alone)</t>
+          <t>Onyx:Total Staff Requested</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1827,7 @@
         </is>
       </c>
       <c r="C35" s="10" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
@@ -1837,7 +1847,7 @@
         </is>
       </c>
       <c r="C36" s="10" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
@@ -1857,7 +1867,7 @@
         </is>
       </c>
       <c r="C37" s="10" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
@@ -1877,7 +1887,7 @@
         </is>
       </c>
       <c r="C38" s="10" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
@@ -1897,7 +1907,7 @@
         </is>
       </c>
       <c r="C39" s="10" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
@@ -1917,7 +1927,7 @@
         </is>
       </c>
       <c r="C40" s="10" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
@@ -1937,7 +1947,7 @@
         </is>
       </c>
       <c r="C41" s="10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
@@ -1957,7 +1967,7 @@
         </is>
       </c>
       <c r="C42" s="10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
@@ -1977,7 +1987,7 @@
         </is>
       </c>
       <c r="C43" s="10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
@@ -1997,7 +2007,7 @@
         </is>
       </c>
       <c r="C44" s="10" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
@@ -2017,7 +2027,7 @@
         </is>
       </c>
       <c r="C45" s="10" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
@@ -2037,7 +2047,7 @@
         </is>
       </c>
       <c r="C46" s="10" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
@@ -2057,7 +2067,7 @@
         </is>
       </c>
       <c r="C47" s="10" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
@@ -2077,7 +2087,7 @@
         </is>
       </c>
       <c r="C48" s="10" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
@@ -2097,7 +2107,7 @@
         </is>
       </c>
       <c r="C49" s="10" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
@@ -2117,7 +2127,7 @@
         </is>
       </c>
       <c r="C50" s="10" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
@@ -2137,7 +2147,7 @@
         </is>
       </c>
       <c r="C51" s="10" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
@@ -2157,7 +2167,7 @@
         </is>
       </c>
       <c r="C52" s="10" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
@@ -2177,7 +2187,7 @@
         </is>
       </c>
       <c r="C53" s="10" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
@@ -2197,7 +2207,7 @@
         </is>
       </c>
       <c r="C54" s="10" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
@@ -2217,7 +2227,7 @@
         </is>
       </c>
       <c r="C55" s="10" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
@@ -2237,7 +2247,7 @@
         </is>
       </c>
       <c r="C56" s="10" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
@@ -2257,7 +2267,7 @@
         </is>
       </c>
       <c r="C57" s="10" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
@@ -2298,28 +2308,28 @@
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>• Every column name appears only once.</t>
+          <t>• Same colors on every column.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>• Same colors on every stack (no special highlighting).</t>
+          <t>• Each column name appears only once.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>• Requested Resources ↔ Total Staff Requested ↔ Required.</t>
+          <t>• Requested Resources and Required Resources are treated the same: each stands alone.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>• Required Resources is listed on its own (not double-mapped to those same fields).</t>
+          <t>• Total Staff Requested ↔ Required (Onyx ↔ Master).</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2608,16 +2618,8 @@
           <t>Requested Resources</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>Total Staff Requested</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
+      <c r="B36" s="7" t="n"/>
+      <c r="C36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="n"/>
@@ -2639,19 +2641,15 @@
       <c r="C40" s="8" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>Assignment Count</t>
-        </is>
-      </c>
+      <c r="A42" s="7" t="n"/>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Total Staff Sent</t>
+          <t>Total Staff Requested</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Assignments</t>
+          <t>Required</t>
         </is>
       </c>
     </row>
@@ -2663,13 +2661,17 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Unfilled Count</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="n"/>
+          <t>Assignment Count</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Total Staff Sent</t>
+        </is>
+      </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Unfilled</t>
+          <t>Assignments</t>
         </is>
       </c>
     </row>
@@ -2679,57 +2681,57 @@
       <c r="C46" s="8" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="n"/>
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>Total Saved</t>
-        </is>
-      </c>
-      <c r="C48" s="7" t="n"/>
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>Unfilled Count</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="n"/>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>Unfilled</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="n"/>
-      <c r="B49" s="9" t="inlineStr">
-        <is>
-          <t>max(0, Total Staff Requested − Total Staff Sent)</t>
-        </is>
-      </c>
+      <c r="B49" s="8" t="n"/>
       <c r="C49" s="8" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>GSF Job</t>
-        </is>
-      </c>
+      <c r="A51" s="7" t="n"/>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>Ticket Type</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
-          <t>GSF</t>
-        </is>
-      </c>
+          <t>Total Saved</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="8" t="n"/>
-      <c r="B52" s="8" t="n"/>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>max(0, Total Staff Requested − Total Staff Sent)</t>
+        </is>
+      </c>
       <c r="C52" s="8" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>GSF AFAD</t>
+          <t>GSF Job</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>AFAD Sent</t>
-        </is>
-      </c>
-      <c r="C54" s="7" t="n"/>
+          <t>Ticket Type</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>GSF</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="n"/>
@@ -2739,12 +2741,12 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>Timesheets</t>
+          <t>GSF AFAD</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>AFAD Sent</t>
         </is>
       </c>
       <c r="C57" s="7" t="n"/>
@@ -2757,10 +2759,14 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>Job Location Address</t>
-        </is>
-      </c>
-      <c r="B60" s="7" t="n"/>
+          <t>Timesheets</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
       <c r="C60" s="7" t="n"/>
     </row>
     <row r="61">
@@ -2771,7 +2777,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>Assigned Employees</t>
+          <t>Job Location Address</t>
         </is>
       </c>
       <c r="B63" s="7" t="n"/>
@@ -2785,7 +2791,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>Assigned Equipment</t>
+          <t>Assigned Employees</t>
         </is>
       </c>
       <c r="B66" s="7" t="n"/>
@@ -2799,7 +2805,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>GSF Operator</t>
+          <t>Assigned Equipment</t>
         </is>
       </c>
       <c r="B69" s="7" t="n"/>
@@ -2813,7 +2819,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>Second GSF Operator</t>
+          <t>GSF Operator</t>
         </is>
       </c>
       <c r="B72" s="7" t="n"/>
@@ -2827,7 +2833,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>Completed Timesheets</t>
+          <t>Second GSF Operator</t>
         </is>
       </c>
       <c r="B75" s="7" t="n"/>
@@ -2841,7 +2847,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>Total Timesheets</t>
+          <t>Completed Timesheets</t>
         </is>
       </c>
       <c r="B78" s="7" t="n"/>
@@ -2855,7 +2861,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>Project Notes</t>
+          <t>Total Timesheets</t>
         </is>
       </c>
       <c r="B81" s="7" t="n"/>
@@ -2869,7 +2875,7 @@
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>Cancellation Count</t>
+          <t>Project Notes</t>
         </is>
       </c>
       <c r="B84" s="7" t="n"/>
@@ -2883,7 +2889,7 @@
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>Cancellation Information</t>
+          <t>Cancellation Count</t>
         </is>
       </c>
       <c r="B87" s="7" t="n"/>
@@ -2893,6 +2899,20 @@
       <c r="A88" s="8" t="n"/>
       <c r="B88" s="8" t="n"/>
       <c r="C88" s="8" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="inlineStr">
+        <is>
+          <t>Cancellation Information</t>
+        </is>
+      </c>
+      <c r="B90" s="7" t="n"/>
+      <c r="C90" s="7" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="8" t="n"/>
+      <c r="B91" s="8" t="n"/>
+      <c r="C91" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Restore distinct Roads / Onyx / Master row colors
Keep equal Requested/Required treatment and no repeated column names.

Co-authored-by: echenry6f <echenry6f@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Roads_Onyx_Master_Column_Crosswalk.xlsx
+++ b/Roads_Onyx_Master_Column_Crosswalk.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,7 +49,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001A2332"/>
+      <color rgb="000D6E6E"/>
       <sz val="10"/>
     </font>
     <font>
@@ -73,14 +73,8 @@
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -94,17 +88,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEF2F5"/>
+        <fgColor rgb="00E8F6F0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00FFF8E8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F7F9FA"/>
+        <fgColor rgb="00E8F0FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F7F7"/>
       </patternFill>
     </fill>
   </fills>
@@ -134,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -150,20 +149,36 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -572,10 +587,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1">
+    <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Each column name appears once. Same colors on every stack. Requested Resources and Required Resources are both listed on their own; Onyx Total Staff Requested pairs with Master Required. Bold = heading · Italic = formula/rule.</t>
+          <t>Green = Roads · Cream = Onyx · Blue = Master. Each column name appears once. Blanks mean no match in that view. Bold = heading · Italic = formula/rule.</t>
         </is>
       </c>
     </row>
@@ -863,38 +878,38 @@
       <c r="AE5" s="8" t="n"/>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>cooresponding Onyx Column</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Subcontractor</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>Ticket #</t>
         </is>
       </c>
       <c r="E6" s="7" t="n"/>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="10" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
@@ -902,40 +917,40 @@
       <c r="I6" s="7" t="n"/>
       <c r="J6" s="7" t="n"/>
       <c r="K6" s="7" t="n"/>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="L6" s="10" t="inlineStr">
         <is>
           <t>Work Hours</t>
         </is>
       </c>
       <c r="M6" s="7" t="n"/>
       <c r="N6" s="7" t="n"/>
-      <c r="O6" s="6" t="inlineStr">
+      <c r="O6" s="10" t="inlineStr">
         <is>
           <t>Total Staff Requested</t>
         </is>
       </c>
-      <c r="P6" s="6" t="inlineStr">
+      <c r="P6" s="10" t="inlineStr">
         <is>
           <t>Total Staff Sent</t>
         </is>
       </c>
       <c r="Q6" s="7" t="n"/>
-      <c r="R6" s="6" t="inlineStr">
+      <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Total Saved</t>
         </is>
       </c>
-      <c r="S6" s="6" t="inlineStr">
+      <c r="S6" s="10" t="inlineStr">
         <is>
           <t>Ticket Type</t>
         </is>
       </c>
-      <c r="T6" s="6" t="inlineStr">
+      <c r="T6" s="10" t="inlineStr">
         <is>
           <t>AFAD Sent</t>
         </is>
       </c>
-      <c r="U6" s="6" t="inlineStr">
+      <c r="U6" s="10" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -952,7 +967,7 @@
       <c r="AE6" s="7" t="n"/>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>(Onyx formula)</t>
         </is>
@@ -973,7 +988,7 @@
       <c r="O7" s="8" t="n"/>
       <c r="P7" s="8" t="n"/>
       <c r="Q7" s="8" t="n"/>
-      <c r="R7" s="9" t="inlineStr">
+      <c r="R7" s="11" t="inlineStr">
         <is>
           <t>max(0, Total Staff Requested − Total Staff Sent)</t>
         </is>
@@ -993,81 +1008,81 @@
       <c r="AE7" s="8" t="n"/>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Cooresponding Master Column</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
       <c r="C8" s="7" t="n"/>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>Job Number</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>WO Number</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>Dispatching</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="13" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H8" s="13" t="inlineStr">
         <is>
           <t>Job Location</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I8" s="13" t="inlineStr">
         <is>
           <t>Crew Lead</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J8" s="13" t="inlineStr">
         <is>
           <t>Customer Foreman</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="K8" s="13" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="L8" s="6" t="inlineStr">
+      <c r="L8" s="13" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
       <c r="M8" s="7" t="n"/>
       <c r="N8" s="7" t="n"/>
-      <c r="O8" s="6" t="inlineStr">
+      <c r="O8" s="13" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="P8" s="6" t="inlineStr">
+      <c r="P8" s="13" t="inlineStr">
         <is>
           <t>Assignments</t>
         </is>
       </c>
-      <c r="Q8" s="6" t="inlineStr">
+      <c r="Q8" s="13" t="inlineStr">
         <is>
           <t>Unfilled</t>
         </is>
       </c>
       <c r="R8" s="7" t="n"/>
-      <c r="S8" s="6" t="inlineStr">
+      <c r="S8" s="13" t="inlineStr">
         <is>
           <t>GSF</t>
         </is>
@@ -1086,7 +1101,7 @@
       <c r="AE8" s="7" t="n"/>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>(Master formula)</t>
         </is>
@@ -1176,1100 +1191,1100 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="C3" s="10" t="n">
+      <c r="C3" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" s="16" t="inlineStr">
         <is>
           <t>Onyx:Client; Master:Customer</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C4" s="10" t="n">
+      <c r="C4" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>Roads:Customer; Master:Customer</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="C5" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="16" t="inlineStr">
         <is>
           <t>Roads:Customer; Onyx:Client</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Subcontractor</t>
         </is>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="D6" s="16" t="inlineStr">
         <is>
           <t>Onyx:Subcontractor</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Subcontractor</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="16" t="inlineStr">
         <is>
           <t>Roads:Subcontractor</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>Job Number</t>
         </is>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>Onyx:Ticket #; Master:Job Number</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Ticket #</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>Roads:Job Number; Master:Job Number</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>Job Number</t>
         </is>
       </c>
-      <c r="C10" s="10" t="n">
+      <c r="C10" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>Roads:Job Number; Onyx:Ticket #</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>WO Number</t>
         </is>
       </c>
-      <c r="C11" s="10" t="n">
+      <c r="C11" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>Master:WO Number</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>WO Number</t>
         </is>
       </c>
-      <c r="C12" s="10" t="n">
+      <c r="C12" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D12" s="16" t="inlineStr">
         <is>
           <t>Roads:WO Number</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>Dispatching</t>
         </is>
       </c>
-      <c r="C13" s="10" t="n">
+      <c r="C13" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>Onyx:Branch; Master:Dispatching</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
         <is>
           <t>Roads:Dispatching; Master:Dispatching</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="20" t="inlineStr">
         <is>
           <t>Dispatching</t>
         </is>
       </c>
-      <c r="C15" s="10" t="n">
+      <c r="C15" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D15" s="16" t="inlineStr">
         <is>
           <t>Roads:Dispatching; Onyx:Branch</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="C16" s="10" t="n">
+      <c r="C16" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="16" t="inlineStr">
         <is>
           <t>Onyx:Job Type; Master:Job Type</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="C17" s="10" t="n">
+      <c r="C17" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="D17" s="16" t="inlineStr">
         <is>
           <t>Roads:Job Type; Master:Job Type</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="20" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="C18" s="10" t="n">
+      <c r="C18" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="D18" s="16" t="inlineStr">
         <is>
           <t>Roads:Job Type; Onyx:Job Type</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>Job Location Name</t>
         </is>
       </c>
-      <c r="C19" s="10" t="n">
+      <c r="C19" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="D19" s="16" t="inlineStr">
         <is>
           <t>Onyx:Location; Master:Job Location</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="18" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="C20" s="10" t="n">
+      <c r="C20" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="D20" s="16" t="inlineStr">
         <is>
           <t>Roads:Job Location Name; Master:Job Location</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="20" t="inlineStr">
         <is>
           <t>Job Location</t>
         </is>
       </c>
-      <c r="C21" s="10" t="n">
+      <c r="C21" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="D21" s="10" t="inlineStr">
+      <c r="D21" s="16" t="inlineStr">
         <is>
           <t>Roads:Job Location Name; Onyx:Location</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>Crew Lead</t>
         </is>
       </c>
-      <c r="C22" s="10" t="n">
+      <c r="C22" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="D22" s="10" t="inlineStr">
+      <c r="D22" s="16" t="inlineStr">
         <is>
           <t>Master:Crew Lead</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>Crew Lead</t>
         </is>
       </c>
-      <c r="C23" s="10" t="n">
+      <c r="C23" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D23" s="16" t="inlineStr">
         <is>
           <t>Roads:Crew Lead</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>Foreman</t>
         </is>
       </c>
-      <c r="C24" s="10" t="n">
+      <c r="C24" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="D24" s="10" t="inlineStr">
+      <c r="D24" s="16" t="inlineStr">
         <is>
           <t>Master:Customer Foreman</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B25" s="20" t="inlineStr">
         <is>
           <t>Customer Foreman</t>
         </is>
       </c>
-      <c r="C25" s="10" t="n">
+      <c r="C25" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="D25" s="16" t="inlineStr">
         <is>
           <t>Roads:Foreman</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>Assignment Date</t>
         </is>
       </c>
-      <c r="C26" s="10" t="n">
+      <c r="C26" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="D26" s="10" t="inlineStr">
+      <c r="D26" s="16" t="inlineStr">
         <is>
           <t>Master:Date</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B27" s="20" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C27" s="10" t="n">
+      <c r="C27" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="D27" s="10" t="inlineStr">
+      <c r="D27" s="16" t="inlineStr">
         <is>
           <t>Roads:Assignment Date</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B28" s="11" t="inlineStr">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>Start Time</t>
         </is>
       </c>
-      <c r="C28" s="10" t="n">
+      <c r="C28" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="D28" s="10" t="inlineStr">
+      <c r="D28" s="16" t="inlineStr">
         <is>
           <t>Onyx:Work Hours; Master:Start</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>Work Hours</t>
         </is>
       </c>
-      <c r="C29" s="10" t="n">
+      <c r="C29" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="D29" s="10" t="inlineStr">
+      <c r="D29" s="16" t="inlineStr">
         <is>
           <t>Roads:Start Time; Master:Start</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="inlineStr">
+      <c r="A30" s="19" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="C30" s="10" t="n">
+      <c r="C30" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="D30" s="10" t="inlineStr">
+      <c r="D30" s="16" t="inlineStr">
         <is>
           <t>Roads:Start Time; Onyx:Work Hours</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="inlineStr">
+      <c r="A31" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B31" s="11" t="inlineStr">
+      <c r="B31" s="15" t="inlineStr">
         <is>
           <t>Requested Resources</t>
         </is>
       </c>
-      <c r="C31" s="10" t="n">
+      <c r="C31" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="D31" s="10" t="inlineStr">
+      <c r="D31" s="16" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="inlineStr">
+      <c r="A32" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B32" s="11" t="inlineStr">
+      <c r="B32" s="15" t="inlineStr">
         <is>
           <t>Required Resources</t>
         </is>
       </c>
-      <c r="C32" s="10" t="n">
+      <c r="C32" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="D32" s="10" t="inlineStr">
+      <c r="D32" s="16" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B33" s="11" t="inlineStr">
+      <c r="B33" s="18" t="inlineStr">
         <is>
           <t>Total Staff Requested</t>
         </is>
       </c>
-      <c r="C33" s="10" t="n">
+      <c r="C33" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="D33" s="10" t="inlineStr">
+      <c r="D33" s="16" t="inlineStr">
         <is>
           <t>Master:Required</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="inlineStr">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B34" s="11" t="inlineStr">
+      <c r="B34" s="20" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="C34" s="10" t="n">
+      <c r="C34" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="D34" s="10" t="inlineStr">
+      <c r="D34" s="16" t="inlineStr">
         <is>
           <t>Onyx:Total Staff Requested</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="inlineStr">
+      <c r="A35" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B35" s="11" t="inlineStr">
+      <c r="B35" s="15" t="inlineStr">
         <is>
           <t>Assignment Count</t>
         </is>
       </c>
-      <c r="C35" s="10" t="n">
+      <c r="C35" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="D35" s="10" t="inlineStr">
+      <c r="D35" s="16" t="inlineStr">
         <is>
           <t>Onyx:Total Staff Sent; Master:Assignments</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="inlineStr">
+      <c r="A36" s="17" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B36" s="18" t="inlineStr">
         <is>
           <t>Total Staff Sent</t>
         </is>
       </c>
-      <c r="C36" s="10" t="n">
+      <c r="C36" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="D36" s="10" t="inlineStr">
+      <c r="D36" s="16" t="inlineStr">
         <is>
           <t>Roads:Assignment Count; Master:Assignments</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="inlineStr">
+      <c r="A37" s="19" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B37" s="11" t="inlineStr">
+      <c r="B37" s="20" t="inlineStr">
         <is>
           <t>Assignments</t>
         </is>
       </c>
-      <c r="C37" s="10" t="n">
+      <c r="C37" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="D37" s="10" t="inlineStr">
+      <c r="D37" s="16" t="inlineStr">
         <is>
           <t>Roads:Assignment Count; Onyx:Total Staff Sent</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="inlineStr">
+      <c r="A38" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B38" s="11" t="inlineStr">
+      <c r="B38" s="15" t="inlineStr">
         <is>
           <t>Unfilled Count</t>
         </is>
       </c>
-      <c r="C38" s="10" t="n">
+      <c r="C38" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="D38" s="10" t="inlineStr">
+      <c r="D38" s="16" t="inlineStr">
         <is>
           <t>Master:Unfilled</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="10" t="inlineStr">
+      <c r="A39" s="19" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B39" s="11" t="inlineStr">
+      <c r="B39" s="20" t="inlineStr">
         <is>
           <t>Unfilled</t>
         </is>
       </c>
-      <c r="C39" s="10" t="n">
+      <c r="C39" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="D39" s="10" t="inlineStr">
+      <c r="D39" s="16" t="inlineStr">
         <is>
           <t>Roads:Unfilled Count</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="inlineStr">
+      <c r="A40" s="17" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B40" s="11" t="inlineStr">
+      <c r="B40" s="18" t="inlineStr">
         <is>
           <t>Total Saved</t>
         </is>
       </c>
-      <c r="C40" s="10" t="n">
+      <c r="C40" s="16" t="n">
         <v>17</v>
       </c>
-      <c r="D40" s="10" t="inlineStr">
+      <c r="D40" s="16" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="10" t="inlineStr">
+      <c r="A41" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B41" s="11" t="inlineStr">
+      <c r="B41" s="15" t="inlineStr">
         <is>
           <t>GSF Job</t>
         </is>
       </c>
-      <c r="C41" s="10" t="n">
+      <c r="C41" s="16" t="n">
         <v>18</v>
       </c>
-      <c r="D41" s="10" t="inlineStr">
+      <c r="D41" s="16" t="inlineStr">
         <is>
           <t>Onyx:Ticket Type; Master:GSF</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="10" t="inlineStr">
+      <c r="A42" s="17" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B42" s="11" t="inlineStr">
+      <c r="B42" s="18" t="inlineStr">
         <is>
           <t>Ticket Type</t>
         </is>
       </c>
-      <c r="C42" s="10" t="n">
+      <c r="C42" s="16" t="n">
         <v>18</v>
       </c>
-      <c r="D42" s="10" t="inlineStr">
+      <c r="D42" s="16" t="inlineStr">
         <is>
           <t>Roads:GSF Job; Master:GSF</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="10" t="inlineStr">
+      <c r="A43" s="19" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="B43" s="11" t="inlineStr">
+      <c r="B43" s="20" t="inlineStr">
         <is>
           <t>GSF</t>
         </is>
       </c>
-      <c r="C43" s="10" t="n">
+      <c r="C43" s="16" t="n">
         <v>18</v>
       </c>
-      <c r="D43" s="10" t="inlineStr">
+      <c r="D43" s="16" t="inlineStr">
         <is>
           <t>Roads:GSF Job; Onyx:Ticket Type</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="10" t="inlineStr">
+      <c r="A44" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B44" s="11" t="inlineStr">
+      <c r="B44" s="15" t="inlineStr">
         <is>
           <t>GSF AFAD</t>
         </is>
       </c>
-      <c r="C44" s="10" t="n">
+      <c r="C44" s="16" t="n">
         <v>19</v>
       </c>
-      <c r="D44" s="10" t="inlineStr">
+      <c r="D44" s="16" t="inlineStr">
         <is>
           <t>Onyx:AFAD Sent</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="10" t="inlineStr">
+      <c r="A45" s="17" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B45" s="11" t="inlineStr">
+      <c r="B45" s="18" t="inlineStr">
         <is>
           <t>AFAD Sent</t>
         </is>
       </c>
-      <c r="C45" s="10" t="n">
+      <c r="C45" s="16" t="n">
         <v>19</v>
       </c>
-      <c r="D45" s="10" t="inlineStr">
+      <c r="D45" s="16" t="inlineStr">
         <is>
           <t>Roads:GSF AFAD</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="10" t="inlineStr">
+      <c r="A46" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B46" s="11" t="inlineStr">
+      <c r="B46" s="15" t="inlineStr">
         <is>
           <t>Timesheets</t>
         </is>
       </c>
-      <c r="C46" s="10" t="n">
+      <c r="C46" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="D46" s="10" t="inlineStr">
+      <c r="D46" s="16" t="inlineStr">
         <is>
           <t>Onyx:Notes</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="10" t="inlineStr">
+      <c r="A47" s="17" t="inlineStr">
         <is>
           <t>Onyx</t>
         </is>
       </c>
-      <c r="B47" s="11" t="inlineStr">
+      <c r="B47" s="18" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C47" s="10" t="n">
+      <c r="C47" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="D47" s="10" t="inlineStr">
+      <c r="D47" s="16" t="inlineStr">
         <is>
           <t>Roads:Timesheets</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="10" t="inlineStr">
+      <c r="A48" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B48" s="11" t="inlineStr">
+      <c r="B48" s="15" t="inlineStr">
         <is>
           <t>Job Location Address</t>
         </is>
       </c>
-      <c r="C48" s="10" t="n">
+      <c r="C48" s="16" t="n">
         <v>21</v>
       </c>
-      <c r="D48" s="10" t="inlineStr">
+      <c r="D48" s="16" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="10" t="inlineStr">
+      <c r="A49" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B49" s="11" t="inlineStr">
+      <c r="B49" s="15" t="inlineStr">
         <is>
           <t>Assigned Employees</t>
         </is>
       </c>
-      <c r="C49" s="10" t="n">
+      <c r="C49" s="16" t="n">
         <v>22</v>
       </c>
-      <c r="D49" s="10" t="inlineStr">
+      <c r="D49" s="16" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="10" t="inlineStr">
+      <c r="A50" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B50" s="11" t="inlineStr">
+      <c r="B50" s="15" t="inlineStr">
         <is>
           <t>Assigned Equipment</t>
         </is>
       </c>
-      <c r="C50" s="10" t="n">
+      <c r="C50" s="16" t="n">
         <v>23</v>
       </c>
-      <c r="D50" s="10" t="inlineStr">
+      <c r="D50" s="16" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="10" t="inlineStr">
+      <c r="A51" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B51" s="11" t="inlineStr">
+      <c r="B51" s="15" t="inlineStr">
         <is>
           <t>GSF Operator</t>
         </is>
       </c>
-      <c r="C51" s="10" t="n">
+      <c r="C51" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="D51" s="10" t="inlineStr">
+      <c r="D51" s="16" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="10" t="inlineStr">
+      <c r="A52" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B52" s="11" t="inlineStr">
+      <c r="B52" s="15" t="inlineStr">
         <is>
           <t>Second GSF Operator</t>
         </is>
       </c>
-      <c r="C52" s="10" t="n">
+      <c r="C52" s="16" t="n">
         <v>25</v>
       </c>
-      <c r="D52" s="10" t="inlineStr">
+      <c r="D52" s="16" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="10" t="inlineStr">
+      <c r="A53" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B53" s="11" t="inlineStr">
+      <c r="B53" s="15" t="inlineStr">
         <is>
           <t>Completed Timesheets</t>
         </is>
       </c>
-      <c r="C53" s="10" t="n">
+      <c r="C53" s="16" t="n">
         <v>26</v>
       </c>
-      <c r="D53" s="10" t="inlineStr">
+      <c r="D53" s="16" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="10" t="inlineStr">
+      <c r="A54" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B54" s="11" t="inlineStr">
+      <c r="B54" s="15" t="inlineStr">
         <is>
           <t>Total Timesheets</t>
         </is>
       </c>
-      <c r="C54" s="10" t="n">
+      <c r="C54" s="16" t="n">
         <v>27</v>
       </c>
-      <c r="D54" s="10" t="inlineStr">
+      <c r="D54" s="16" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="10" t="inlineStr">
+      <c r="A55" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B55" s="11" t="inlineStr">
+      <c r="B55" s="15" t="inlineStr">
         <is>
           <t>Project Notes</t>
         </is>
       </c>
-      <c r="C55" s="10" t="n">
+      <c r="C55" s="16" t="n">
         <v>28</v>
       </c>
-      <c r="D55" s="10" t="inlineStr">
+      <c r="D55" s="16" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="10" t="inlineStr">
+      <c r="A56" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B56" s="11" t="inlineStr">
+      <c r="B56" s="15" t="inlineStr">
         <is>
           <t>Cancellation Count</t>
         </is>
       </c>
-      <c r="C56" s="10" t="n">
+      <c r="C56" s="16" t="n">
         <v>29</v>
       </c>
-      <c r="D56" s="10" t="inlineStr">
+      <c r="D56" s="16" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="10" t="inlineStr">
+      <c r="A57" s="14" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
-      <c r="B57" s="11" t="inlineStr">
+      <c r="B57" s="15" t="inlineStr">
         <is>
           <t>Cancellation Information</t>
         </is>
       </c>
-      <c r="C57" s="10" t="n">
+      <c r="C57" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="D57" s="10" t="inlineStr">
+      <c r="D57" s="16" t="inlineStr">
         <is>
           <t>(alone)</t>
         </is>
@@ -2289,61 +2304,85 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr"/>
+      <c r="A2" s="22" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
-        <is>
-          <t>• Same colors on every column.</t>
+      <c r="A3" s="22" t="inlineStr">
+        <is>
+          <t>Colors:</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t>• Each column name appears only once.</t>
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Green rows = Roads Export</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>• Requested Resources and Required Resources are treated the same: each stands alone.</t>
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Cream rows = Onyx Report</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>• Total Staff Requested ↔ Required (Onyx ↔ Master).</t>
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Blue rows = Master Dashboard</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>• Assignment Count ↔ Total Staff Sent ↔ Assignments.</t>
-        </is>
-      </c>
+      <c r="A7" s="22" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>• Unfilled Count ↔ Unfilled; Total Saved stands alone.</t>
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>Rules:</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Each column name appears only once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Requested Resources and Required Resources are treated the same (each alone).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Total Staff Requested ↔ Required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Assignment Count ↔ Total Staff Sent ↔ Assignments.</t>
         </is>
       </c>
     </row>
@@ -2374,17 +2413,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>Roads Export</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Onyx Report</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="C2" s="20" t="inlineStr">
         <is>
           <t>Master Dashboard</t>
         </is>
@@ -2396,12 +2435,12 @@
           <t>Customer</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
@@ -2418,7 +2457,7 @@
           <t>Subcontractor</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Subcontractor</t>
         </is>
@@ -2436,12 +2475,12 @@
           <t>Job Number</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Ticket #</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>Job Number</t>
         </is>
@@ -2459,7 +2498,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n"/>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>WO Number</t>
         </is>
@@ -2476,12 +2515,12 @@
           <t>Dispatching</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="13" t="inlineStr">
         <is>
           <t>Dispatching</t>
         </is>
@@ -2498,12 +2537,12 @@
           <t>Job Type</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C18" s="13" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
@@ -2520,12 +2559,12 @@
           <t>Job Location Name</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="13" t="inlineStr">
         <is>
           <t>Job Location</t>
         </is>
@@ -2543,7 +2582,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n"/>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C24" s="13" t="inlineStr">
         <is>
           <t>Crew Lead</t>
         </is>
@@ -2561,7 +2600,7 @@
         </is>
       </c>
       <c r="B27" s="7" t="n"/>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C27" s="13" t="inlineStr">
         <is>
           <t>Customer Foreman</t>
         </is>
@@ -2579,7 +2618,7 @@
         </is>
       </c>
       <c r="B30" s="7" t="n"/>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C30" s="13" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
@@ -2596,12 +2635,12 @@
           <t>Start Time</t>
         </is>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>Work Hours</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C33" s="13" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
@@ -2642,12 +2681,12 @@
     </row>
     <row r="42">
       <c r="A42" s="7" t="n"/>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B42" s="10" t="inlineStr">
         <is>
           <t>Total Staff Requested</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C42" s="13" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
@@ -2664,12 +2703,12 @@
           <t>Assignment Count</t>
         </is>
       </c>
-      <c r="B45" s="6" t="inlineStr">
+      <c r="B45" s="10" t="inlineStr">
         <is>
           <t>Total Staff Sent</t>
         </is>
       </c>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="C45" s="13" t="inlineStr">
         <is>
           <t>Assignments</t>
         </is>
@@ -2687,7 +2726,7 @@
         </is>
       </c>
       <c r="B48" s="7" t="n"/>
-      <c r="C48" s="6" t="inlineStr">
+      <c r="C48" s="13" t="inlineStr">
         <is>
           <t>Unfilled</t>
         </is>
@@ -2700,7 +2739,7 @@
     </row>
     <row r="51">
       <c r="A51" s="7" t="n"/>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="B51" s="10" t="inlineStr">
         <is>
           <t>Total Saved</t>
         </is>
@@ -2709,7 +2748,7 @@
     </row>
     <row r="52">
       <c r="A52" s="8" t="n"/>
-      <c r="B52" s="9" t="inlineStr">
+      <c r="B52" s="11" t="inlineStr">
         <is>
           <t>max(0, Total Staff Requested − Total Staff Sent)</t>
         </is>
@@ -2722,12 +2761,12 @@
           <t>GSF Job</t>
         </is>
       </c>
-      <c r="B54" s="6" t="inlineStr">
+      <c r="B54" s="10" t="inlineStr">
         <is>
           <t>Ticket Type</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C54" s="13" t="inlineStr">
         <is>
           <t>GSF</t>
         </is>
@@ -2744,7 +2783,7 @@
           <t>GSF AFAD</t>
         </is>
       </c>
-      <c r="B57" s="6" t="inlineStr">
+      <c r="B57" s="10" t="inlineStr">
         <is>
           <t>AFAD Sent</t>
         </is>
@@ -2762,7 +2801,7 @@
           <t>Timesheets</t>
         </is>
       </c>
-      <c r="B60" s="6" t="inlineStr">
+      <c r="B60" s="10" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>

</xml_diff>

<commit_message>
Apply Roads/Onyx/Master row colors to blank cells too
No mapping changes — only fix fills so Requested/Required columns
match the same green/cream/blue row colors as every other stack.

Co-authored-by: echenry6f <echenry6f@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Roads_Onyx_Master_Column_Crosswalk.xlsx
+++ b/Roads_Onyx_Master_Column_Crosswalk.xlsx
@@ -133,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -179,6 +179,12 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -590,7 +596,7 @@
     <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Green = Roads · Cream = Onyx · Blue = Master. Each column name appears once. Blanks mean no match in that view. Bold = heading · Italic = formula/rule.</t>
+          <t>Green = Roads · Cream = Onyx · Blue = Master (row colors apply to every column, including blanks). Each column name appears once. Bold = heading · Italic = formula/rule.</t>
         </is>
       </c>
     </row>
@@ -762,7 +768,7 @@
           <t>Required Resources</t>
         </is>
       </c>
-      <c r="O4" s="7" t="n"/>
+      <c r="O4" s="6" t="n"/>
       <c r="P4" s="6" t="inlineStr">
         <is>
           <t>Assignment Count</t>
@@ -773,7 +779,7 @@
           <t>Unfilled Count</t>
         </is>
       </c>
-      <c r="R4" s="7" t="n"/>
+      <c r="R4" s="6" t="n"/>
       <c r="S4" s="6" t="inlineStr">
         <is>
           <t>GSF Job</t>
@@ -846,36 +852,36 @@
           <t>(Roads formula)</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="8" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="8" t="n"/>
-      <c r="G5" s="8" t="n"/>
-      <c r="H5" s="8" t="n"/>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="8" t="n"/>
-      <c r="K5" s="8" t="n"/>
-      <c r="L5" s="8" t="n"/>
-      <c r="M5" s="8" t="n"/>
-      <c r="N5" s="8" t="n"/>
-      <c r="O5" s="8" t="n"/>
-      <c r="P5" s="8" t="n"/>
-      <c r="Q5" s="8" t="n"/>
-      <c r="R5" s="8" t="n"/>
-      <c r="S5" s="8" t="n"/>
-      <c r="T5" s="8" t="n"/>
-      <c r="U5" s="8" t="n"/>
-      <c r="V5" s="8" t="n"/>
-      <c r="W5" s="8" t="n"/>
-      <c r="X5" s="8" t="n"/>
-      <c r="Y5" s="8" t="n"/>
-      <c r="Z5" s="8" t="n"/>
-      <c r="AA5" s="8" t="n"/>
-      <c r="AB5" s="8" t="n"/>
-      <c r="AC5" s="8" t="n"/>
-      <c r="AD5" s="8" t="n"/>
-      <c r="AE5" s="8" t="n"/>
+      <c r="B5" s="23" t="n"/>
+      <c r="C5" s="23" t="n"/>
+      <c r="D5" s="23" t="n"/>
+      <c r="E5" s="23" t="n"/>
+      <c r="F5" s="23" t="n"/>
+      <c r="G5" s="23" t="n"/>
+      <c r="H5" s="23" t="n"/>
+      <c r="I5" s="23" t="n"/>
+      <c r="J5" s="23" t="n"/>
+      <c r="K5" s="23" t="n"/>
+      <c r="L5" s="23" t="n"/>
+      <c r="M5" s="23" t="n"/>
+      <c r="N5" s="23" t="n"/>
+      <c r="O5" s="23" t="n"/>
+      <c r="P5" s="23" t="n"/>
+      <c r="Q5" s="23" t="n"/>
+      <c r="R5" s="23" t="n"/>
+      <c r="S5" s="23" t="n"/>
+      <c r="T5" s="23" t="n"/>
+      <c r="U5" s="23" t="n"/>
+      <c r="V5" s="23" t="n"/>
+      <c r="W5" s="23" t="n"/>
+      <c r="X5" s="23" t="n"/>
+      <c r="Y5" s="23" t="n"/>
+      <c r="Z5" s="23" t="n"/>
+      <c r="AA5" s="23" t="n"/>
+      <c r="AB5" s="23" t="n"/>
+      <c r="AC5" s="23" t="n"/>
+      <c r="AD5" s="23" t="n"/>
+      <c r="AE5" s="23" t="n"/>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
@@ -898,7 +904,7 @@
           <t>Ticket #</t>
         </is>
       </c>
-      <c r="E6" s="7" t="n"/>
+      <c r="E6" s="10" t="n"/>
       <c r="F6" s="10" t="inlineStr">
         <is>
           <t>Branch</t>
@@ -914,16 +920,16 @@
           <t>Location</t>
         </is>
       </c>
-      <c r="I6" s="7" t="n"/>
-      <c r="J6" s="7" t="n"/>
-      <c r="K6" s="7" t="n"/>
+      <c r="I6" s="10" t="n"/>
+      <c r="J6" s="10" t="n"/>
+      <c r="K6" s="10" t="n"/>
       <c r="L6" s="10" t="inlineStr">
         <is>
           <t>Work Hours</t>
         </is>
       </c>
-      <c r="M6" s="7" t="n"/>
-      <c r="N6" s="7" t="n"/>
+      <c r="M6" s="10" t="n"/>
+      <c r="N6" s="10" t="n"/>
       <c r="O6" s="10" t="inlineStr">
         <is>
           <t>Total Staff Requested</t>
@@ -934,7 +940,7 @@
           <t>Total Staff Sent</t>
         </is>
       </c>
-      <c r="Q6" s="7" t="n"/>
+      <c r="Q6" s="10" t="n"/>
       <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Total Saved</t>
@@ -955,16 +961,16 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="V6" s="7" t="n"/>
-      <c r="W6" s="7" t="n"/>
-      <c r="X6" s="7" t="n"/>
-      <c r="Y6" s="7" t="n"/>
-      <c r="Z6" s="7" t="n"/>
-      <c r="AA6" s="7" t="n"/>
-      <c r="AB6" s="7" t="n"/>
-      <c r="AC6" s="7" t="n"/>
-      <c r="AD6" s="7" t="n"/>
-      <c r="AE6" s="7" t="n"/>
+      <c r="V6" s="10" t="n"/>
+      <c r="W6" s="10" t="n"/>
+      <c r="X6" s="10" t="n"/>
+      <c r="Y6" s="10" t="n"/>
+      <c r="Z6" s="10" t="n"/>
+      <c r="AA6" s="10" t="n"/>
+      <c r="AB6" s="10" t="n"/>
+      <c r="AC6" s="10" t="n"/>
+      <c r="AD6" s="10" t="n"/>
+      <c r="AE6" s="10" t="n"/>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
@@ -972,40 +978,40 @@
           <t>(Onyx formula)</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="8" t="n"/>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="8" t="n"/>
-      <c r="K7" s="8" t="n"/>
-      <c r="L7" s="8" t="n"/>
-      <c r="M7" s="8" t="n"/>
-      <c r="N7" s="8" t="n"/>
-      <c r="O7" s="8" t="n"/>
-      <c r="P7" s="8" t="n"/>
-      <c r="Q7" s="8" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="11" t="n"/>
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="11" t="n"/>
+      <c r="I7" s="11" t="n"/>
+      <c r="J7" s="11" t="n"/>
+      <c r="K7" s="11" t="n"/>
+      <c r="L7" s="11" t="n"/>
+      <c r="M7" s="11" t="n"/>
+      <c r="N7" s="11" t="n"/>
+      <c r="O7" s="11" t="n"/>
+      <c r="P7" s="11" t="n"/>
+      <c r="Q7" s="11" t="n"/>
       <c r="R7" s="11" t="inlineStr">
         <is>
           <t>max(0, Total Staff Requested − Total Staff Sent)</t>
         </is>
       </c>
-      <c r="S7" s="8" t="n"/>
-      <c r="T7" s="8" t="n"/>
-      <c r="U7" s="8" t="n"/>
-      <c r="V7" s="8" t="n"/>
-      <c r="W7" s="8" t="n"/>
-      <c r="X7" s="8" t="n"/>
-      <c r="Y7" s="8" t="n"/>
-      <c r="Z7" s="8" t="n"/>
-      <c r="AA7" s="8" t="n"/>
-      <c r="AB7" s="8" t="n"/>
-      <c r="AC7" s="8" t="n"/>
-      <c r="AD7" s="8" t="n"/>
-      <c r="AE7" s="8" t="n"/>
+      <c r="S7" s="11" t="n"/>
+      <c r="T7" s="11" t="n"/>
+      <c r="U7" s="11" t="n"/>
+      <c r="V7" s="11" t="n"/>
+      <c r="W7" s="11" t="n"/>
+      <c r="X7" s="11" t="n"/>
+      <c r="Y7" s="11" t="n"/>
+      <c r="Z7" s="11" t="n"/>
+      <c r="AA7" s="11" t="n"/>
+      <c r="AB7" s="11" t="n"/>
+      <c r="AC7" s="11" t="n"/>
+      <c r="AD7" s="11" t="n"/>
+      <c r="AE7" s="11" t="n"/>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
@@ -1018,7 +1024,7 @@
           <t>Customer</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n"/>
+      <c r="C8" s="13" t="n"/>
       <c r="D8" s="13" t="inlineStr">
         <is>
           <t>Job Number</t>
@@ -1064,8 +1070,8 @@
           <t>Start</t>
         </is>
       </c>
-      <c r="M8" s="7" t="n"/>
-      <c r="N8" s="7" t="n"/>
+      <c r="M8" s="13" t="n"/>
+      <c r="N8" s="13" t="n"/>
       <c r="O8" s="13" t="inlineStr">
         <is>
           <t>Required</t>
@@ -1081,24 +1087,24 @@
           <t>Unfilled</t>
         </is>
       </c>
-      <c r="R8" s="7" t="n"/>
+      <c r="R8" s="13" t="n"/>
       <c r="S8" s="13" t="inlineStr">
         <is>
           <t>GSF</t>
         </is>
       </c>
-      <c r="T8" s="7" t="n"/>
-      <c r="U8" s="7" t="n"/>
-      <c r="V8" s="7" t="n"/>
-      <c r="W8" s="7" t="n"/>
-      <c r="X8" s="7" t="n"/>
-      <c r="Y8" s="7" t="n"/>
-      <c r="Z8" s="7" t="n"/>
-      <c r="AA8" s="7" t="n"/>
-      <c r="AB8" s="7" t="n"/>
-      <c r="AC8" s="7" t="n"/>
-      <c r="AD8" s="7" t="n"/>
-      <c r="AE8" s="7" t="n"/>
+      <c r="T8" s="13" t="n"/>
+      <c r="U8" s="13" t="n"/>
+      <c r="V8" s="13" t="n"/>
+      <c r="W8" s="13" t="n"/>
+      <c r="X8" s="13" t="n"/>
+      <c r="Y8" s="13" t="n"/>
+      <c r="Z8" s="13" t="n"/>
+      <c r="AA8" s="13" t="n"/>
+      <c r="AB8" s="13" t="n"/>
+      <c r="AC8" s="13" t="n"/>
+      <c r="AD8" s="13" t="n"/>
+      <c r="AE8" s="13" t="n"/>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
@@ -1106,36 +1112,36 @@
           <t>(Master formula)</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="8" t="n"/>
-      <c r="G9" s="8" t="n"/>
-      <c r="H9" s="8" t="n"/>
-      <c r="I9" s="8" t="n"/>
-      <c r="J9" s="8" t="n"/>
-      <c r="K9" s="8" t="n"/>
-      <c r="L9" s="8" t="n"/>
-      <c r="M9" s="8" t="n"/>
-      <c r="N9" s="8" t="n"/>
-      <c r="O9" s="8" t="n"/>
-      <c r="P9" s="8" t="n"/>
-      <c r="Q9" s="8" t="n"/>
-      <c r="R9" s="8" t="n"/>
-      <c r="S9" s="8" t="n"/>
-      <c r="T9" s="8" t="n"/>
-      <c r="U9" s="8" t="n"/>
-      <c r="V9" s="8" t="n"/>
-      <c r="W9" s="8" t="n"/>
-      <c r="X9" s="8" t="n"/>
-      <c r="Y9" s="8" t="n"/>
-      <c r="Z9" s="8" t="n"/>
-      <c r="AA9" s="8" t="n"/>
-      <c r="AB9" s="8" t="n"/>
-      <c r="AC9" s="8" t="n"/>
-      <c r="AD9" s="8" t="n"/>
-      <c r="AE9" s="8" t="n"/>
+      <c r="B9" s="24" t="n"/>
+      <c r="C9" s="24" t="n"/>
+      <c r="D9" s="24" t="n"/>
+      <c r="E9" s="24" t="n"/>
+      <c r="F9" s="24" t="n"/>
+      <c r="G9" s="24" t="n"/>
+      <c r="H9" s="24" t="n"/>
+      <c r="I9" s="24" t="n"/>
+      <c r="J9" s="24" t="n"/>
+      <c r="K9" s="24" t="n"/>
+      <c r="L9" s="24" t="n"/>
+      <c r="M9" s="24" t="n"/>
+      <c r="N9" s="24" t="n"/>
+      <c r="O9" s="24" t="n"/>
+      <c r="P9" s="24" t="n"/>
+      <c r="Q9" s="24" t="n"/>
+      <c r="R9" s="24" t="n"/>
+      <c r="S9" s="24" t="n"/>
+      <c r="T9" s="24" t="n"/>
+      <c r="U9" s="24" t="n"/>
+      <c r="V9" s="24" t="n"/>
+      <c r="W9" s="24" t="n"/>
+      <c r="X9" s="24" t="n"/>
+      <c r="Y9" s="24" t="n"/>
+      <c r="Z9" s="24" t="n"/>
+      <c r="AA9" s="24" t="n"/>
+      <c r="AB9" s="24" t="n"/>
+      <c r="AC9" s="24" t="n"/>
+      <c r="AD9" s="24" t="n"/>
+      <c r="AE9" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2447,9 +2453,9 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="n"/>
-      <c r="B4" s="8" t="n"/>
-      <c r="C4" s="8" t="n"/>
+      <c r="A4" s="23" t="n"/>
+      <c r="B4" s="11" t="n"/>
+      <c r="C4" s="24" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2462,12 +2468,12 @@
           <t>Subcontractor</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n"/>
+      <c r="C6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n"/>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
+      <c r="A7" s="23" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="24" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -2487,9 +2493,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="n"/>
-      <c r="B10" s="8" t="n"/>
-      <c r="C10" s="8" t="n"/>
+      <c r="A10" s="23" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="24" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -2497,7 +2503,7 @@
           <t>WO Number</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n"/>
+      <c r="B12" s="10" t="n"/>
       <c r="C12" s="13" t="inlineStr">
         <is>
           <t>WO Number</t>
@@ -2505,9 +2511,9 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="n"/>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="8" t="n"/>
+      <c r="A13" s="23" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="24" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -2527,9 +2533,9 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="n"/>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="8" t="n"/>
+      <c r="A16" s="23" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="24" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -2549,9 +2555,9 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="n"/>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="8" t="n"/>
+      <c r="A19" s="23" t="n"/>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="24" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -2571,9 +2577,9 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="n"/>
-      <c r="B22" s="8" t="n"/>
-      <c r="C22" s="8" t="n"/>
+      <c r="A22" s="23" t="n"/>
+      <c r="B22" s="11" t="n"/>
+      <c r="C22" s="24" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -2581,7 +2587,7 @@
           <t>Crew Lead</t>
         </is>
       </c>
-      <c r="B24" s="7" t="n"/>
+      <c r="B24" s="10" t="n"/>
       <c r="C24" s="13" t="inlineStr">
         <is>
           <t>Crew Lead</t>
@@ -2589,9 +2595,9 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="n"/>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="8" t="n"/>
+      <c r="A25" s="23" t="n"/>
+      <c r="B25" s="11" t="n"/>
+      <c r="C25" s="24" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -2599,7 +2605,7 @@
           <t>Foreman</t>
         </is>
       </c>
-      <c r="B27" s="7" t="n"/>
+      <c r="B27" s="10" t="n"/>
       <c r="C27" s="13" t="inlineStr">
         <is>
           <t>Customer Foreman</t>
@@ -2607,9 +2613,9 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="n"/>
-      <c r="B28" s="8" t="n"/>
-      <c r="C28" s="8" t="n"/>
+      <c r="A28" s="23" t="n"/>
+      <c r="B28" s="11" t="n"/>
+      <c r="C28" s="24" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -2617,7 +2623,7 @@
           <t>Assignment Date</t>
         </is>
       </c>
-      <c r="B30" s="7" t="n"/>
+      <c r="B30" s="10" t="n"/>
       <c r="C30" s="13" t="inlineStr">
         <is>
           <t>Date</t>
@@ -2625,9 +2631,9 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="n"/>
-      <c r="B31" s="8" t="n"/>
-      <c r="C31" s="8" t="n"/>
+      <c r="A31" s="23" t="n"/>
+      <c r="B31" s="11" t="n"/>
+      <c r="C31" s="24" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -2647,9 +2653,9 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="n"/>
-      <c r="B34" s="8" t="n"/>
-      <c r="C34" s="8" t="n"/>
+      <c r="A34" s="23" t="n"/>
+      <c r="B34" s="11" t="n"/>
+      <c r="C34" s="24" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -2657,13 +2663,13 @@
           <t>Requested Resources</t>
         </is>
       </c>
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="7" t="n"/>
+      <c r="B36" s="10" t="n"/>
+      <c r="C36" s="13" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="n"/>
-      <c r="B37" s="8" t="n"/>
-      <c r="C37" s="8" t="n"/>
+      <c r="A37" s="23" t="n"/>
+      <c r="B37" s="11" t="n"/>
+      <c r="C37" s="24" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -2671,16 +2677,16 @@
           <t>Required Resources</t>
         </is>
       </c>
-      <c r="B39" s="7" t="n"/>
-      <c r="C39" s="7" t="n"/>
+      <c r="B39" s="10" t="n"/>
+      <c r="C39" s="13" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="n"/>
-      <c r="B40" s="8" t="n"/>
-      <c r="C40" s="8" t="n"/>
+      <c r="A40" s="23" t="n"/>
+      <c r="B40" s="11" t="n"/>
+      <c r="C40" s="24" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="n"/>
+      <c r="A42" s="6" t="n"/>
       <c r="B42" s="10" t="inlineStr">
         <is>
           <t>Total Staff Requested</t>
@@ -2693,9 +2699,9 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="n"/>
-      <c r="B43" s="8" t="n"/>
-      <c r="C43" s="8" t="n"/>
+      <c r="A43" s="23" t="n"/>
+      <c r="B43" s="11" t="n"/>
+      <c r="C43" s="24" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
@@ -2715,9 +2721,9 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="n"/>
-      <c r="B46" s="8" t="n"/>
-      <c r="C46" s="8" t="n"/>
+      <c r="A46" s="23" t="n"/>
+      <c r="B46" s="11" t="n"/>
+      <c r="C46" s="24" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
@@ -2725,7 +2731,7 @@
           <t>Unfilled Count</t>
         </is>
       </c>
-      <c r="B48" s="7" t="n"/>
+      <c r="B48" s="10" t="n"/>
       <c r="C48" s="13" t="inlineStr">
         <is>
           <t>Unfilled</t>
@@ -2733,27 +2739,27 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="n"/>
-      <c r="B49" s="8" t="n"/>
-      <c r="C49" s="8" t="n"/>
+      <c r="A49" s="23" t="n"/>
+      <c r="B49" s="11" t="n"/>
+      <c r="C49" s="24" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="n"/>
+      <c r="A51" s="6" t="n"/>
       <c r="B51" s="10" t="inlineStr">
         <is>
           <t>Total Saved</t>
         </is>
       </c>
-      <c r="C51" s="7" t="n"/>
+      <c r="C51" s="13" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="8" t="n"/>
+      <c r="A52" s="23" t="n"/>
       <c r="B52" s="11" t="inlineStr">
         <is>
           <t>max(0, Total Staff Requested − Total Staff Sent)</t>
         </is>
       </c>
-      <c r="C52" s="8" t="n"/>
+      <c r="C52" s="24" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
@@ -2773,9 +2779,9 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="8" t="n"/>
-      <c r="B55" s="8" t="n"/>
-      <c r="C55" s="8" t="n"/>
+      <c r="A55" s="23" t="n"/>
+      <c r="B55" s="11" t="n"/>
+      <c r="C55" s="24" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
@@ -2788,12 +2794,12 @@
           <t>AFAD Sent</t>
         </is>
       </c>
-      <c r="C57" s="7" t="n"/>
+      <c r="C57" s="13" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="8" t="n"/>
-      <c r="B58" s="8" t="n"/>
-      <c r="C58" s="8" t="n"/>
+      <c r="A58" s="23" t="n"/>
+      <c r="B58" s="11" t="n"/>
+      <c r="C58" s="24" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
@@ -2806,12 +2812,12 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="C60" s="7" t="n"/>
+      <c r="C60" s="13" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="8" t="n"/>
-      <c r="B61" s="8" t="n"/>
-      <c r="C61" s="8" t="n"/>
+      <c r="A61" s="23" t="n"/>
+      <c r="B61" s="11" t="n"/>
+      <c r="C61" s="24" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
@@ -2819,13 +2825,13 @@
           <t>Job Location Address</t>
         </is>
       </c>
-      <c r="B63" s="7" t="n"/>
-      <c r="C63" s="7" t="n"/>
+      <c r="B63" s="10" t="n"/>
+      <c r="C63" s="13" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="8" t="n"/>
-      <c r="B64" s="8" t="n"/>
-      <c r="C64" s="8" t="n"/>
+      <c r="A64" s="23" t="n"/>
+      <c r="B64" s="11" t="n"/>
+      <c r="C64" s="24" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
@@ -2833,13 +2839,13 @@
           <t>Assigned Employees</t>
         </is>
       </c>
-      <c r="B66" s="7" t="n"/>
-      <c r="C66" s="7" t="n"/>
+      <c r="B66" s="10" t="n"/>
+      <c r="C66" s="13" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="8" t="n"/>
-      <c r="B67" s="8" t="n"/>
-      <c r="C67" s="8" t="n"/>
+      <c r="A67" s="23" t="n"/>
+      <c r="B67" s="11" t="n"/>
+      <c r="C67" s="24" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
@@ -2847,13 +2853,13 @@
           <t>Assigned Equipment</t>
         </is>
       </c>
-      <c r="B69" s="7" t="n"/>
-      <c r="C69" s="7" t="n"/>
+      <c r="B69" s="10" t="n"/>
+      <c r="C69" s="13" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="8" t="n"/>
-      <c r="B70" s="8" t="n"/>
-      <c r="C70" s="8" t="n"/>
+      <c r="A70" s="23" t="n"/>
+      <c r="B70" s="11" t="n"/>
+      <c r="C70" s="24" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
@@ -2861,13 +2867,13 @@
           <t>GSF Operator</t>
         </is>
       </c>
-      <c r="B72" s="7" t="n"/>
-      <c r="C72" s="7" t="n"/>
+      <c r="B72" s="10" t="n"/>
+      <c r="C72" s="13" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="8" t="n"/>
-      <c r="B73" s="8" t="n"/>
-      <c r="C73" s="8" t="n"/>
+      <c r="A73" s="23" t="n"/>
+      <c r="B73" s="11" t="n"/>
+      <c r="C73" s="24" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
@@ -2875,13 +2881,13 @@
           <t>Second GSF Operator</t>
         </is>
       </c>
-      <c r="B75" s="7" t="n"/>
-      <c r="C75" s="7" t="n"/>
+      <c r="B75" s="10" t="n"/>
+      <c r="C75" s="13" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="8" t="n"/>
-      <c r="B76" s="8" t="n"/>
-      <c r="C76" s="8" t="n"/>
+      <c r="A76" s="23" t="n"/>
+      <c r="B76" s="11" t="n"/>
+      <c r="C76" s="24" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
@@ -2889,13 +2895,13 @@
           <t>Completed Timesheets</t>
         </is>
       </c>
-      <c r="B78" s="7" t="n"/>
-      <c r="C78" s="7" t="n"/>
+      <c r="B78" s="10" t="n"/>
+      <c r="C78" s="13" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="8" t="n"/>
-      <c r="B79" s="8" t="n"/>
-      <c r="C79" s="8" t="n"/>
+      <c r="A79" s="23" t="n"/>
+      <c r="B79" s="11" t="n"/>
+      <c r="C79" s="24" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
@@ -2903,13 +2909,13 @@
           <t>Total Timesheets</t>
         </is>
       </c>
-      <c r="B81" s="7" t="n"/>
-      <c r="C81" s="7" t="n"/>
+      <c r="B81" s="10" t="n"/>
+      <c r="C81" s="13" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="8" t="n"/>
-      <c r="B82" s="8" t="n"/>
-      <c r="C82" s="8" t="n"/>
+      <c r="A82" s="23" t="n"/>
+      <c r="B82" s="11" t="n"/>
+      <c r="C82" s="24" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
@@ -2917,13 +2923,13 @@
           <t>Project Notes</t>
         </is>
       </c>
-      <c r="B84" s="7" t="n"/>
-      <c r="C84" s="7" t="n"/>
+      <c r="B84" s="10" t="n"/>
+      <c r="C84" s="13" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="8" t="n"/>
-      <c r="B85" s="8" t="n"/>
-      <c r="C85" s="8" t="n"/>
+      <c r="A85" s="23" t="n"/>
+      <c r="B85" s="11" t="n"/>
+      <c r="C85" s="24" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
@@ -2931,13 +2937,13 @@
           <t>Cancellation Count</t>
         </is>
       </c>
-      <c r="B87" s="7" t="n"/>
-      <c r="C87" s="7" t="n"/>
+      <c r="B87" s="10" t="n"/>
+      <c r="C87" s="13" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="8" t="n"/>
-      <c r="B88" s="8" t="n"/>
-      <c r="C88" s="8" t="n"/>
+      <c r="A88" s="23" t="n"/>
+      <c r="B88" s="11" t="n"/>
+      <c r="C88" s="24" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
@@ -2945,13 +2951,13 @@
           <t>Cancellation Information</t>
         </is>
       </c>
-      <c r="B90" s="7" t="n"/>
-      <c r="C90" s="7" t="n"/>
+      <c r="B90" s="10" t="n"/>
+      <c r="C90" s="13" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="8" t="n"/>
-      <c r="B91" s="8" t="n"/>
-      <c r="C91" s="8" t="n"/>
+      <c r="A91" s="23" t="n"/>
+      <c r="B91" s="11" t="n"/>
+      <c r="C91" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Add number-calculation formulas to notes and Formulas sheet
Document how Total Saved, Unfilled, Assignment Count, AFAD Sent, and
related numeric fields are derived, alongside correspondence notes.

Co-authored-by: echenry6f <echenry6f@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Roads_Onyx_Master_Column_Crosswalk.xlsx
+++ b/Roads_Onyx_Master_Column_Crosswalk.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column Crosswalk" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend &amp; Notes" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correspondence Index" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Number Formulas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,6 +71,11 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -127,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -166,9 +172,16 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -538,34 +551,34 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
-    <col width="18" customWidth="1" min="25" max="25"/>
-    <col width="18" customWidth="1" min="26" max="26"/>
-    <col width="18" customWidth="1" min="27" max="27"/>
-    <col width="18" customWidth="1" min="28" max="28"/>
-    <col width="18" customWidth="1" min="29" max="29"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="20" customWidth="1" min="28" max="28"/>
+    <col width="20" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -575,10 +588,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="56" customHeight="1">
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Columns stay in each file’s listed order (REC / OX / MD numbering). Green = Roads Export (REC) · Cream = Onyx (OX) · Blue = Master Dashboard (MD). If a field matches another system’s column that is not directly above/below, the formula row notes e.g. (Corresponds with 17 in REC and 13 in MD). Bold = heading · Italic = formula / correspondence note.</t>
+          <t>Columns stay in each file’s listed order (REC / OX / MD numbering). Green = Roads Export (REC) · Cream = Onyx (OX) · Blue = Master Dashboard (MD). Italic notes include calculation formulas where numbers are derived, and (Corresponds with …) when a match is not directly above/below. Bold = heading · Italic = formula / notes.</t>
         </is>
       </c>
     </row>
@@ -673,7 +686,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" ht="40" customHeight="1">
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Roads Export (REC)</t>
@@ -820,7 +833,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="40" customHeight="1">
+    <row r="5" ht="48" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>(REC formula / notes)</t>
@@ -828,11 +841,19 @@
       </c>
       <c r="B5" s="7" t="n"/>
       <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Entered / imported requested headcount (often 0 on non-GSF rows in sample)</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Entered / imported required headcount for the job</t>
+        </is>
+      </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>(Corresponds with 12 in MD)</t>
+          <t>Unfilled Count = max(0, Required Resources − Assignment Count) · (Corresponds with 12 in MD)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -844,7 +865,7 @@
       <c r="I5" s="7" t="n"/>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>(Corresponds with 12 in OX)</t>
+          <t>List of assigned GSF AFAD devices; OX AFAD Sent = COUNT of those devices · (Corresponds with 12 in OX)</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
@@ -885,11 +906,19 @@
       </c>
       <c r="S5" s="7" t="inlineStr">
         <is>
-          <t>(Corresponds with 10 in OX and 11 in MD)</t>
-        </is>
-      </c>
-      <c r="T5" s="7" t="n"/>
-      <c r="U5" s="7" t="n"/>
+          <t>Assignment Count = COUNT of confirmed people in Assigned Employees · (Corresponds with 10 in OX and 11 in MD)</t>
+        </is>
+      </c>
+      <c r="T5" s="7" t="inlineStr">
+        <is>
+          <t>Completed Timesheets = COUNT of timesheets with completed/approved status</t>
+        </is>
+      </c>
+      <c r="U5" s="7" t="inlineStr">
+        <is>
+          <t>Total Timesheets = COUNT of all timesheets on the job</t>
+        </is>
+      </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
           <t>(Corresponds with 13 in OX)</t>
@@ -902,7 +931,11 @@
       </c>
       <c r="X5" s="7" t="n"/>
       <c r="Y5" s="7" t="n"/>
-      <c r="Z5" s="7" t="n"/>
+      <c r="Z5" s="7" t="inlineStr">
+        <is>
+          <t>Cancellation Count = COUNT of cancellation records in Cancellation Information</t>
+        </is>
+      </c>
       <c r="AA5" s="7" t="n"/>
       <c r="AB5" s="7" t="inlineStr">
         <is>
@@ -911,7 +944,7 @@
       </c>
       <c r="AC5" s="7" t="n"/>
     </row>
-    <row r="6" ht="40" customHeight="1">
+    <row r="6" ht="48" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Onyx (OX)</t>
@@ -998,7 +1031,7 @@
       <c r="AB6" s="9" t="n"/>
       <c r="AC6" s="9" t="n"/>
     </row>
-    <row r="7" ht="40" customHeight="1">
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>(OX formula / notes)</t>
@@ -1038,22 +1071,22 @@
       </c>
       <c r="J7" s="10" t="inlineStr">
         <is>
-          <t>(Corresponds with 10 in MD)</t>
+          <t>Entered / imported staff requested (or pulled from dispatch) · (Corresponds with 10 in MD)</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
-          <t>(Corresponds with 18 in REC and 11 in MD)</t>
+          <t>Entered / imported staff sent (or pulled from dispatch) · (Corresponds with 18 in REC and 11 in MD)</t>
         </is>
       </c>
       <c r="L7" s="10" t="inlineStr">
         <is>
-          <t>max(0, Total Staff Requested − Total Staff Sent)</t>
+          <t>Total Saved = max(0, Total Staff Requested − Total Staff Sent)</t>
         </is>
       </c>
       <c r="M7" s="10" t="inlineStr">
         <is>
-          <t>(Corresponds with 9 in REC)</t>
+          <t>AFAD Sent = COUNT of GSF AFAD devices on REC GSF AFAD for that job · (Corresponds with 9 in REC)</t>
         </is>
       </c>
       <c r="N7" s="10" t="inlineStr">
@@ -1077,7 +1110,7 @@
       <c r="AB7" s="10" t="n"/>
       <c r="AC7" s="10" t="n"/>
     </row>
-    <row r="8" ht="40" customHeight="1">
+    <row r="8" ht="48" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Master Dashboard (MD)</t>
@@ -1168,7 +1201,7 @@
       <c r="AB8" s="12" t="n"/>
       <c r="AC8" s="12" t="n"/>
     </row>
-    <row r="9" ht="40" customHeight="1">
+    <row r="9" ht="48" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>(MD formula / notes)</t>
@@ -1217,17 +1250,17 @@
       </c>
       <c r="K9" s="13" t="inlineStr">
         <is>
-          <t>(Corresponds with 9 in OX)</t>
+          <t>Entered / imported required headcount for the job · (Corresponds with 9 in OX)</t>
         </is>
       </c>
       <c r="L9" s="13" t="inlineStr">
         <is>
-          <t>(Corresponds with 18 in REC and 10 in OX)</t>
+          <t>Entered / imported assigned headcount (filled slots) · (Corresponds with 18 in REC and 10 in OX)</t>
         </is>
       </c>
       <c r="M9" s="13" t="inlineStr">
         <is>
-          <t>(Corresponds with 5 in REC)</t>
+          <t>Unfilled = Required − Assignments · (Corresponds with 5 in REC)</t>
         </is>
       </c>
       <c r="N9" s="13" t="inlineStr">
@@ -1270,7 +1303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1279,7 +1312,7 @@
     <row r="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>How to read this sheet</t>
+          <t>How to read this sheet + number formulas</t>
         </is>
       </c>
     </row>
@@ -1289,83 +1322,74 @@
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>Abbreviations:</t>
+          <t>Abbreviations: REC = Roads Export · OX = Onyx · MD = Master Dashboard</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • REC = Roads Export</t>
-        </is>
-      </c>
+      <c r="A4" s="15" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • OX = Onyx</t>
+          <t>Colors: Green = REC · Cream = OX · Blue = MD (including blank cells in that row).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • MD = Master Dashboard</t>
-        </is>
-      </c>
+      <c r="A6" s="15" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr"/>
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>Correspondence notes appear only when a match is NOT directly above/below, e.g.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>Order:</t>
+          <t xml:space="preserve">  (Corresponds with 17 in REC and 13 in MD)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • REC columns 1–28 are in Roads Export PDF order (not regrouped).</t>
-        </is>
-      </c>
+      <c r="A9" s="15" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • OX columns 1–13 are in Onyx report order.</t>
-        </is>
+      <c r="A10" s="16">
+        <f>========= NUMBER FORMULAS ==========</f>
+        <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • MD columns 1–14 are in Master Dashboard order.</t>
-        </is>
-      </c>
+      <c r="A11" s="15" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • The Index row is that position number within each file’s list.</t>
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Onyx (OX):</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr"/>
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Total Saved = max(0, Total Staff Requested − Total Staff Sent)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>Colors:</t>
+          <t xml:space="preserve">  • AFAD Sent = COUNT of GSF AFAD devices listed on REC GSF AFAD for that job</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Green = REC · Cream = OX · Blue = MD (including blank cells in that row).</t>
+          <t xml:space="preserve">  • Total Staff Requested / Total Staff Sent = entered or pulled from dispatch (inputs)</t>
         </is>
       </c>
     </row>
@@ -1373,54 +1397,92 @@
       <c r="A16" s="15" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>Correspondence notes:</t>
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Master Dashboard (MD):</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Written in the italic formula/notes row.</t>
+          <t xml:space="preserve">  • Unfilled = Required − Assignments</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Only when a match is NOT directly above/below in the same Index column.</t>
+          <t xml:space="preserve">  • Required / Assignments = entered or pulled from dispatch (inputs)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Example: (Corresponds with 17 in REC and 13 in MD)</t>
-        </is>
-      </c>
+      <c r="A20" s="15" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • If partners share the same Index column, no correspondence note is needed.</t>
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>Roads Export (REC):</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="inlineStr"/>
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Unfilled Count = max(0, Required Resources − Assignment Count)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>No column name is repeated. Requested Resources and Required Resources are each alone;</t>
+          <t xml:space="preserve">  • Assignment Count = COUNT of confirmed people in Assigned Employees</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>OX Total Staff Requested corresponds with MD Required.</t>
+          <t xml:space="preserve">  • Completed Timesheets = COUNT of completed/approved timesheets on the job</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Total Timesheets = COUNT of all timesheets on the job</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Cancellation Count = COUNT of records in Cancellation Information</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Requested Resources / Required Resources = entered or imported headcount (inputs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • GSF AFAD = list of assigned AFAD devices (OX AFAD Sent counts them)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>Identity fields (Customer/Client, Job Number/Ticket #, etc.) are keys, not calculated.</t>
         </is>
       </c>
     </row>
@@ -1440,8 +1502,8 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1474,306 +1536,306 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="n">
+      <c r="A3" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="C3" s="17" t="inlineStr">
+      <c r="C3" s="18" t="inlineStr">
         <is>
           <t>1 / Client</t>
         </is>
       </c>
-      <c r="D3" s="18" t="inlineStr">
+      <c r="D3" s="19" t="inlineStr">
         <is>
           <t>1 / Customer</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="n">
+      <c r="A4" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>Subcontractor</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>2 / Subcontractor</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr"/>
+      <c r="D4" s="19" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="n">
+      <c r="A5" s="17" t="n">
         <v>14</v>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Job Number</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>4 / Ticket #</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>5 / Job Number</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n">
+      <c r="A6" s="17" t="n">
         <v>27</v>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>WO Number</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr"/>
-      <c r="D6" s="18" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr"/>
+      <c r="D6" s="19" t="inlineStr">
         <is>
           <t>7 / WO Number</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="n">
+      <c r="A7" s="17" t="n">
         <v>13</v>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Dispatching</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>7 / Branch</t>
         </is>
       </c>
-      <c r="D7" s="18" t="inlineStr">
+      <c r="D7" s="19" t="inlineStr">
         <is>
           <t>4 / Dispatching</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n">
+      <c r="A8" s="17" t="n">
         <v>17</v>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>3 / Job Type</t>
         </is>
       </c>
-      <c r="D8" s="18" t="inlineStr">
+      <c r="D8" s="19" t="inlineStr">
         <is>
           <t>13 / Job Type</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="n">
+      <c r="A9" s="17" t="n">
         <v>15</v>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Job Location Name</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>6 / Location</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>6 / Job Location</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="n">
+      <c r="A10" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>Crew Lead</t>
         </is>
       </c>
-      <c r="C10" s="17" t="inlineStr"/>
-      <c r="D10" s="18" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr"/>
+      <c r="D10" s="19" t="inlineStr">
         <is>
           <t>2 / Crew Lead</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="n">
+      <c r="A11" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>Foreman</t>
         </is>
       </c>
-      <c r="C11" s="17" t="inlineStr"/>
-      <c r="D11" s="18" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr"/>
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>3 / Customer Foreman</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="n">
+      <c r="A12" s="17" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>Assignment Date</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr"/>
-      <c r="D12" s="18" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr"/>
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>8 / Date</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="n">
+      <c r="A13" s="17" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>Start Time</t>
         </is>
       </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="C13" s="18" t="inlineStr">
         <is>
           <t>8 / Work Hours</t>
         </is>
       </c>
-      <c r="D13" s="18" t="inlineStr">
+      <c r="D13" s="19" t="inlineStr">
         <is>
           <t>9 / Start</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr"/>
-      <c r="B14" s="16" t="inlineStr"/>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr"/>
+      <c r="B14" s="17" t="inlineStr"/>
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>9 / Total Staff Requested</t>
         </is>
       </c>
-      <c r="D14" s="18" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>10 / Required</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="n">
+      <c r="A15" s="17" t="n">
         <v>18</v>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>Assignment Count</t>
         </is>
       </c>
-      <c r="C15" s="17" t="inlineStr">
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>10 / Total Staff Sent</t>
         </is>
       </c>
-      <c r="D15" s="18" t="inlineStr">
+      <c r="D15" s="19" t="inlineStr">
         <is>
           <t>11 / Assignments</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="n">
+      <c r="A16" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>Unfilled Count</t>
         </is>
       </c>
-      <c r="C16" s="17" t="inlineStr"/>
-      <c r="D16" s="18" t="inlineStr">
+      <c r="C16" s="18" t="inlineStr"/>
+      <c r="D16" s="19" t="inlineStr">
         <is>
           <t>12 / Unfilled</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="n">
+      <c r="A17" s="17" t="n">
         <v>22</v>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>GSF Job</t>
         </is>
       </c>
-      <c r="C17" s="17" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>5 / Ticket Type</t>
         </is>
       </c>
-      <c r="D17" s="18" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>14 / GSF</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="n">
+      <c r="A18" s="17" t="n">
         <v>9</v>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>GSF AFAD</t>
         </is>
       </c>
-      <c r="C18" s="17" t="inlineStr">
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>12 / AFAD Sent</t>
         </is>
       </c>
-      <c r="D18" s="18" t="inlineStr"/>
+      <c r="D18" s="19" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="n">
+      <c r="A19" s="17" t="n">
         <v>21</v>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Timesheets</t>
         </is>
       </c>
-      <c r="C19" s="17" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr">
         <is>
           <t>13 / Notes</t>
         </is>
       </c>
-      <c r="D19" s="18" t="inlineStr"/>
+      <c r="D19" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1781,4 +1843,305 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>How the numbers are calculated</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Formula / rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>OX</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t>Total Saved</t>
+        </is>
+      </c>
+      <c r="C3" s="21" t="inlineStr">
+        <is>
+          <t>max(0, Total Staff Requested − Total Staff Sent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>OX</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>AFAD Sent</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>COUNT of devices listed in REC GSF AFAD for that job</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>OX</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>Total Staff Requested</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>Input (entered or pulled from dispatch)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>OX</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>Total Staff Sent</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>Input (entered or pulled from dispatch)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>Unfilled</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>Required − Assignments</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Input (entered or pulled from dispatch)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>Assignments</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>Input (entered or pulled from dispatch)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>Unfilled Count</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="inlineStr">
+        <is>
+          <t>max(0, Required Resources − Assignment Count)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>Assignment Count</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="inlineStr">
+        <is>
+          <t>COUNT of confirmed people in Assigned Employees</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>Completed Timesheets</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="inlineStr">
+        <is>
+          <t>COUNT of completed/approved timesheets on the job</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>Total Timesheets</t>
+        </is>
+      </c>
+      <c r="C13" s="25" t="inlineStr">
+        <is>
+          <t>COUNT of all timesheets on the job</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>Cancellation Count</t>
+        </is>
+      </c>
+      <c r="C14" s="25" t="inlineStr">
+        <is>
+          <t>COUNT of records in Cancellation Information</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>Requested Resources</t>
+        </is>
+      </c>
+      <c r="C15" s="25" t="inlineStr">
+        <is>
+          <t>Input (entered or imported)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>Required Resources</t>
+        </is>
+      </c>
+      <c r="C16" s="25" t="inlineStr">
+        <is>
+          <t>Input (entered or imported)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>GSF AFAD</t>
+        </is>
+      </c>
+      <c r="C17" s="25" t="inlineStr">
+        <is>
+          <t>List of assigned AFAD devices (counted by OX AFAD Sent)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add GSF Utilization (GU) band with formulas and rollup links
Include GU columns in native order, document Utilization/Integration/
Fulfillment/People Saved formulas, and link office rollups to REC/OX/MD.

Co-authored-by: echenry6f <echenry6f@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Roads_Onyx_Master_Column_Crosswalk.xlsx
+++ b/Roads_Onyx_Master_Column_Crosswalk.xlsx
@@ -8,9 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column Crosswalk" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend &amp; Notes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correspondence Index" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Number Formulas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Number Formulas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend &amp; Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correspondence Index" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,7 +38,7 @@
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="005A6577"/>
-      <sz val="9"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -50,7 +50,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="000D6E6E"/>
-      <sz val="10"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -62,7 +62,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001A2332"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -73,13 +73,8 @@
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -104,6 +99,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E8F0FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5E6F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -133,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -170,18 +170,31 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -547,51 +560,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC9"/>
+  <dimension ref="A1:AC11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
-    <col width="20" customWidth="1" min="25" max="25"/>
-    <col width="20" customWidth="1" min="26" max="26"/>
-    <col width="20" customWidth="1" min="27" max="27"/>
-    <col width="20" customWidth="1" min="28" max="28"/>
-    <col width="20" customWidth="1" min="29" max="29"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="18" customWidth="1" min="27" max="27"/>
+    <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Roads Export ↔ Onyx Report ↔ Master Dashboard (native column order)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="60" customHeight="1">
+          <t>REC ↔ OX ↔ MD ↔ GU (GSF Utilization) — native column order + formulas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="58" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Columns stay in each file’s listed order (REC / OX / MD numbering). Green = Roads Export (REC) · Cream = Onyx (OX) · Blue = Master Dashboard (MD). Italic notes include calculation formulas where numbers are derived, and (Corresponds with …) when a match is not directly above/below. Bold = heading · Italic = formula / notes.</t>
+          <t>REC = Roads Export · OX = Onyx · MD = Master Dashboard · GU = GSF Utilization Report. Columns stay in each file’s listed order. Green=REC · Cream=OX · Blue=MD · Rose=GU. Italic notes = calculation formulas and (Corresponds with …) when not directly above/below.</t>
         </is>
       </c>
     </row>
@@ -686,7 +699,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" ht="48" customHeight="1">
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Roads Export (REC)</t>
@@ -833,7 +846,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="48" customHeight="1">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>(REC formula / notes)</t>
@@ -843,12 +856,12 @@
       <c r="C5" s="7" t="n"/>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Entered / imported requested headcount (often 0 on non-GSF rows in sample)</t>
+          <t>Input (entered/imported requested headcount)</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Entered / imported required headcount for the job</t>
+          <t>Input (entered/imported required headcount)</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -865,7 +878,7 @@
       <c r="I5" s="7" t="n"/>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>List of assigned GSF AFAD devices; OX AFAD Sent = COUNT of those devices · (Corresponds with 12 in OX)</t>
+          <t>List of GSF AFAD devices; OX AFAD Sent / GU In Field Sets roll up from these · (Corresponds with 12 in OX and 8 in GU)</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
@@ -885,12 +898,12 @@
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>(Corresponds with 7 in OX and 4 in MD)</t>
+          <t>(Corresponds with 7 in OX, 4 in MD, and 2 in GU)</t>
         </is>
       </c>
       <c r="O5" s="7" t="inlineStr">
         <is>
-          <t>(Corresponds with 4 in OX and 5 in MD)</t>
+          <t>(Corresponds with 4 in OX, 5 in MD, and 11 in GU)</t>
         </is>
       </c>
       <c r="P5" s="7" t="inlineStr">
@@ -906,12 +919,12 @@
       </c>
       <c r="S5" s="7" t="inlineStr">
         <is>
-          <t>Assignment Count = COUNT of confirmed people in Assigned Employees · (Corresponds with 10 in OX and 11 in MD)</t>
+          <t>Assignment Count = COUNT of confirmed people in Assigned Employees · (Corresponds with 10 in OX, 11 in MD, 7 in GU, and 12 in GU)</t>
         </is>
       </c>
       <c r="T5" s="7" t="inlineStr">
         <is>
-          <t>Completed Timesheets = COUNT of timesheets with completed/approved status</t>
+          <t>Completed Timesheets = COUNT of completed/approved timesheets</t>
         </is>
       </c>
       <c r="U5" s="7" t="inlineStr">
@@ -926,14 +939,14 @@
       </c>
       <c r="W5" s="7" t="inlineStr">
         <is>
-          <t>(Corresponds with 5 in OX and 14 in MD)</t>
+          <t>(Corresponds with 5 in OX, 14 in MD, and 10 in GU)</t>
         </is>
       </c>
       <c r="X5" s="7" t="n"/>
       <c r="Y5" s="7" t="n"/>
       <c r="Z5" s="7" t="inlineStr">
         <is>
-          <t>Cancellation Count = COUNT of cancellation records in Cancellation Information</t>
+          <t>Cancellation Count = COUNT of records in Cancellation Information</t>
         </is>
       </c>
       <c r="AA5" s="7" t="n"/>
@@ -944,7 +957,7 @@
       </c>
       <c r="AC5" s="7" t="n"/>
     </row>
-    <row r="6" ht="48" customHeight="1">
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Onyx (OX)</t>
@@ -1031,7 +1044,7 @@
       <c r="AB6" s="9" t="n"/>
       <c r="AC6" s="9" t="n"/>
     </row>
-    <row r="7" ht="48" customHeight="1">
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>(OX formula / notes)</t>
@@ -1046,12 +1059,12 @@
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>(Corresponds with 14 in REC and 5 in MD)</t>
+          <t>(Corresponds with 14 in REC, 5 in MD, and 11 in GU)</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>(Corresponds with 22 in REC and 14 in MD)</t>
+          <t>(Corresponds with 22 in REC, 14 in MD, and 10 in GU)</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -1061,7 +1074,7 @@
       </c>
       <c r="H7" s="10" t="inlineStr">
         <is>
-          <t>(Corresponds with 13 in REC and 4 in MD)</t>
+          <t>(Corresponds with 13 in REC, 4 in MD, and 2 in GU)</t>
         </is>
       </c>
       <c r="I7" s="10" t="inlineStr">
@@ -1071,12 +1084,12 @@
       </c>
       <c r="J7" s="10" t="inlineStr">
         <is>
-          <t>Entered / imported staff requested (or pulled from dispatch) · (Corresponds with 10 in MD)</t>
+          <t>Input (entered or pulled from dispatch) · (Corresponds with 10 in MD)</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
-          <t>Entered / imported staff sent (or pulled from dispatch) · (Corresponds with 18 in REC and 11 in MD)</t>
+          <t>Input (entered or pulled from dispatch) · (Corresponds with 18 in REC, 11 in MD, 7 in GU, and 12 in GU)</t>
         </is>
       </c>
       <c r="L7" s="10" t="inlineStr">
@@ -1086,7 +1099,7 @@
       </c>
       <c r="M7" s="10" t="inlineStr">
         <is>
-          <t>AFAD Sent = COUNT of GSF AFAD devices on REC GSF AFAD for that job · (Corresponds with 9 in REC)</t>
+          <t>AFAD Sent = COUNT of devices on REC GSF AFAD · (Corresponds with 9 in REC and 8 in GU)</t>
         </is>
       </c>
       <c r="N7" s="10" t="inlineStr">
@@ -1110,7 +1123,7 @@
       <c r="AB7" s="10" t="n"/>
       <c r="AC7" s="10" t="n"/>
     </row>
-    <row r="8" ht="48" customHeight="1">
+    <row r="8" ht="42" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Master Dashboard (MD)</t>
@@ -1201,7 +1214,7 @@
       <c r="AB8" s="12" t="n"/>
       <c r="AC8" s="12" t="n"/>
     </row>
-    <row r="9" ht="48" customHeight="1">
+    <row r="9" ht="42" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>(MD formula / notes)</t>
@@ -1220,12 +1233,12 @@
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>(Corresponds with 13 in REC and 7 in OX)</t>
+          <t>(Corresponds with 13 in REC, 7 in OX, and 2 in GU)</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>(Corresponds with 14 in REC and 4 in OX)</t>
+          <t>(Corresponds with 14 in REC, 4 in OX, and 11 in GU)</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -1250,12 +1263,12 @@
       </c>
       <c r="K9" s="13" t="inlineStr">
         <is>
-          <t>Entered / imported required headcount for the job · (Corresponds with 9 in OX)</t>
+          <t>Input (entered or pulled from dispatch) · (Corresponds with 9 in OX)</t>
         </is>
       </c>
       <c r="L9" s="13" t="inlineStr">
         <is>
-          <t>Entered / imported assigned headcount (filled slots) · (Corresponds with 18 in REC and 10 in OX)</t>
+          <t>Input (entered or pulled from dispatch) · (Corresponds with 18 in REC, 10 in OX, 7 in GU, and 12 in GU)</t>
         </is>
       </c>
       <c r="M9" s="13" t="inlineStr">
@@ -1270,7 +1283,7 @@
       </c>
       <c r="O9" s="13" t="inlineStr">
         <is>
-          <t>(Corresponds with 22 in REC and 5 in OX)</t>
+          <t>(Corresponds with 22 in REC, 5 in OX, and 10 in GU)</t>
         </is>
       </c>
       <c r="P9" s="13" t="n"/>
@@ -1287,6 +1300,180 @@
       <c r="AA9" s="13" t="n"/>
       <c r="AB9" s="13" t="n"/>
       <c r="AC9" s="13" t="n"/>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>GSF Utilization (GU)</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Offices</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>GSF Utilization %</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>GSF infield set/total jobs %</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>GSF Integration (Crews)</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>GSF Fulfillment Crews %</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Flagging Crews</t>
+        </is>
+      </c>
+      <c r="I10" s="15" t="inlineStr">
+        <is>
+          <t>GSF In Field Sets</t>
+        </is>
+      </c>
+      <c r="J10" s="15" t="inlineStr">
+        <is>
+          <t>GSF Sets on Hand (Working Days)</t>
+        </is>
+      </c>
+      <c r="K10" s="15" t="inlineStr">
+        <is>
+          <t>GSF Jobs</t>
+        </is>
+      </c>
+      <c r="L10" s="15" t="inlineStr">
+        <is>
+          <t>Total Jobs</t>
+        </is>
+      </c>
+      <c r="M10" s="15" t="inlineStr">
+        <is>
+          <t>Total Crews</t>
+        </is>
+      </c>
+      <c r="N10" s="15" t="inlineStr">
+        <is>
+          <t>People Saved</t>
+        </is>
+      </c>
+      <c r="O10" s="15" t="n"/>
+      <c r="P10" s="15" t="n"/>
+      <c r="Q10" s="15" t="n"/>
+      <c r="R10" s="15" t="n"/>
+      <c r="S10" s="15" t="n"/>
+      <c r="T10" s="15" t="n"/>
+      <c r="U10" s="15" t="n"/>
+      <c r="V10" s="15" t="n"/>
+      <c r="W10" s="15" t="n"/>
+      <c r="X10" s="15" t="n"/>
+      <c r="Y10" s="15" t="n"/>
+      <c r="Z10" s="15" t="n"/>
+      <c r="AA10" s="15" t="n"/>
+      <c r="AB10" s="15" t="n"/>
+      <c r="AC10" s="15" t="n"/>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>(GU formula / notes)</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Parent company of Offices (DIR, PDB, TTC, WDW, WTC)</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Office name; corresponds to REC/MD Dispatching and OX Branch · (Corresponds with 13 in REC, 7 in OX, and 4 in MD)</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>GSF Utilization % = GSF In Field Sets ÷ GSF Sets on Hand (Working Days)</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>GSF infield set/total jobs % = GSF Jobs ÷ Total Jobs</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>GSF Integration (Crews) % = GSF Sets on Hand ÷ Flagging Crews</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>GSF Fulfillment Crews % = GSF In Field Sets ÷ Flagging Crews</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Rollup ≈ SUM of flagging Assignment Count / Staff Sent / Assignments for the office · (Corresponds with 18 in REC, 10 in OX, and 11 in MD)</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Rollup ≈ SUM of AFAD Sent / COUNT of REC GSF AFAD devices for the office · (Corresponds with 13 in GU)</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Inventory input: sets available (working days)</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Rollup = COUNT of jobs where GSF Job/Ticket Type/GSF = Yes · (Corresponds with 22 in REC, 5 in OX, and 14 in MD)</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Rollup = COUNT of all jobs (Job Number / Ticket #) for the office · (Corresponds with 14 in REC, 4 in OX, and 5 in MD)</t>
+        </is>
+      </c>
+      <c r="M11" s="16" t="inlineStr">
+        <is>
+          <t>Rollup ≈ SUM of Staff Sent / Assignments / Assignment Count for the office · (Corresponds with 18 in REC, 10 in OX, and 11 in MD)</t>
+        </is>
+      </c>
+      <c r="N11" s="16" t="inlineStr">
+        <is>
+          <t>People Saved = GSF In Field Sets · (Corresponds with 8 in GU)</t>
+        </is>
+      </c>
+      <c r="O11" s="16" t="n"/>
+      <c r="P11" s="16" t="n"/>
+      <c r="Q11" s="16" t="n"/>
+      <c r="R11" s="16" t="n"/>
+      <c r="S11" s="16" t="n"/>
+      <c r="T11" s="16" t="n"/>
+      <c r="U11" s="16" t="n"/>
+      <c r="V11" s="16" t="n"/>
+      <c r="W11" s="16" t="n"/>
+      <c r="X11" s="16" t="n"/>
+      <c r="Y11" s="16" t="n"/>
+      <c r="Z11" s="16" t="n"/>
+      <c r="AA11" s="16" t="n"/>
+      <c r="AB11" s="16" t="n"/>
+      <c r="AC11" s="16" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1303,190 +1490,297 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="78" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
-        <is>
-          <t>How to read this sheet + number formulas</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>How the numbers are calculated (including GSF Utilization)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="inlineStr"/>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Formula / rule</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>Abbreviations: REC = Roads Export · OX = Onyx · MD = Master Dashboard</t>
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>GU</t>
+        </is>
+      </c>
+      <c r="B3" s="18" t="inlineStr">
+        <is>
+          <t>GSF Utilization %</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="inlineStr">
+        <is>
+          <t>GSF In Field Sets ÷ GSF Sets on Hand (Working Days)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr"/>
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>GU</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>GSF infield set/total jobs %</t>
+        </is>
+      </c>
+      <c r="C4" s="19" t="inlineStr">
+        <is>
+          <t>GSF Jobs ÷ Total Jobs</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>Colors: Green = REC · Cream = OX · Blue = MD (including blank cells in that row).</t>
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>GU</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>GSF Integration (Crews) %</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>GSF Sets on Hand ÷ Flagging Crews</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr"/>
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>GU</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>GSF Fulfillment Crews %</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>GSF In Field Sets ÷ Flagging Crews</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>Correspondence notes appear only when a match is NOT directly above/below, e.g.</t>
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>GU</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>People Saved</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>People Saved = GSF In Field Sets</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  (Corresponds with 17 in REC and 13 in MD)</t>
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>GU</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Company Totals (G–M)</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>SUM of office rows; then recompute % from summed totals (not average of %)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr"/>
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>GU</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Beaver Falls check</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>122÷440≈28% Utilization; 67÷1079≈6% job mix; 440÷401.5≈109.6% Integration; 122÷401.5≈30% Fulfillment</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="16">
-        <f>========= NUMBER FORMULAS ==========</f>
-        <v/>
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>OX</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>Total Saved</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>max(0, Total Staff Requested − Total Staff Sent)</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr"/>
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>OX</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>AFAD Sent</t>
+        </is>
+      </c>
+      <c r="C11" s="22" t="inlineStr">
+        <is>
+          <t>COUNT of devices listed in REC GSF AFAD</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>Onyx (OX):</t>
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>Unfilled</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="inlineStr">
+        <is>
+          <t>Required − Assignments</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Total Saved = max(0, Total Staff Requested − Total Staff Sent)</t>
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>Unfilled Count</t>
+        </is>
+      </c>
+      <c r="C13" s="28" t="inlineStr">
+        <is>
+          <t>max(0, Required Resources − Assignment Count)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • AFAD Sent = COUNT of GSF AFAD devices listed on REC GSF AFAD for that job</t>
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="B14" s="27" t="inlineStr">
+        <is>
+          <t>Assignment Count</t>
+        </is>
+      </c>
+      <c r="C14" s="28" t="inlineStr">
+        <is>
+          <t>COUNT of confirmed people in Assigned Employees</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Total Staff Requested / Total Staff Sent = entered or pulled from dispatch (inputs)</t>
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="inlineStr">
+        <is>
+          <t>Completed Timesheets</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="inlineStr">
+        <is>
+          <t>COUNT of completed/approved timesheets</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr"/>
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="B16" s="27" t="inlineStr">
+        <is>
+          <t>Total Timesheets</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="inlineStr">
+        <is>
+          <t>COUNT of all timesheets on the job</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>Master Dashboard (MD):</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Unfilled = Required − Assignments</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Required / Assignments = entered or pulled from dispatch (inputs)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="15" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>Roads Export (REC):</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Unfilled Count = max(0, Required Resources − Assignment Count)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Assignment Count = COUNT of confirmed people in Assigned Employees</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Completed Timesheets = COUNT of completed/approved timesheets on the job</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Total Timesheets = COUNT of all timesheets on the job</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Cancellation Count = COUNT of records in Cancellation Information</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Requested Resources / Required Resources = entered or imported headcount (inputs)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • GSF AFAD = list of assigned AFAD devices (OX AFAD Sent counts them)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="15" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>Identity fields (Customer/Client, Job Number/Ticket #, etc.) are keys, not calculated.</t>
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="B17" s="27" t="inlineStr">
+        <is>
+          <t>Cancellation Count</t>
+        </is>
+      </c>
+      <c r="C17" s="28" t="inlineStr">
+        <is>
+          <t>COUNT of records in Cancellation Information</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1497,350 +1791,67 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>All cross-system correspondences</t>
+      <c r="A1" s="29" t="inlineStr">
+        <is>
+          <t>Legend</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>REC #</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>REC column</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>OX # / column</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>MD # / column</t>
-        </is>
-      </c>
+      <c r="A2" s="30" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="17" t="inlineStr">
-        <is>
-          <t>Customer</t>
-        </is>
-      </c>
-      <c r="C3" s="18" t="inlineStr">
-        <is>
-          <t>1 / Client</t>
-        </is>
-      </c>
-      <c r="D3" s="19" t="inlineStr">
-        <is>
-          <t>1 / Customer</t>
+      <c r="A3" s="30" t="inlineStr">
+        <is>
+          <t>Abbreviations: REC = Roads Export · OX = Onyx · MD = Master Dashboard · GU = GSF Utilization Report</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="17" t="inlineStr">
-        <is>
-          <t>Subcontractor</t>
-        </is>
-      </c>
-      <c r="C4" s="18" t="inlineStr">
-        <is>
-          <t>2 / Subcontractor</t>
-        </is>
-      </c>
-      <c r="D4" s="19" t="inlineStr"/>
+      <c r="A4" s="30" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="n">
-        <v>14</v>
-      </c>
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>Job Number</t>
-        </is>
-      </c>
-      <c r="C5" s="18" t="inlineStr">
-        <is>
-          <t>4 / Ticket #</t>
-        </is>
-      </c>
-      <c r="D5" s="19" t="inlineStr">
-        <is>
-          <t>5 / Job Number</t>
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Colors: Green=REC · Cream=OX · Blue=MD · Rose=GU</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="n">
-        <v>27</v>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>WO Number</t>
-        </is>
-      </c>
-      <c r="C6" s="18" t="inlineStr"/>
-      <c r="D6" s="19" t="inlineStr">
-        <is>
-          <t>7 / WO Number</t>
-        </is>
-      </c>
+      <c r="A6" s="30" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="n">
-        <v>13</v>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>Dispatching</t>
-        </is>
-      </c>
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>7 / Branch</t>
-        </is>
-      </c>
-      <c r="D7" s="19" t="inlineStr">
-        <is>
-          <t>4 / Dispatching</t>
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>GU is an office-level rollup. Job-level REC/OX/MD rows feed GU when summed/counted by office (e.g. Beaver Falls).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="n">
-        <v>17</v>
-      </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>Job Type</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>3 / Job Type</t>
-        </is>
-      </c>
-      <c r="D8" s="19" t="inlineStr">
-        <is>
-          <t>13 / Job Type</t>
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>Example from GU PDF — WDW Beaver Falls: Sets 122, On Hand 440 → Utilization 28%; GSF Jobs 67 / Total Jobs 1079 → 6%.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="n">
-        <v>15</v>
-      </c>
-      <c r="B9" s="17" t="inlineStr">
-        <is>
-          <t>Job Location Name</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>6 / Location</t>
-        </is>
-      </c>
-      <c r="D9" s="19" t="inlineStr">
-        <is>
-          <t>6 / Job Location</t>
-        </is>
-      </c>
+      <c r="A9" s="30" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="17" t="inlineStr">
-        <is>
-          <t>Crew Lead</t>
-        </is>
-      </c>
-      <c r="C10" s="18" t="inlineStr"/>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>2 / Crew Lead</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="17" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="17" t="inlineStr">
-        <is>
-          <t>Foreman</t>
-        </is>
-      </c>
-      <c r="C11" s="18" t="inlineStr"/>
-      <c r="D11" s="19" t="inlineStr">
-        <is>
-          <t>3 / Customer Foreman</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="17" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>Assignment Date</t>
-        </is>
-      </c>
-      <c r="C12" s="18" t="inlineStr"/>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>8 / Date</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="17" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>Start Time</t>
-        </is>
-      </c>
-      <c r="C13" s="18" t="inlineStr">
-        <is>
-          <t>8 / Work Hours</t>
-        </is>
-      </c>
-      <c r="D13" s="19" t="inlineStr">
-        <is>
-          <t>9 / Start</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="17" t="inlineStr"/>
-      <c r="B14" s="17" t="inlineStr"/>
-      <c r="C14" s="18" t="inlineStr">
-        <is>
-          <t>9 / Total Staff Requested</t>
-        </is>
-      </c>
-      <c r="D14" s="19" t="inlineStr">
-        <is>
-          <t>10 / Required</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="17" t="n">
-        <v>18</v>
-      </c>
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>Assignment Count</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>10 / Total Staff Sent</t>
-        </is>
-      </c>
-      <c r="D15" s="19" t="inlineStr">
-        <is>
-          <t>11 / Assignments</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="17" t="n">
-        <v>5</v>
-      </c>
-      <c r="B16" s="17" t="inlineStr">
-        <is>
-          <t>Unfilled Count</t>
-        </is>
-      </c>
-      <c r="C16" s="18" t="inlineStr"/>
-      <c r="D16" s="19" t="inlineStr">
-        <is>
-          <t>12 / Unfilled</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="17" t="n">
-        <v>22</v>
-      </c>
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>GSF Job</t>
-        </is>
-      </c>
-      <c r="C17" s="18" t="inlineStr">
-        <is>
-          <t>5 / Ticket Type</t>
-        </is>
-      </c>
-      <c r="D17" s="19" t="inlineStr">
-        <is>
-          <t>14 / GSF</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="17" t="n">
-        <v>9</v>
-      </c>
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>GSF AFAD</t>
-        </is>
-      </c>
-      <c r="C18" s="18" t="inlineStr">
-        <is>
-          <t>12 / AFAD Sent</t>
-        </is>
-      </c>
-      <c r="D18" s="19" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="17" t="n">
-        <v>21</v>
-      </c>
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>Timesheets</t>
-        </is>
-      </c>
-      <c r="C19" s="18" t="inlineStr">
-        <is>
-          <t>13 / Notes</t>
-        </is>
-      </c>
-      <c r="D19" s="19" t="inlineStr"/>
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>See Number Formulas sheet for full calculation list.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1851,296 +1862,422 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>How the numbers are calculated</t>
+          <t>Cross-system correspondences (job-level + GU rollups)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>REC #</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Column</t>
+          <t>OX #</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Formula / rule</t>
+          <t>MD #</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>GU #</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
-        <is>
-          <t>OX</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="inlineStr">
-        <is>
-          <t>Total Saved</t>
-        </is>
-      </c>
-      <c r="C3" s="21" t="inlineStr">
-        <is>
-          <t>max(0, Total Staff Requested − Total Staff Sent)</t>
+      <c r="A3" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="17" t="inlineStr"/>
+      <c r="E3" s="31" t="inlineStr">
+        <is>
+          <t>Customer ↔ Client ↔ Customer</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
-        <is>
-          <t>OX</t>
-        </is>
-      </c>
-      <c r="B4" s="20" t="inlineStr">
-        <is>
-          <t>AFAD Sent</t>
-        </is>
-      </c>
-      <c r="C4" s="21" t="inlineStr">
-        <is>
-          <t>COUNT of devices listed in REC GSF AFAD for that job</t>
+      <c r="A4" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="23" t="inlineStr"/>
+      <c r="D4" s="17" t="inlineStr"/>
+      <c r="E4" s="31" t="inlineStr">
+        <is>
+          <t>Subcontractor ↔ Subcontractor</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>OX</t>
-        </is>
-      </c>
-      <c r="B5" s="20" t="inlineStr">
-        <is>
-          <t>Total Staff Requested</t>
-        </is>
-      </c>
-      <c r="C5" s="21" t="inlineStr">
-        <is>
-          <t>Input (entered or pulled from dispatch)</t>
+      <c r="A5" s="26" t="n">
+        <v>14</v>
+      </c>
+      <c r="B5" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" s="17" t="inlineStr"/>
+      <c r="E5" s="31" t="inlineStr">
+        <is>
+          <t>Job Number ↔ Ticket # ↔ Job Number</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>OX</t>
-        </is>
-      </c>
-      <c r="B6" s="20" t="inlineStr">
-        <is>
-          <t>Total Staff Sent</t>
-        </is>
-      </c>
-      <c r="C6" s="21" t="inlineStr">
-        <is>
-          <t>Input (entered or pulled from dispatch)</t>
+      <c r="A6" s="26" t="n">
+        <v>27</v>
+      </c>
+      <c r="B6" s="20" t="inlineStr"/>
+      <c r="C6" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="D6" s="17" t="inlineStr"/>
+      <c r="E6" s="31" t="inlineStr">
+        <is>
+          <t>WO Number ↔ WO Number</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="B7" s="22" t="inlineStr">
-        <is>
-          <t>Unfilled</t>
-        </is>
-      </c>
-      <c r="C7" s="23" t="inlineStr">
-        <is>
-          <t>Required − Assignments</t>
+      <c r="A7" s="26" t="n">
+        <v>13</v>
+      </c>
+      <c r="B7" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="17" t="inlineStr"/>
+      <c r="E7" s="31" t="inlineStr">
+        <is>
+          <t>Dispatching ↔ Branch ↔ Dispatching</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="B8" s="22" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C8" s="23" t="inlineStr">
-        <is>
-          <t>Input (entered or pulled from dispatch)</t>
+      <c r="A8" s="26" t="n">
+        <v>17</v>
+      </c>
+      <c r="B8" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>13</v>
+      </c>
+      <c r="D8" s="17" t="inlineStr"/>
+      <c r="E8" s="31" t="inlineStr">
+        <is>
+          <t>Job Type ↔ Job Type ↔ Job Type</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="B9" s="22" t="inlineStr">
-        <is>
-          <t>Assignments</t>
-        </is>
-      </c>
-      <c r="C9" s="23" t="inlineStr">
-        <is>
-          <t>Input (entered or pulled from dispatch)</t>
+      <c r="A9" s="26" t="n">
+        <v>15</v>
+      </c>
+      <c r="B9" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="D9" s="17" t="inlineStr"/>
+      <c r="E9" s="31" t="inlineStr">
+        <is>
+          <t>Job Location Name ↔ Location ↔ Job Location</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="B10" s="24" t="inlineStr">
-        <is>
-          <t>Unfilled Count</t>
-        </is>
-      </c>
-      <c r="C10" s="25" t="inlineStr">
-        <is>
-          <t>max(0, Required Resources − Assignment Count)</t>
+      <c r="A10" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="20" t="inlineStr"/>
+      <c r="C10" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="17" t="inlineStr"/>
+      <c r="E10" s="31" t="inlineStr">
+        <is>
+          <t>Crew Lead ↔ Crew Lead</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="B11" s="24" t="inlineStr">
-        <is>
-          <t>Assignment Count</t>
-        </is>
-      </c>
-      <c r="C11" s="25" t="inlineStr">
-        <is>
-          <t>COUNT of confirmed people in Assigned Employees</t>
+      <c r="A11" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="20" t="inlineStr"/>
+      <c r="C11" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="17" t="inlineStr"/>
+      <c r="E11" s="31" t="inlineStr">
+        <is>
+          <t>Foreman ↔ Customer Foreman</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="B12" s="24" t="inlineStr">
-        <is>
-          <t>Completed Timesheets</t>
-        </is>
-      </c>
-      <c r="C12" s="25" t="inlineStr">
-        <is>
-          <t>COUNT of completed/approved timesheets on the job</t>
+      <c r="A12" s="26" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="20" t="inlineStr"/>
+      <c r="C12" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D12" s="17" t="inlineStr"/>
+      <c r="E12" s="31" t="inlineStr">
+        <is>
+          <t>Assignment Date ↔ Date</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="B13" s="24" t="inlineStr">
-        <is>
-          <t>Total Timesheets</t>
-        </is>
-      </c>
-      <c r="C13" s="25" t="inlineStr">
-        <is>
-          <t>COUNT of all timesheets on the job</t>
+      <c r="A13" s="26" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="D13" s="17" t="inlineStr"/>
+      <c r="E13" s="31" t="inlineStr">
+        <is>
+          <t>Start Time ↔ Work Hours ↔ Start</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="B14" s="24" t="inlineStr">
-        <is>
-          <t>Cancellation Count</t>
-        </is>
-      </c>
-      <c r="C14" s="25" t="inlineStr">
-        <is>
-          <t>COUNT of records in Cancellation Information</t>
+      <c r="A14" s="26" t="inlineStr"/>
+      <c r="B14" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" s="17" t="inlineStr"/>
+      <c r="E14" s="31" t="inlineStr">
+        <is>
+          <t>Total Staff Requested ↔ Required</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="B15" s="24" t="inlineStr">
-        <is>
-          <t>Requested Resources</t>
-        </is>
-      </c>
-      <c r="C15" s="25" t="inlineStr">
-        <is>
-          <t>Input (entered or imported)</t>
+      <c r="A15" s="26" t="n">
+        <v>18</v>
+      </c>
+      <c r="B15" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>11</v>
+      </c>
+      <c r="D15" s="17" t="inlineStr"/>
+      <c r="E15" s="31" t="inlineStr">
+        <is>
+          <t>Assignment Count ↔ Total Staff Sent ↔ Assignments</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="B16" s="24" t="inlineStr">
-        <is>
-          <t>Required Resources</t>
-        </is>
-      </c>
-      <c r="C16" s="25" t="inlineStr">
-        <is>
-          <t>Input (entered or imported)</t>
+      <c r="A16" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" s="20" t="inlineStr"/>
+      <c r="C16" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="D16" s="17" t="inlineStr"/>
+      <c r="E16" s="31" t="inlineStr">
+        <is>
+          <t>Unfilled Count ↔ Unfilled</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="B17" s="24" t="inlineStr">
-        <is>
-          <t>GSF AFAD</t>
-        </is>
-      </c>
-      <c r="C17" s="25" t="inlineStr">
-        <is>
-          <t>List of assigned AFAD devices (counted by OX AFAD Sent)</t>
+      <c r="A17" s="26" t="n">
+        <v>22</v>
+      </c>
+      <c r="B17" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" s="23" t="n">
+        <v>14</v>
+      </c>
+      <c r="D17" s="17" t="inlineStr"/>
+      <c r="E17" s="31" t="inlineStr">
+        <is>
+          <t>GSF Job ↔ Ticket Type ↔ GSF</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="26" t="n">
+        <v>9</v>
+      </c>
+      <c r="B18" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="C18" s="23" t="inlineStr"/>
+      <c r="D18" s="17" t="inlineStr"/>
+      <c r="E18" s="31" t="inlineStr">
+        <is>
+          <t>GSF AFAD ↔ AFAD Sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="26" t="n">
+        <v>21</v>
+      </c>
+      <c r="B19" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="C19" s="23" t="inlineStr"/>
+      <c r="D19" s="17" t="inlineStr"/>
+      <c r="E19" s="31" t="inlineStr">
+        <is>
+          <t>Timesheets ↔ Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="32" t="inlineStr">
+        <is>
+          <t>GU rollup links</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="31" t="n"/>
+      <c r="B22" s="31" t="n"/>
+      <c r="C22" s="31" t="n"/>
+      <c r="D22" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="31" t="inlineStr">
+        <is>
+          <t>GU 2 Offices ↔ REC 13, OX 7, MD 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="31" t="n"/>
+      <c r="B23" s="31" t="n"/>
+      <c r="C23" s="31" t="n"/>
+      <c r="D23" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="E23" s="31" t="inlineStr">
+        <is>
+          <t>GU 7 Flagging Crews ↔ REC 18, OX 10, MD 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="31" t="n"/>
+      <c r="B24" s="31" t="n"/>
+      <c r="C24" s="31" t="n"/>
+      <c r="D24" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E24" s="31" t="inlineStr">
+        <is>
+          <t>GU 8 GSF In Field Sets ↔ REC 9, OX 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="31" t="n"/>
+      <c r="B25" s="31" t="n"/>
+      <c r="C25" s="31" t="n"/>
+      <c r="D25" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="E25" s="31" t="inlineStr">
+        <is>
+          <t>GU 10 GSF Jobs ↔ REC 22, OX 5, MD 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="31" t="n"/>
+      <c r="B26" s="31" t="n"/>
+      <c r="C26" s="31" t="n"/>
+      <c r="D26" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="E26" s="31" t="inlineStr">
+        <is>
+          <t>GU 11 Total Jobs ↔ REC 14, OX 4, MD 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="31" t="n"/>
+      <c r="B27" s="31" t="n"/>
+      <c r="C27" s="31" t="n"/>
+      <c r="D27" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="E27" s="31" t="inlineStr">
+        <is>
+          <t>GU 12 Total Crews ↔ REC 18, OX 10, MD 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="31" t="n"/>
+      <c r="B28" s="31" t="n"/>
+      <c r="C28" s="31" t="n"/>
+      <c r="D28" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="E28" s="31" t="inlineStr">
+        <is>
+          <t>GU 13 People Saved = GU 8 GSF In Field Sets</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Document GU multi-day grain vs single-day REC/OX/MD sources
Clarify that GSF Utilization percentages are calculated from the same
source fields as Roads/Onyx/Master, but rolled across numerous days by
office — not from a single-day export snapshot.

Co-authored-by: echenry6f <echenry6f@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Roads_Onyx_Master_Column_Crosswalk.xlsx
+++ b/Roads_Onyx_Master_Column_Crosswalk.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,8 +73,30 @@
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -106,8 +128,28 @@
         <fgColor rgb="00F5E6F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6DCE4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -129,11 +171,25 @@
         <color rgb="00D0D7E2"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -195,6 +251,54 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -601,10 +705,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="58" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>REC = Roads Export · OX = Onyx · MD = Master Dashboard · GU = GSF Utilization Report. Columns stay in each file’s listed order. Green=REC · Cream=OX · Blue=MD · Rose=GU. Italic notes = calculation formulas and (Corresponds with …) when not directly above/below.</t>
+    <row r="2" ht="52" customHeight="1">
+      <c r="A2" s="33" t="inlineStr">
+        <is>
+          <t>REC = Roads Export · OX = Onyx · MD = Master Dashboard · GU = GSF Utilization Report. Columns stay in each file’s listed order. Green=REC · Cream=OX · Blue=MD · Rose=GU. Italic notes = calculation formulas and (Corresponds with …) when not directly above/below. TIME GRAIN: REC/OX/MD views compared are SINGLE-day job lists; GU percentages are generated from those same source fields rolled across NUMEROUS days by office.</t>
         </is>
       </c>
     </row>
@@ -1404,59 +1508,59 @@
           <t>Office name; corresponds to REC/MD Dispatching and OX Branch · (Corresponds with 13 in REC, 7 in OX, and 4 in MD)</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>GSF Utilization % = GSF In Field Sets ÷ GSF Sets on Hand (Working Days)</t>
-        </is>
-      </c>
-      <c r="E11" s="16" t="inlineStr">
-        <is>
-          <t>GSF infield set/total jobs % = GSF Jobs ÷ Total Jobs</t>
-        </is>
-      </c>
-      <c r="F11" s="16" t="inlineStr">
-        <is>
-          <t>GSF Integration (Crews) % = GSF Sets on Hand ÷ Flagging Crews</t>
-        </is>
-      </c>
-      <c r="G11" s="16" t="inlineStr">
-        <is>
-          <t>GSF Fulfillment Crews % = GSF In Field Sets ÷ Flagging Crews</t>
-        </is>
-      </c>
-      <c r="H11" s="16" t="inlineStr">
-        <is>
-          <t>Rollup ≈ SUM of flagging Assignment Count / Staff Sent / Assignments for the office · (Corresponds with 18 in REC, 10 in OX, and 11 in MD)</t>
-        </is>
-      </c>
-      <c r="I11" s="16" t="inlineStr">
-        <is>
-          <t>Rollup ≈ SUM of AFAD Sent / COUNT of REC GSF AFAD devices for the office · (Corresponds with 13 in GU)</t>
-        </is>
-      </c>
-      <c r="J11" s="16" t="inlineStr">
-        <is>
-          <t>Inventory input: sets available (working days)</t>
-        </is>
-      </c>
-      <c r="K11" s="16" t="inlineStr">
-        <is>
-          <t>Rollup = COUNT of jobs where GSF Job/Ticket Type/GSF = Yes · (Corresponds with 22 in REC, 5 in OX, and 14 in MD)</t>
-        </is>
-      </c>
-      <c r="L11" s="16" t="inlineStr">
-        <is>
-          <t>Rollup = COUNT of all jobs (Job Number / Ticket #) for the office · (Corresponds with 14 in REC, 4 in OX, and 5 in MD)</t>
-        </is>
-      </c>
-      <c r="M11" s="16" t="inlineStr">
-        <is>
-          <t>Rollup ≈ SUM of Staff Sent / Assignments / Assignment Count for the office · (Corresponds with 18 in REC, 10 in OX, and 11 in MD)</t>
-        </is>
-      </c>
-      <c r="N11" s="16" t="inlineStr">
-        <is>
-          <t>People Saved = GSF In Field Sets · (Corresponds with 8 in GU)</t>
+      <c r="D11" s="34" t="inlineStr">
+        <is>
+          <t>GSF Utilization % = GSF In Field Sets ÷ GSF Sets on Hand — generated from multi-day rolled source counts (not a single-day export)</t>
+        </is>
+      </c>
+      <c r="E11" s="34" t="inlineStr">
+        <is>
+          <t>GSF infield set/total jobs % = GSF Jobs ÷ Total Jobs — generated from multi-day rolled source counts</t>
+        </is>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>GSF Integration (Crews) % = GSF Sets on Hand ÷ Flagging Crews — generated from multi-day rolled source counts</t>
+        </is>
+      </c>
+      <c r="G11" s="34" t="inlineStr">
+        <is>
+          <t>GSF Fulfillment Crews % = GSF In Field Sets ÷ Flagging Crews — generated from multi-day rolled source counts</t>
+        </is>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>Multi-day rollup ≈ SUM of flagging Assignment Count / Staff Sent / Assignments for the office · (Corresponds with 18 in REC, 10 in OX, and 11 in MD)</t>
+        </is>
+      </c>
+      <c r="I11" s="34" t="inlineStr">
+        <is>
+          <t>Multi-day rollup ≈ SUM of AFAD Sent / COUNT of REC GSF AFAD devices for the office · (Corresponds with 13 in GU)</t>
+        </is>
+      </c>
+      <c r="J11" s="34" t="inlineStr">
+        <is>
+          <t>Inventory input over the period: sets available (working days) — multi-day, not from a single job row</t>
+        </is>
+      </c>
+      <c r="K11" s="34" t="inlineStr">
+        <is>
+          <t>Multi-day rollup = COUNT of jobs where GSF Job/Ticket Type/GSF = Yes · (Corresponds with 22 in REC, 5 in OX, and 14 in MD)</t>
+        </is>
+      </c>
+      <c r="L11" s="34" t="inlineStr">
+        <is>
+          <t>Multi-day rollup = COUNT of all jobs (Job Number / Ticket #) for the office · (Corresponds with 14 in REC, 4 in OX, and 5 in MD)</t>
+        </is>
+      </c>
+      <c r="M11" s="34" t="inlineStr">
+        <is>
+          <t>Multi-day rollup ≈ SUM of Staff Sent / Assignments / Assignment Count for the office · (Corresponds with 18 in REC, 10 in OX, and 11 in MD)</t>
+        </is>
+      </c>
+      <c r="N11" s="34" t="inlineStr">
+        <is>
+          <t>People Saved = GSF In Field Sets (same multi-day rollup) · (Corresponds with 8 in GU)</t>
         </is>
       </c>
       <c r="O11" s="16" t="n"/>
@@ -1490,288 +1594,516 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="78" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>How the numbers are calculated (including GSF Utilization)</t>
-        </is>
-      </c>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="35" t="inlineStr">
+        <is>
+          <t>How GSF Utilization % are built from REC / OX / MD sources</t>
+        </is>
+      </c>
+      <c r="B1" s="36" t="n"/>
+      <c r="C1" s="36" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="36" t="n"/>
+      <c r="B2" s="36" t="n"/>
+      <c r="C2" s="36" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>TIME GRAIN (important)</t>
+        </is>
+      </c>
+      <c r="B3" s="36" t="n"/>
+      <c r="C3" s="36" t="n"/>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="37" t="inlineStr">
+        <is>
+          <t>REC / OX / MD</t>
+        </is>
+      </c>
+      <c r="B4" s="38" t="inlineStr">
+        <is>
+          <t>Job-level views compared earlier</t>
+        </is>
+      </c>
+      <c r="C4" s="38" t="inlineStr">
+        <is>
+          <t>Each export/screenshot shows ONE day (or one day’s jobs). Same job keys (Job Number / Ticket #) line up across those three for that day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="39" t="inlineStr">
+        <is>
+          <t>GU (this document)</t>
+        </is>
+      </c>
+      <c r="B5" s="40" t="inlineStr">
+        <is>
+          <t>Office-level rollup</t>
+        </is>
+      </c>
+      <c r="C5" s="40" t="inlineStr">
+        <is>
+          <t>GSF Utilization aggregates the SAME kinds of source fields across NUMEROUS days (period totals), then computes percentages from those period sums — not from a single-day snapshot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="36" t="n"/>
+      <c r="B6" s="36" t="n"/>
+      <c r="C6" s="36" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>SOURCE → GU INPUT COLUMNS (what gets summed / counted over the period)</t>
+        </is>
+      </c>
+      <c r="B7" s="36" t="n"/>
+      <c r="C7" s="36" t="n"/>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="41" t="inlineStr">
         <is>
           <t>System</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B8" s="41" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C8" s="41" t="inlineStr">
         <is>
           <t>Formula / rule</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="39" t="inlineStr">
         <is>
           <t>GU</t>
         </is>
       </c>
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B9" s="36" t="inlineStr">
+        <is>
+          <t>Flagging Crews (col 7)</t>
+        </is>
+      </c>
+      <c r="C9" s="42" t="inlineStr">
+        <is>
+          <t>Period SUM of flagging staff from sources: REC Assignment Count · OX Total Staff Sent · MD Assignments (by office)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="39" t="inlineStr">
+        <is>
+          <t>GU</t>
+        </is>
+      </c>
+      <c r="B10" s="36" t="inlineStr">
+        <is>
+          <t>GSF In Field Sets (col 8)</t>
+        </is>
+      </c>
+      <c r="C10" s="42" t="inlineStr">
+        <is>
+          <t>Period SUM/COUNT of GSF AFAD devices: REC GSF AFAD · OX AFAD Sent (by office)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="39" t="inlineStr">
+        <is>
+          <t>GU</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="inlineStr">
+        <is>
+          <t>GSF Sets on Hand (col 9)</t>
+        </is>
+      </c>
+      <c r="C11" s="42" t="inlineStr">
+        <is>
+          <t>Inventory input over the period: sets available (working days) — not taken from a single job row</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="39" t="inlineStr">
+        <is>
+          <t>GU</t>
+        </is>
+      </c>
+      <c r="B12" s="36" t="inlineStr">
+        <is>
+          <t>GSF Jobs (col 10)</t>
+        </is>
+      </c>
+      <c r="C12" s="42" t="inlineStr">
+        <is>
+          <t>Period COUNT of jobs flagged GSF: REC GSF Job · OX Ticket Type · MD GSF (by office)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="39" t="inlineStr">
+        <is>
+          <t>GU</t>
+        </is>
+      </c>
+      <c r="B13" s="36" t="inlineStr">
+        <is>
+          <t>Total Jobs (col 11)</t>
+        </is>
+      </c>
+      <c r="C13" s="42" t="inlineStr">
+        <is>
+          <t>Period COUNT of all jobs: REC Job Number · OX Ticket # · MD Job Number (by office)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="39" t="inlineStr">
+        <is>
+          <t>GU</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="inlineStr">
+        <is>
+          <t>Total Crews (col 12)</t>
+        </is>
+      </c>
+      <c r="C14" s="42" t="inlineStr">
+        <is>
+          <t>Period SUM of crew counts ≈ same source fields as Flagging Crews (REC 18 / OX 10 / MD 11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="36" t="n"/>
+      <c r="B15" s="36" t="n"/>
+      <c r="C15" s="36" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>PERCENTAGES GENERATED FROM THOSE ROLLED COLUMNS</t>
+        </is>
+      </c>
+      <c r="B16" s="36" t="n"/>
+      <c r="C16" s="36" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="41" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="B17" s="41" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="C17" s="41" t="inlineStr">
+        <is>
+          <t>Formula / rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="39" t="inlineStr">
+        <is>
+          <t>GU</t>
+        </is>
+      </c>
+      <c r="B18" s="36" t="inlineStr">
         <is>
           <t>GSF Utilization %</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
-        <is>
-          <t>GSF In Field Sets ÷ GSF Sets on Hand (Working Days)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="C18" s="42" t="inlineStr">
+        <is>
+          <t>GSF In Field Sets ÷ GSF Sets on Hand (Working Days)   [period H ÷ period I]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="39" t="inlineStr">
         <is>
           <t>GU</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B19" s="36" t="inlineStr">
         <is>
           <t>GSF infield set/total jobs %</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
-        <is>
-          <t>GSF Jobs ÷ Total Jobs</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="C19" s="42" t="inlineStr">
+        <is>
+          <t>GSF Jobs ÷ Total Jobs   [period J ÷ period K]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="39" t="inlineStr">
         <is>
           <t>GU</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B20" s="36" t="inlineStr">
         <is>
           <t>GSF Integration (Crews) %</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
-        <is>
-          <t>GSF Sets on Hand ÷ Flagging Crews</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="C20" s="42" t="inlineStr">
+        <is>
+          <t>GSF Sets on Hand ÷ Flagging Crews   [period I ÷ period G]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="39" t="inlineStr">
         <is>
           <t>GU</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B21" s="36" t="inlineStr">
         <is>
           <t>GSF Fulfillment Crews %</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>GSF In Field Sets ÷ Flagging Crews</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="C21" s="42" t="inlineStr">
+        <is>
+          <t>GSF In Field Sets ÷ Flagging Crews   [period H ÷ period G]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>GU</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B22" s="36" t="inlineStr">
         <is>
           <t>People Saved</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
-        <is>
-          <t>People Saved = GSF In Field Sets</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="C22" s="42" t="inlineStr">
+        <is>
+          <t>People Saved = GSF In Field Sets   [period M = period H]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="39" t="inlineStr">
         <is>
           <t>GU</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Company Totals (G–M)</t>
-        </is>
-      </c>
-      <c r="C8" s="19" t="inlineStr">
-        <is>
-          <t>SUM of office rows; then recompute % from summed totals (not average of %)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="B23" s="36" t="inlineStr">
+        <is>
+          <t>Company / Grand Totals</t>
+        </is>
+      </c>
+      <c r="C23" s="42" t="inlineStr">
+        <is>
+          <t>SUM office rows for G–M; recompute % from summed totals (do not average office % values)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="39" t="inlineStr">
         <is>
           <t>GU</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Beaver Falls check</t>
-        </is>
-      </c>
-      <c r="C9" s="19" t="inlineStr">
+      <c r="B24" s="36" t="inlineStr">
+        <is>
+          <t>Beaver Falls check (PDF)</t>
+        </is>
+      </c>
+      <c r="C24" s="42" t="inlineStr">
         <is>
           <t>122÷440≈28% Utilization; 67÷1079≈6% job mix; 440÷401.5≈109.6% Integration; 122÷401.5≈30% Fulfillment</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="20" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="36" t="n"/>
+      <c r="B25" s="36" t="n"/>
+      <c r="C25" s="36" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="35" t="inlineStr">
+        <is>
+          <t>JOB-LEVEL FORMULAS (single-day REC / OX / MD)</t>
+        </is>
+      </c>
+      <c r="B26" s="36" t="n"/>
+      <c r="C26" s="36" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="41" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="B27" s="41" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="C27" s="41" t="inlineStr">
+        <is>
+          <t>Formula / rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="43" t="inlineStr">
         <is>
           <t>OX</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
+      <c r="B28" s="36" t="inlineStr">
         <is>
           <t>Total Saved</t>
         </is>
       </c>
-      <c r="C10" s="22" t="inlineStr">
+      <c r="C28" s="42" t="inlineStr">
         <is>
           <t>max(0, Total Staff Requested − Total Staff Sent)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="43" t="inlineStr">
         <is>
           <t>OX</t>
         </is>
       </c>
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B29" s="36" t="inlineStr">
         <is>
           <t>AFAD Sent</t>
         </is>
       </c>
-      <c r="C11" s="22" t="inlineStr">
+      <c r="C29" s="42" t="inlineStr">
         <is>
           <t>COUNT of devices listed in REC GSF AFAD</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="23" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="43" t="inlineStr">
         <is>
           <t>MD</t>
         </is>
       </c>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B30" s="36" t="inlineStr">
         <is>
           <t>Unfilled</t>
         </is>
       </c>
-      <c r="C12" s="25" t="inlineStr">
+      <c r="C30" s="42" t="inlineStr">
         <is>
           <t>Required − Assignments</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="26" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="43" t="inlineStr">
         <is>
           <t>REC</t>
         </is>
       </c>
-      <c r="B13" s="27" t="inlineStr">
+      <c r="B31" s="36" t="inlineStr">
         <is>
           <t>Unfilled Count</t>
         </is>
       </c>
-      <c r="C13" s="28" t="inlineStr">
+      <c r="C31" s="42" t="inlineStr">
         <is>
           <t>max(0, Required Resources − Assignment Count)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="26" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="43" t="inlineStr">
         <is>
           <t>REC</t>
         </is>
       </c>
-      <c r="B14" s="27" t="inlineStr">
+      <c r="B32" s="36" t="inlineStr">
         <is>
           <t>Assignment Count</t>
         </is>
       </c>
-      <c r="C14" s="28" t="inlineStr">
+      <c r="C32" s="42" t="inlineStr">
         <is>
           <t>COUNT of confirmed people in Assigned Employees</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="26" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="43" t="inlineStr">
         <is>
           <t>REC</t>
         </is>
       </c>
-      <c r="B15" s="27" t="inlineStr">
+      <c r="B33" s="36" t="inlineStr">
         <is>
           <t>Completed Timesheets</t>
         </is>
       </c>
-      <c r="C15" s="28" t="inlineStr">
+      <c r="C33" s="42" t="inlineStr">
         <is>
           <t>COUNT of completed/approved timesheets</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="26" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="43" t="inlineStr">
         <is>
           <t>REC</t>
         </is>
       </c>
-      <c r="B16" s="27" t="inlineStr">
+      <c r="B34" s="36" t="inlineStr">
         <is>
           <t>Total Timesheets</t>
         </is>
       </c>
-      <c r="C16" s="28" t="inlineStr">
+      <c r="C34" s="42" t="inlineStr">
         <is>
           <t>COUNT of all timesheets on the job</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="26" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="43" t="inlineStr">
         <is>
           <t>REC</t>
         </is>
       </c>
-      <c r="B17" s="27" t="inlineStr">
+      <c r="B35" s="36" t="inlineStr">
         <is>
           <t>Cancellation Count</t>
         </is>
       </c>
-      <c r="C17" s="28" t="inlineStr">
+      <c r="C35" s="42" t="inlineStr">
         <is>
           <t>COUNT of records in Cancellation Information</t>
         </is>
@@ -1791,63 +2123,130 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="29" t="inlineStr">
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="44" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="30" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="30" t="inlineStr">
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="45" t="inlineStr">
         <is>
           <t>Abbreviations: REC = Roads Export · OX = Onyx · MD = Master Dashboard · GU = GSF Utilization Report</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="30" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="30" t="inlineStr">
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="45" t="inlineStr">
         <is>
           <t>Colors: Green=REC · Cream=OX · Blue=MD · Rose=GU</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="30" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="30" t="inlineStr">
-        <is>
-          <t>GU is an office-level rollup. Job-level REC/OX/MD rows feed GU when summed/counted by office (e.g. Beaver Falls).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="30" t="inlineStr">
-        <is>
-          <t>Example from GU PDF — WDW Beaver Falls: Sets 122, On Hand 440 → Utilization 28%; GSF Jobs 67 / Total Jobs 1079 → 6%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="30" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="30" t="inlineStr">
-        <is>
-          <t>See Number Formulas sheet for full calculation list.</t>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="45" t="inlineStr"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="44" t="inlineStr">
+        <is>
+          <t>TIME GRAIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="46" t="inlineStr">
+        <is>
+          <t>REC / OX / MD (the sources compared earlier): share job-level information for a SINGLE day. Matching keys (Job Number / Ticket # / Dispatching) line up for that day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="47" t="inlineStr">
+        <is>
+          <t>GU (GSF Utilization Report): uses the SAME kinds of source fields, but rolled up across NUMEROUS days into office/company period totals. Percentages are then computed from those multi-day totals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="45" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="44" t="inlineStr">
+        <is>
+          <t>HOW PERCENTAGES ARE GENERATED</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="47" t="inlineStr">
+        <is>
+          <t>GU % columns are not typed in — they are calculated from the rolled source counts:</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • GSF Utilization % = In Field Sets ÷ Sets on Hand</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • GSF infield set/total jobs % = GSF Jobs ÷ Total Jobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • GSF Integration (Crews) % = Sets on Hand ÷ Flagging Crews</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • GSF Fulfillment Crews % = In Field Sets ÷ Flagging Crews</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • People Saved = In Field Sets</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="45" t="inlineStr">
+        <is>
+          <t>Footer check on the PDF: Corrected Grand 11469 ÷ 23265.0 = 49.30% → 49%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="45" t="inlineStr"/>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="45" t="inlineStr">
+        <is>
+          <t>Example — WDW Beaver Falls on GU: Sets 122, On Hand 440 → Utilization 28%; GSF Jobs 67 / Total Jobs 1079 → 6%. Those office totals are period aggregates, not one day’s Roads/Onyx/Master export.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="45" t="inlineStr">
+        <is>
+          <t>See Number Formulas sheet for the full source → rollup → % chain.</t>
         </is>
       </c>
     </row>
@@ -1862,7 +2261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2275,9 +2674,32 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="48" t="inlineStr">
+        <is>
+          <t>TIME GRAIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="49" t="inlineStr">
+        <is>
+          <t>REC/OX/MD correspondences above are job-level and match on a SINGLE day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="50" t="inlineStr">
+        <is>
+          <t>GU links are the SAME fields summed/counted across NUMEROUS days by office; GU % are then calculated from those period totals.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A31:E31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Validate GU Utilization: sets × weekdays (Washington Aug 17–23)
Washington Roads export confirms Utilization = GSF job-days ÷
(physical sets × weekday working days): 14 ÷ (6×5) = 46.67% → 47%.

Co-authored-by: echenry6f <echenry6f@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Roads_Onyx_Master_Column_Crosswalk.xlsx
+++ b/Roads_Onyx_Master_Column_Crosswalk.xlsx
@@ -96,7 +96,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -148,8 +148,13 @@
         <fgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -185,11 +190,55 @@
         <color rgb="00B0B0B0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -299,6 +348,11 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1594,7 +1648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1608,8 +1662,8 @@
           <t>How GSF Utilization % are built from REC / OX / MD sources</t>
         </is>
       </c>
-      <c r="B1" s="36" t="n"/>
-      <c r="C1" s="36" t="n"/>
+      <c r="B1" s="51" t="n"/>
+      <c r="C1" s="52" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="36" t="n"/>
@@ -2106,6 +2160,64 @@
       <c r="C35" s="42" t="inlineStr">
         <is>
           <t>COUNT of records in Cancellation Information</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="53" t="inlineStr">
+        <is>
+          <t>VALIDATED — Washington Aug 17–23 (Util 47%, 6 physical sets)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="54" t="inlineStr">
+        <is>
+          <t>GU</t>
+        </is>
+      </c>
+      <c r="B38" s="48" t="inlineStr">
+        <is>
+          <t>GSF Sets on Hand (Working Days)</t>
+        </is>
+      </c>
+      <c r="C38" s="49" t="inlineStr">
+        <is>
+          <t>Physical sets at office × COUNT of Mon–Fri weekdays in period  (Washington: 6×5=30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="54" t="inlineStr">
+        <is>
+          <t>GU</t>
+        </is>
+      </c>
+      <c r="B39" s="48" t="inlineStr">
+        <is>
+          <t>GSF In Field Sets</t>
+        </is>
+      </c>
+      <c r="C39" s="49" t="inlineStr">
+        <is>
+          <t>COUNT of job-days with GSF Job=Yes (1 set per GSF job-day; weekend deployments count)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="54" t="inlineStr">
+        <is>
+          <t>GU</t>
+        </is>
+      </c>
+      <c r="B40" s="48" t="inlineStr">
+        <is>
+          <t>GSF Utilization %</t>
+        </is>
+      </c>
+      <c r="C40" s="49" t="inlineStr">
+        <is>
+          <t>In Field Sets ÷ Sets on Hand  →  Washington check: 14÷30=46.67%→47%</t>
         </is>
       </c>
     </row>
@@ -2123,7 +2235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2247,6 +2359,20 @@
       <c r="A19" s="45" t="inlineStr">
         <is>
           <t>See Number Formulas sheet for the full source → rollup → % chain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="53" t="inlineStr">
+        <is>
+          <t>VALIDATED Sets on Hand formula (Washington Aug 17–23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="55" t="inlineStr">
+        <is>
+          <t>GSF Sets on Hand (Working Days) = physical sets × weekday working days. Utilization = In Field Sets ÷ that product. Washington: 14÷(6×5)=46.67%→47%.</t>
         </is>
       </c>
     </row>

</xml_diff>